<commit_message>
Auto Update Prices: Sat May  9 22:10:16 UTC 2026
</commit_message>
<xml_diff>
--- a/가격이력.xlsx
+++ b/가격이력.xlsx
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -525,7 +525,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -572,7 +572,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -713,7 +713,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -760,7 +760,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -948,7 +948,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -995,7 +995,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1089,7 +1089,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1136,7 +1136,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1230,7 +1230,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1324,7 +1324,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1371,7 +1371,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1418,7 +1418,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1512,7 +1512,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1559,7 +1559,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1606,7 +1606,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1653,7 +1653,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1700,7 +1700,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1747,7 +1747,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1794,7 +1794,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1841,7 +1841,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1888,7 +1888,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1935,7 +1935,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1982,7 +1982,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2029,7 +2029,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2076,7 +2076,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2123,7 +2123,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2170,7 +2170,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2217,7 +2217,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2264,7 +2264,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2311,7 +2311,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2358,7 +2358,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2405,7 +2405,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2452,7 +2452,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2499,7 +2499,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2593,7 +2593,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2640,7 +2640,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2734,7 +2734,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2781,7 +2781,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2828,7 +2828,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2875,7 +2875,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2922,7 +2922,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2969,7 +2969,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3016,7 +3016,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3063,7 +3063,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3110,7 +3110,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3157,7 +3157,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3204,7 +3204,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3251,7 +3251,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3298,7 +3298,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3345,7 +3345,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3392,7 +3392,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3439,7 +3439,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3486,7 +3486,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3533,7 +3533,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3580,7 +3580,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3627,7 +3627,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3674,7 +3674,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3721,7 +3721,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3768,7 +3768,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3815,7 +3815,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3862,7 +3862,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3909,7 +3909,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3956,7 +3956,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4003,7 +4003,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4050,7 +4050,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4144,7 +4144,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4191,7 +4191,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4238,7 +4238,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4285,7 +4285,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4332,7 +4332,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4379,7 +4379,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4426,7 +4426,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4473,7 +4473,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4520,7 +4520,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4567,7 +4567,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4614,7 +4614,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4661,7 +4661,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4708,7 +4708,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4755,7 +4755,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4802,7 +4802,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4849,7 +4849,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4896,7 +4896,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4943,7 +4943,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4990,7 +4990,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -5037,7 +5037,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -5084,7 +5084,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5131,7 +5131,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -5178,7 +5178,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -5225,7 +5225,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -5272,7 +5272,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -5319,7 +5319,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -5366,7 +5366,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -5413,7 +5413,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -5460,7 +5460,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5554,7 +5554,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5601,7 +5601,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5648,7 +5648,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5695,7 +5695,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5742,7 +5742,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -5789,7 +5789,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -5836,7 +5836,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -5883,7 +5883,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -5930,7 +5930,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -5977,7 +5977,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -6024,7 +6024,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -6071,7 +6071,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -6118,7 +6118,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -6165,7 +6165,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -6212,7 +6212,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -6259,7 +6259,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -6306,7 +6306,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -6353,7 +6353,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -6400,7 +6400,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -6447,7 +6447,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -6494,7 +6494,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -6541,7 +6541,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -6588,7 +6588,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -6635,7 +6635,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -6682,7 +6682,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -6729,7 +6729,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -6776,7 +6776,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -6823,7 +6823,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -6870,7 +6870,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -6964,7 +6964,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -7011,7 +7011,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -7058,7 +7058,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -7105,7 +7105,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -7152,7 +7152,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -7199,7 +7199,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -7246,7 +7246,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -7293,7 +7293,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -7340,7 +7340,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -7387,7 +7387,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -7434,7 +7434,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -7481,7 +7481,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -7528,7 +7528,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -7575,7 +7575,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -7622,7 +7622,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -7669,7 +7669,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -7716,7 +7716,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -7763,7 +7763,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -7810,7 +7810,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -7857,7 +7857,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -7904,7 +7904,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -7951,7 +7951,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -7998,7 +7998,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -8045,7 +8045,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -8092,7 +8092,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -8139,7 +8139,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -8186,7 +8186,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -8233,7 +8233,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -8280,7 +8280,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -8374,7 +8374,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -8421,7 +8421,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -8468,7 +8468,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -8515,7 +8515,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -8562,7 +8562,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -8609,7 +8609,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -8656,7 +8656,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -8703,7 +8703,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -8750,7 +8750,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -8797,7 +8797,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -8844,7 +8844,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -8891,7 +8891,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -8938,7 +8938,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -8985,7 +8985,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -9032,7 +9032,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -9079,7 +9079,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -9126,7 +9126,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -9173,7 +9173,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -9220,7 +9220,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -9267,7 +9267,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -9314,7 +9314,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -9361,7 +9361,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -9408,7 +9408,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -9455,7 +9455,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -9502,7 +9502,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -9549,7 +9549,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -9596,7 +9596,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -9643,7 +9643,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -9690,7 +9690,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -9737,7 +9737,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -9784,7 +9784,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -9831,7 +9831,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -9878,7 +9878,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -9925,7 +9925,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -9972,7 +9972,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -10019,7 +10019,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -10066,7 +10066,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -10113,7 +10113,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -10160,7 +10160,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -10207,7 +10207,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -10254,7 +10254,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -10301,7 +10301,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -10348,7 +10348,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -10395,7 +10395,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -10442,7 +10442,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -10489,7 +10489,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -10536,7 +10536,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -10583,7 +10583,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -10630,7 +10630,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -10677,7 +10677,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -10724,7 +10724,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -10771,7 +10771,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -10819,7 +10819,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -10867,7 +10867,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -10914,7 +10914,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -10962,7 +10962,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -11011,7 +11011,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -11060,7 +11060,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -11109,7 +11109,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -11158,7 +11158,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -11205,7 +11205,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-05-09 18:38</t>
+          <t>2026-05-09 22:10</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">

</xml_diff>

<commit_message>
Auto Update Prices: Sun May 10 22:35:38 UTC 2026
</commit_message>
<xml_diff>
--- a/가격이력.xlsx
+++ b/가격이력.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I123"/>
+  <dimension ref="A1:I115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-10 12:53</t>
+          <t>2026-05-10 21:53</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -525,7 +525,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-10 12:53</t>
+          <t>2026-05-10 21:53</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -572,7 +572,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-10 12:53</t>
+          <t>2026-05-10 21:53</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-10 12:53</t>
+          <t>2026-05-10 21:53</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-10 12:53</t>
+          <t>2026-05-10 21:53</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -713,7 +713,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-10 12:54</t>
+          <t>2026-05-10 21:53</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -760,7 +760,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-10 12:54</t>
+          <t>2026-05-10 21:53</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-10 12:54</t>
+          <t>2026-05-10 21:53</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-10 12:54</t>
+          <t>2026-05-10 21:54</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-10 12:54</t>
+          <t>2026-05-10 21:54</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -948,7 +948,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-10 12:54</t>
+          <t>2026-05-10 21:55</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -995,7 +995,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-10 12:54</t>
+          <t>2026-05-10 21:55</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-10 12:54</t>
+          <t>2026-05-10 21:55</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1089,7 +1089,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-10 12:54</t>
+          <t>2026-05-10 21:56</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1136,7 +1136,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-10 12:55</t>
+          <t>2026-05-10 21:57</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-10 12:55</t>
+          <t>2026-05-10 21:57</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1230,7 +1230,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-10 12:55</t>
+          <t>2026-05-10 21:58</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-10 12:55</t>
+          <t>2026-05-10 21:58</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1324,7 +1324,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-10 12:55</t>
+          <t>2026-05-10 21:58</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1371,7 +1371,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-10 12:55</t>
+          <t>2026-05-10 21:58</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1418,7 +1418,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-10 12:55</t>
+          <t>2026-05-10 21:58</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-10 12:55</t>
+          <t>2026-05-10 21:58</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1512,7 +1512,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-10 12:55</t>
+          <t>2026-05-10 21:58</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1559,7 +1559,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-10 12:55</t>
+          <t>2026-05-10 21:58</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1606,7 +1606,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-10 12:55</t>
+          <t>2026-05-10 21:58</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1653,7 +1653,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-10 12:55</t>
+          <t>2026-05-10 21:58</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1700,7 +1700,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 21:59</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1747,7 +1747,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 21:59</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1794,7 +1794,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 21:59</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1841,7 +1841,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 21:59</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1888,7 +1888,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 21:59</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1935,7 +1935,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 21:59</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1982,7 +1982,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 21:59</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2029,7 +2029,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 21:59</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2076,7 +2076,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 21:59</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2123,7 +2123,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 21:59</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2170,7 +2170,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 22:00</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2217,7 +2217,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 22:00</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2264,7 +2264,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 22:00</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2311,7 +2311,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 22:00</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2358,7 +2358,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 22:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2405,7 +2405,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 22:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2452,7 +2452,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 22:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2499,7 +2499,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 22:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 22:00</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2593,7 +2593,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 22:01</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2640,7 +2640,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 22:01</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 22:01</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2734,7 +2734,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 22:01</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2781,7 +2781,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 22:01</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2828,7 +2828,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-10 12:56</t>
+          <t>2026-05-10 22:02</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2875,7 +2875,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-10 12:57</t>
+          <t>2026-05-10 22:02</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2922,7 +2922,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-10 12:57</t>
+          <t>2026-05-10 22:03</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2969,7 +2969,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-10 12:57</t>
+          <t>2026-05-10 22:03</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3016,7 +3016,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-10 12:57</t>
+          <t>2026-05-10 22:03</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3063,7 +3063,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-10 12:57</t>
+          <t>2026-05-10 22:03</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3110,7 +3110,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-10 12:57</t>
+          <t>2026-05-10 22:03</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3157,7 +3157,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-10 12:57</t>
+          <t>2026-05-10 22:04</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3204,7 +3204,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-10 12:57</t>
+          <t>2026-05-10 22:04</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3251,7 +3251,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-10 12:57</t>
+          <t>2026-05-10 22:04</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3298,7 +3298,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-05-10 12:57</t>
+          <t>2026-05-10 22:04</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3345,7 +3345,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-10 12:58</t>
+          <t>2026-05-10 22:04</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3392,7 +3392,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-10 12:58</t>
+          <t>2026-05-10 22:05</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3439,7 +3439,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-10 12:58</t>
+          <t>2026-05-10 22:05</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3486,7 +3486,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-05-10 12:58</t>
+          <t>2026-05-10 22:05</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3533,7 +3533,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-10 12:58</t>
+          <t>2026-05-10 22:05</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3580,7 +3580,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-10 12:58</t>
+          <t>2026-05-10 22:06</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3627,7 +3627,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-10 12:59</t>
+          <t>2026-05-10 22:07</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3674,7 +3674,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-05-10 12:59</t>
+          <t>2026-05-10 22:07</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3721,7 +3721,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-10 12:59</t>
+          <t>2026-05-10 22:08</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3768,7 +3768,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-05-10 12:59</t>
+          <t>2026-05-10 22:08</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3815,7 +3815,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-10 12:59</t>
+          <t>2026-05-10 22:09</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3862,7 +3862,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-05-10 13:00</t>
+          <t>2026-05-10 22:11</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3909,7 +3909,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-10 13:01</t>
+          <t>2026-05-10 22:13</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3956,7 +3956,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-05-10 13:01</t>
+          <t>2026-05-10 22:13</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4003,7 +4003,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-10 13:01</t>
+          <t>2026-05-10 22:13</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4050,7 +4050,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-05-10 13:01</t>
+          <t>2026-05-10 22:14</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-10 13:02</t>
+          <t>2026-05-10 22:17</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4144,7 +4144,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05-10 13:03</t>
+          <t>2026-05-10 22:17</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4191,7 +4191,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-10 13:03</t>
+          <t>2026-05-10 22:17</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4238,7 +4238,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-05-10 13:03</t>
+          <t>2026-05-10 22:17</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4285,7 +4285,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-10 13:04</t>
+          <t>2026-05-10 22:19</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4332,7 +4332,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-05-10 13:04</t>
+          <t>2026-05-10 22:20</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4379,7 +4379,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-10 13:04</t>
+          <t>2026-05-10 22:20</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4426,7 +4426,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-05-10 13:04</t>
+          <t>2026-05-10 22:20</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4473,7 +4473,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-10 13:04</t>
+          <t>2026-05-10 22:20</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4520,7 +4520,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-05-10 13:04</t>
+          <t>2026-05-10 22:21</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4567,7 +4567,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-10 13:04</t>
+          <t>2026-05-10 22:21</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4614,7 +4614,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-05-10 13:04</t>
+          <t>2026-05-10 22:22</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4661,7 +4661,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-10 13:07</t>
+          <t>2026-05-10 22:25</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4708,7 +4708,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-05-10 13:07</t>
+          <t>2026-05-10 22:26</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4755,7 +4755,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-10 13:07</t>
+          <t>2026-05-10 22:26</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4802,7 +4802,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-05-10 13:07</t>
+          <t>2026-05-10 22:26</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4849,7 +4849,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-10 13:07</t>
+          <t>2026-05-10 22:26</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4896,7 +4896,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-05-10 13:07</t>
+          <t>2026-05-10 22:26</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4943,7 +4943,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-10 13:07</t>
+          <t>2026-05-10 22:26</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4990,7 +4990,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-05-10 13:07</t>
+          <t>2026-05-10 22:27</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -5037,7 +5037,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-10 13:07</t>
+          <t>2026-05-10 22:27</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -5084,7 +5084,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-05-10 13:07</t>
+          <t>2026-05-10 22:28</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5131,7 +5131,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-10 13:08</t>
+          <t>2026-05-10 22:29</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -5178,7 +5178,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-05-10 13:08</t>
+          <t>2026-05-10 22:29</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -5225,7 +5225,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-05-10 13:09</t>
+          <t>2026-05-10 22:31</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -5272,7 +5272,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-05-10 13:09</t>
+          <t>2026-05-10 22:31</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -5319,7 +5319,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-05-10 13:09</t>
+          <t>2026-05-10 22:31</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -5366,7 +5366,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-05-10 13:09</t>
+          <t>2026-05-10 22:31</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -5413,7 +5413,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-05-10 13:09</t>
+          <t>2026-05-10 22:31</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -5460,7 +5460,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-05-10 13:09</t>
+          <t>2026-05-10 22:31</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-10 13:09</t>
+          <t>2026-05-10 22:31</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5554,7 +5554,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-10 13:09</t>
+          <t>2026-05-10 22:31</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5601,7 +5601,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-10 13:09</t>
+          <t>2026-05-10 22:31</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5648,7 +5648,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-10 13:09</t>
+          <t>2026-05-10 22:32</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5695,7 +5695,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-10 13:09</t>
+          <t>2026-05-10 22:32</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5742,7 +5742,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-10 13:09</t>
+          <t>2026-05-10 22:32</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -5789,7 +5789,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-10 13:09</t>
+          <t>2026-05-10 22:32</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -5830,434 +5830,6 @@
       <c r="I115" t="inlineStr">
         <is>
           <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000582</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>2026-05-10 13:10</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>제이비티엠(농산물)</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>감자</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>★26년 햇감자
-★개당중량
- -중 : 40-70g 내외
- -대 : 70-110g 내외
- -특 : 110-160g 내외
- -왕특 : 160g이상
-햇감자 시즌 초반이라 중·후반기에 비해
-전체적인 알의 크기가 조금 작을 수 있습니다.
-★수미감자산지계획
-김제(하우스) - 밀양(하우스) - 경남 일대(노지)
-★고품위 상품</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr"/>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>4/16(목)
-부터~</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>시트참조</t>
-        </is>
-      </c>
-      <c r="H116" t="inlineStr">
-        <is>
-          <t>별도확인</t>
-        </is>
-      </c>
-      <c r="I116" t="inlineStr">
-        <is>
-          <t>https://docs.google.com/spreadsheets/d/1g0Bxmz773DqPjCfYgBNyBtlYKxYuLJYY2zasqiC5u7Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>2026-05-10 13:10</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>제이비티엠(농산물)</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>감자</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>★ 26년 햇하우스설봉감자(~5월까지)
- - 6월부터 노지 햇설봉감자 예정
-★ 산지정보 : 밀양/김제/창녕/강릉
-★ 개당중량 및 용도
- -   특  : 120g ~ 250g (조리용, 찜용)
- -   대  : 60 ~ 120g (찜용)
-★ 박스 입수량
- - 1.5kg : 특 : 6-12개 내외
-           . 대 : 12-25개 내외
- -  3kg  : 특 : 12-25개 내외
-           : 대 : 25-50개 내외
- -  5kg  : 특 : 20-41개 내외
-           : 대 : 41-83개 내외</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr"/>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>4/14일(화)
-부터</t>
-        </is>
-      </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>시트참조</t>
-        </is>
-      </c>
-      <c r="H117" t="inlineStr">
-        <is>
-          <t>별도확인</t>
-        </is>
-      </c>
-      <c r="I117" t="inlineStr">
-        <is>
-          <t>https://docs.google.com/spreadsheets/d/1g0Bxmz773DqPjCfYgBNyBtlYKxYuLJYY2zasqiC5u7Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>2026-05-10 13:10</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>제이비티엠(농산물)</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>감자</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>★ 26년 햇하우스홍감자(~5월까지)
- - 6월부터 노지 햇홍감자 예정
-★ 산지정보 : 밀양/남해/진주/함안/괴산/태안/양구
-★ 개당중량 및 용도
- -  왕특 : 250g 이상 (조리용)
- -   특  : 120g ~ 250g (조리용, 찜용)
- -   대  : 60 ~ 120g (찜용)
-★ 박스 입수량
- - 1.5kg : 왕특 : 3-6개 내외
-             특 : 6-12개 내외
-           . 대 : 12-25개 내외
- -  3kg  : 왕특 : 7-12개 내외
-           : 특 : 12-25개 내외
-           : 대 : 25-50개 내외
- -  5kg  : 왕특 : 10-20개 내외
-           : 특 : 20-41개 내외
-           : 대 : 41-83개 내외
-★고품위 상품</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr"/>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>4/14(화)
-부터</t>
-        </is>
-      </c>
-      <c r="G118" t="inlineStr">
-        <is>
-          <t>시트참조</t>
-        </is>
-      </c>
-      <c r="H118" t="inlineStr">
-        <is>
-          <t>별도확인</t>
-        </is>
-      </c>
-      <c r="I118" t="inlineStr">
-        <is>
-          <t>https://docs.google.com/spreadsheets/d/1g0Bxmz773DqPjCfYgBNyBtlYKxYuLJYY2zasqiC5u7Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>2026-05-10 13:10</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>제이비티엠(농산물)</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>양파</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>★실중량
-★품목별 개당중량 및 입수수량
- -당근 : 240g 내외(2~3개)
- -감자 : 150g 내외(3~4개)
- -양파 : 240g 내외(2~3개)</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr"/>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>8/20일(수)
-부터</t>
-        </is>
-      </c>
-      <c r="G119" t="inlineStr">
-        <is>
-          <t>시트참조</t>
-        </is>
-      </c>
-      <c r="H119" t="inlineStr">
-        <is>
-          <t>별도확인</t>
-        </is>
-      </c>
-      <c r="I119" t="inlineStr">
-        <is>
-          <t>https://docs.google.com/spreadsheets/d/1g0Bxmz773DqPjCfYgBNyBtlYKxYuLJYY2zasqiC5u7Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>2026-05-10 13:10</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>제이비티엠(농산물)</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>양파</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>#실중량
-#가정용 햇양파
-#원산지 : 경남~경북 일대
-#포장방법 : 박스 포장
-#개당중량
- 소 : 100g 이하
-중 :  100g ~ 150g
-대 : 150g ~ 200g
-특대 : 200g 이상</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr"/>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>5/07일(목)
-부터</t>
-        </is>
-      </c>
-      <c r="G120" t="inlineStr">
-        <is>
-          <t>시트참조</t>
-        </is>
-      </c>
-      <c r="H120" t="inlineStr">
-        <is>
-          <t>별도확인</t>
-        </is>
-      </c>
-      <c r="I120" t="inlineStr">
-        <is>
-          <t>https://docs.google.com/spreadsheets/d/1g0Bxmz773DqPjCfYgBNyBtlYKxYuLJYY2zasqiC5u7Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>2026-05-10 13:10</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>제이비티엠(과일)</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>토마토</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>★국내산
-★대추방울토마토 품종 : 더하드, 노나리
-★출고기준 : 1~3번과중 과육이 튼튼한것만 출고
-★4키로 옵션 추가
-★프리미엄급 품위
-★매주 수요일 공급가 변동</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr"/>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>5/08일(금)
-부터
-~
-12일(화)
-까지</t>
-        </is>
-      </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>시트참조</t>
-        </is>
-      </c>
-      <c r="H121" t="inlineStr">
-        <is>
-          <t>별도확인</t>
-        </is>
-      </c>
-      <c r="I121" t="inlineStr">
-        <is>
-          <t>https://docs.google.com/spreadsheets/d/1g0Bxmz773DqPjCfYgBNyBtlYKxYuLJYY2zasqiC5u7Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>2026-05-10 13:10</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>제이비티엠(과일)</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>참외</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>#옵션중,, 망고가 들어가 있는 옵션은 (골드망고)로 
-확인 부탁드립니다.
-#품위 위주의 구성으로 최대한 가격을 잡은 구성으로,,
-상시 판매로 가격변동을 최소화하여 공급 예정
-#원물별 SPEC
-▷사과: 개 당 300g~375g 내외 (국내산/경북 일대)
-▷참외: 개 당 300g~400g 내외 (국내산/경북 일대)
-▷골드망고: 개 당 320g~410g 내외 (수입산/베트남,태국)
-▷오렌지: 개 당 250g~340g 내외 (수입산/미국,호주)
-▷용과: 개 당 480g~550g 내외 (수입산/베트남)</t>
-        </is>
-      </c>
-      <c r="E122" t="inlineStr"/>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>3/18일(수)
-부터</t>
-        </is>
-      </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>시트참조</t>
-        </is>
-      </c>
-      <c r="H122" t="inlineStr">
-        <is>
-          <t>별도확인</t>
-        </is>
-      </c>
-      <c r="I122" t="inlineStr">
-        <is>
-          <t>https://docs.google.com/spreadsheets/d/1g0Bxmz773DqPjCfYgBNyBtlYKxYuLJYY2zasqiC5u7Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>2026-05-10 13:10</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>제이비티엠(과일)</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>수박</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>#하우스수박
-#비파괴당도선별 11브릭스 이상제품
-#상품/정품 구분기준
- -상품 : 기형/미색 등(당도는 정품과 동일)
- -정품 : 프리미엄
-#중량 구분기준(실중량)
- -동절기 : 500g기준(예:6kg~6.5kg / 6.5kg~7kg)
- -하절기 : 1kg기준(예:6kg~7kg)
-#포장방식 : 에어셀+박스</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr"/>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>5/08일(금)
-부터</t>
-        </is>
-      </c>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>시트참조</t>
-        </is>
-      </c>
-      <c r="H123" t="inlineStr">
-        <is>
-          <t>별도확인</t>
-        </is>
-      </c>
-      <c r="I123" t="inlineStr">
-        <is>
-          <t>https://docs.google.com/spreadsheets/d/1g0Bxmz773DqPjCfYgBNyBtlYKxYuLJYY2zasqiC5u7Y</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto Update Prices: Mon May 11 22:54:03 UTC 2026
</commit_message>
<xml_diff>
--- a/가격이력.xlsx
+++ b/가격이력.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I115"/>
+  <dimension ref="A1:I122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-10 21:53</t>
+          <t>2026-05-11 22:10</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -488,12 +488,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>SVIP ★ 하우스 대극천복숭아 ★</t>
+          <t>하우스 흑미수박</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -518,14 +518,14 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010048</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010144</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-10 21:53</t>
+          <t>2026-05-11 22:10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -535,12 +535,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>SVIP ★ 하우스 대석자두 ★</t>
+          <t>스테비아방울토마토</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -565,14 +565,14 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010045</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010143</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-10 21:53</t>
+          <t>2026-05-11 22:11</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -582,12 +582,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SVIP ★ 하우스 복숭아 ★</t>
+          <t>우곡수박</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -612,14 +612,14 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010044</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010136</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-10 21:53</t>
+          <t>2026-05-11 22:11</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>[VIP] 하우스복숭아</t>
+          <t>천도복숭아</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -659,14 +659,14 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010007</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010109</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-10 21:53</t>
+          <t>2026-05-11 22:11</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -676,12 +676,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>[VIP] 하우스자두</t>
+          <t>신비복숭아</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -706,14 +706,14 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010006</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010108</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-10 21:53</t>
+          <t>2026-05-11 22:11</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -723,12 +723,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>수박 (가정용/정품)</t>
+          <t>SVIP ★ 하우스 대극천복숭아 ★</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -753,14 +753,14 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009976</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010048</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-10 21:53</t>
+          <t>2026-05-11 22:11</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -770,12 +770,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>SVIP ★ 하우스 대석자두 ★</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -800,14 +800,14 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009960</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010045</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-10 21:53</t>
+          <t>2026-05-11 22:11</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>하우스 신선복숭아</t>
+          <t>SVIP ★ 하우스 복숭아 ★</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -847,14 +847,14 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009959</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010044</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-10 21:54</t>
+          <t>2026-05-11 22:11</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -864,12 +864,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>햇양파</t>
+          <t>[VIP] 하우스복숭아</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -894,14 +894,14 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009925</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010007</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-10 21:54</t>
+          <t>2026-05-11 22:12</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -911,12 +911,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>[VIP] 하우스자두</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -941,14 +941,14 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009854</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010006</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-10 21:55</t>
+          <t>2026-05-11 22:12</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -958,12 +958,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>완숙 찰 토마토</t>
+          <t>수박 (가정용/정품)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -988,14 +988,14 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009762</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009976</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-10 21:55</t>
+          <t>2026-05-11 22:12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1005,12 +1005,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>짭짤이 토마토</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1035,14 +1035,14 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009744</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009960</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-10 21:55</t>
+          <t>2026-05-11 22:12</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1052,12 +1052,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>특★가 양파</t>
+          <t>하우스 신선복숭아</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1082,14 +1082,14 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009488</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009959</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-10 21:56</t>
+          <t>2026-05-11 22:13</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1099,12 +1099,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>★ 특~가 망고수박 ★</t>
+          <t>햇양파</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1129,29 +1129,29 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009445</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009925</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-10 21:57</t>
+          <t>2026-05-11 22:13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>팡이농장</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 혼합과</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1176,29 +1176,29 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011646</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009854</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-10 21:57</t>
+          <t>2026-05-11 22:13</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>팡이농장</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 대과</t>
+          <t>완숙 찰 토마토</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1223,29 +1223,29 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011645</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009762</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-10 21:58</t>
+          <t>2026-05-11 22:14</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>팡이농장</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 로얄과</t>
+          <t>짭짤이 토마토</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1270,29 +1270,29 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011644</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009744</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-10 21:58</t>
+          <t>2026-05-11 22:14</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>팡이농장</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 소과</t>
+          <t>특★가 양파</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1317,14 +1317,14 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011643</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009488</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-10 21:58</t>
+          <t>2026-05-11 22:15</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 혼합과</t>
+          <t>행사 (박스포함) 참외 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1364,14 +1364,14 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011642</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011646</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-10 21:58</t>
+          <t>2026-05-11 22:15</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 대과</t>
+          <t>행사 (박스포함) 참외 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1411,14 +1411,14 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011641</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011645</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-10 21:58</t>
+          <t>2026-05-11 22:16</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 로얄과</t>
+          <t>행사 (박스포함) 참외 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1458,14 +1458,14 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011640</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011644</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-10 21:58</t>
+          <t>2026-05-11 22:16</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 소과</t>
+          <t>행사 (박스포함) 참외 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1505,14 +1505,14 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011639</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011643</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-10 21:58</t>
+          <t>2026-05-11 22:16</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 혼합과</t>
+          <t>행사 (박스포함) 참외 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1552,14 +1552,14 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011638</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011642</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-10 21:58</t>
+          <t>2026-05-11 22:16</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 대과</t>
+          <t>행사 (박스포함) 참외 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1599,14 +1599,14 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011637</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011641</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-10 21:58</t>
+          <t>2026-05-11 22:16</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 로얄과</t>
+          <t>행사 (박스포함) 참외 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1646,14 +1646,14 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011636</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011640</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-10 21:58</t>
+          <t>2026-05-11 22:16</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 소과</t>
+          <t>행사 (박스포함) 참외 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1693,14 +1693,14 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011635</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011639</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-10 21:59</t>
+          <t>2026-05-11 22:16</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
+          <t>행사 (박스포함) 참외 가정용 / 10kg / 혼합과</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1740,14 +1740,14 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011638</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-10 21:59</t>
+          <t>2026-05-11 22:16</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
+          <t>행사 (박스포함) 참외 가정용 / 10kg / 대과</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1787,14 +1787,14 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011637</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-10 21:59</t>
+          <t>2026-05-11 22:16</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
+          <t>행사 (박스포함) 참외 가정용 / 10kg / 로얄과</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1834,14 +1834,14 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011636</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-10 21:59</t>
+          <t>2026-05-11 22:16</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
+          <t>행사 (박스포함) 참외 가정용 / 10kg / 소과</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1881,14 +1881,14 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011635</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-10 21:59</t>
+          <t>2026-05-11 22:17</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1898,12 +1898,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>흑대추방울토마토 5kg</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1928,14 +1928,14 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011224</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-10 21:59</t>
+          <t>2026-05-11 22:17</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1945,12 +1945,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>흑대추방울토마토 2kg</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1975,14 +1975,14 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011223</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-10 21:59</t>
+          <t>2026-05-11 22:17</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1992,12 +1992,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>흑대추방울토마토 1kg</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2022,14 +2022,14 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011222</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-10 21:59</t>
+          <t>2026-05-11 22:17</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2069,14 +2069,14 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-10 21:59</t>
+          <t>2026-05-11 22:17</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2086,12 +2086,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
+          <t>흑대추방울토마토 5kg</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2116,14 +2116,14 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011224</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-10 21:59</t>
+          <t>2026-05-11 22:17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2133,12 +2133,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
+          <t>흑대추방울토마토 2kg</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2163,14 +2163,14 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011223</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-10 22:00</t>
+          <t>2026-05-11 22:17</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2180,12 +2180,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
+          <t>흑대추방울토마토 1kg</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2210,14 +2210,14 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011222</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-10 22:00</t>
+          <t>2026-05-11 22:17</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2232,7 +2232,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2257,14 +2257,14 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-10 22:00</t>
+          <t>2026-05-11 22:17</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2304,14 +2304,14 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-10 22:00</t>
+          <t>2026-05-11 22:17</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2351,14 +2351,14 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-10 22:00</t>
+          <t>2026-05-11 22:17</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2398,14 +2398,14 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-10 22:00</t>
+          <t>2026-05-11 22:18</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2445,14 +2445,14 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-10 22:00</t>
+          <t>2026-05-11 22:18</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2492,14 +2492,14 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-10 22:00</t>
+          <t>2026-05-11 22:18</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2539,14 +2539,14 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-10 22:00</t>
+          <t>2026-05-11 22:18</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2586,14 +2586,14 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011123</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-10 22:01</t>
+          <t>2026-05-11 22:18</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2603,12 +2603,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토★4kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2633,14 +2633,14 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010320</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-10 22:01</t>
+          <t>2026-05-11 22:18</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2650,12 +2650,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토★3kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2680,14 +2680,14 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010319</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-10 22:01</t>
+          <t>2026-05-11 22:18</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2697,12 +2697,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토 4kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2727,14 +2727,14 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010318</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-10 22:01</t>
+          <t>2026-05-11 22:18</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2744,12 +2744,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토 3kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 혼합과</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2774,14 +2774,14 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010317</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011123</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-10 22:01</t>
+          <t>2026-05-11 22:19</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>(박스포함)★완숙토마토 10kg / 혼합과</t>
+          <t>(박스포함) 완숙토마토★4kg / 혼합과</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2821,14 +2821,14 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010108</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010320</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-10 22:02</t>
+          <t>2026-05-11 22:19</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>(박스포함)★완숙토마토 5kg / 혼합과</t>
+          <t>(박스포함) 완숙토마토★3kg / 혼합과</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2868,29 +2868,29 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010107</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010319</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-10 22:02</t>
+          <t>2026-05-11 22:19</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>(박스포함) 완숙토마토 4kg / 혼합과</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2915,29 +2915,29 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002048</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010318</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-10 22:03</t>
+          <t>2026-05-11 22:19</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>하우스 천도복숭아</t>
+          <t>(박스포함) 완숙토마토 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2962,29 +2962,29 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002047</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010317</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-10 22:03</t>
+          <t>2026-05-11 22:19</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>[예약판매] 하우스 대극천복숭아</t>
+          <t>(박스포함)★완숙토마토 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3009,14 +3009,14 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001975</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010107</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-10 22:03</t>
+          <t>2026-05-11 22:20</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3026,12 +3026,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>★특가★ 하우스 대석자두</t>
+          <t>정품 우곡수박</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3056,14 +3056,14 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002042</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002058</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-10 22:03</t>
+          <t>2026-05-11 22:21</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3073,12 +3073,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>하우스 대석자두</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3103,14 +3103,14 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001958</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002048</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-10 22:03</t>
+          <t>2026-05-11 22:21</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>하우스 털복숭아</t>
+          <t>하우스 천도복숭아</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3150,14 +3150,14 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001942</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002047</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-10 22:04</t>
+          <t>2026-05-11 22:21</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3167,12 +3167,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>★특가★ 가정용 하우스수박</t>
+          <t>[예약판매] 하우스 대극천복숭아</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3197,14 +3197,14 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001975</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-10 22:04</t>
+          <t>2026-05-11 22:21</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3214,12 +3214,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2026 국내산 햇감자</t>
+          <t>★특가★ 하우스 대석자두</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3244,14 +3244,14 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002042</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-10 22:04</t>
+          <t>2026-05-11 22:21</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3261,12 +3261,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>2026 국내산 햇양파</t>
+          <t>하우스 대석자두</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3291,14 +3291,14 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001958</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-05-10 22:04</t>
+          <t>2026-05-11 22:21</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3308,12 +3308,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외 (박스포함)</t>
+          <t>하우스 털복숭아</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3338,14 +3338,14 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001942</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-10 22:04</t>
+          <t>2026-05-11 22:22</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3355,12 +3355,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외</t>
+          <t>★특가★ 가정용 하우스수박</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3385,14 +3385,14 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-10 22:05</t>
+          <t>2026-05-11 22:22</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3402,12 +3402,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>★특가★ 짭짤이토마토</t>
+          <t>2026 국내산 햇감자</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3432,14 +3432,14 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001857</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-10 22:05</t>
+          <t>2026-05-11 22:22</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3449,12 +3449,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>★특가★ 대추방울토마토</t>
+          <t>2026 국내산 햇양파</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3479,14 +3479,14 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-05-10 22:05</t>
+          <t>2026-05-11 22:22</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3496,12 +3496,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>★특가★ 유럽종 완숙토마토</t>
+          <t>★특가★ 성주 꿀참외 (박스포함)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3526,14 +3526,14 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-10 22:05</t>
+          <t>2026-05-11 22:22</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3543,12 +3543,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>스테비아 방울토마토</t>
+          <t>★특가★ 성주 꿀참외</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3573,14 +3573,14 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-10 22:06</t>
+          <t>2026-05-11 22:23</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3595,7 +3595,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>흑대추방울토마토</t>
+          <t>★특가★ 짭짤이토마토</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3620,29 +3620,29 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001718</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001857</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-10 22:07</t>
+          <t>2026-05-11 22:23</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>★별담특가 가정용 참외★</t>
+          <t>★특가★ 대추방울토마토</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3667,29 +3667,29 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-05-10 22:07</t>
+          <t>2026-05-11 22:23</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>2026 햇양파</t>
+          <t>★특가★ 유럽종 완숙토마토</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3714,29 +3714,29 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-10 22:08</t>
+          <t>2026-05-11 22:24</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>스테비아 방울토마토</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3761,29 +3761,29 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-05-10 22:08</t>
+          <t>2026-05-11 22:24</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>흑대추방울토마토</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3808,14 +3808,14 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001718</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-10 22:09</t>
+          <t>2026-05-11 22:25</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3825,12 +3825,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>★별담특가 가정용 참외★</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3855,14 +3855,14 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-05-10 22:11</t>
+          <t>2026-05-11 22:25</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3872,12 +3872,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>대저 토마토</t>
+          <t>2026 햇양파</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3902,29 +3902,29 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008441</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-10 22:13</t>
+          <t>2026-05-11 22:26</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3949,29 +3949,29 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008676</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-05-10 22:13</t>
+          <t>2026-05-11 22:26</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3996,29 +3996,29 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-10 22:13</t>
+          <t>2026-05-11 22:26</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4043,29 +4043,29 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-05-10 22:14</t>
+          <t>2026-05-11 22:27</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>대저토마토</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4090,29 +4090,29 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-10 22:17</t>
+          <t>2026-05-11 22:29</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>🔥초특가🔥 [N-81] 가정용 성주참외</t>
+          <t>대저 토마토</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4137,29 +4137,29 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001101</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008441</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05-10 22:17</t>
+          <t>2026-05-11 22:31</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>[N-81] 가성비 성주참외</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -4184,19 +4184,19 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001013</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-10 22:17</t>
+          <t>2026-05-11 22:31</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4206,7 +4206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4231,29 +4231,29 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-05-10 22:17</t>
+          <t>2026-05-11 22:31</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>가정용 하우스수박 (기박)</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -4278,29 +4278,29 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-10 22:19</t>
+          <t>2026-05-11 22:32</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
+          <t>대저토마토</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -4325,19 +4325,19 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-05-10 22:20</t>
+          <t>2026-05-11 22:34</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4347,7 +4347,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
+          <t>★당도보장★ 농협선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -4372,29 +4372,29 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-10 22:20</t>
+          <t>2026-05-11 22:35</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>농협인증 당도선별 스테비아 수박</t>
+          <t>[N-81] 신비복숭아</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4419,29 +4419,29 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-05-10 22:20</t>
+          <t>2026-05-11 22:35</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>국내산 무주 수박무말랭이</t>
+          <t>🔥초특가🔥 [N-81] 가정용 성주참외</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4466,29 +4466,29 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001101</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-10 22:20</t>
+          <t>2026-05-11 22:35</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>정품 수박</t>
+          <t>[N-81] 가성비 성주참외</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4513,29 +4513,29 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001013</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-05-10 22:21</t>
+          <t>2026-05-11 22:35</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>대추 방울 토마토 소과</t>
+          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4560,19 +4560,19 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-10 22:21</t>
+          <t>2026-05-11 22:35</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -4582,7 +4582,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>가정용 흑수박 5kg 이상</t>
+          <t>가정용 하우스수박 (기박)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4607,14 +4607,14 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-05-10 22:22</t>
+          <t>2026-05-11 22:37</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4624,12 +4624,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
+          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4654,29 +4654,29 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-10 22:25</t>
+          <t>2026-05-11 22:38</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>❤️성주참외</t>
+          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4701,19 +4701,19 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-05-10 22:26</t>
+          <t>2026-05-11 22:38</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>농협인증 당도선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -4748,29 +4748,29 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-10 22:26</t>
+          <t>2026-05-11 22:38</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>국내산 무주 수박무말랭이</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4795,29 +4795,29 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-05-10 22:26</t>
+          <t>2026-05-11 22:39</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>정품 수박</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4842,29 +4842,29 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-10 22:26</t>
+          <t>2026-05-11 22:39</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>햇 홍감자</t>
+          <t>대추 방울 토마토 소과</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4889,29 +4889,29 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-05-10 22:26</t>
+          <t>2026-05-11 22:39</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>햇 설봉감자</t>
+          <t>가정용 흑수박 5kg 이상</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4936,29 +4936,29 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-10 22:26</t>
+          <t>2026-05-11 22:40</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>특가 대추방울토마토</t>
+          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4983,14 +4983,14 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-05-10 22:27</t>
+          <t>2026-05-11 22:44</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -5000,12 +5000,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>햇 수미감자</t>
+          <t>하우스 털 복숭아</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -5030,14 +5030,14 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-10 22:27</t>
+          <t>2026-05-11 22:44</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -5047,12 +5047,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>대저 흑대추방울토마토</t>
+          <t>❤️성주참외</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -5077,14 +5077,14 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-05-10 22:28</t>
+          <t>2026-05-11 22:44</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5094,12 +5094,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>부여 대추방울토마토</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -5124,14 +5124,14 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-10 22:29</t>
+          <t>2026-05-11 22:44</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -5141,12 +5141,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>성주참외</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5171,14 +5171,14 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001969</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-05-10 22:29</t>
+          <t>2026-05-11 22:44</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -5188,12 +5188,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>대저 토마토 / 짭짤이</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5218,19 +5218,19 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002113</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-05-10 22:31</t>
+          <t>2026-05-11 22:45</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>2026년 햇 감자</t>
+          <t>햇 홍감자</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5265,19 +5265,19 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-05-10 22:31</t>
+          <t>2026-05-11 22:45</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -5287,7 +5287,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>두백감자 ★7월 재오픈</t>
+          <t>햇 설봉감자</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -5312,29 +5312,29 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-05-10 22:31</t>
+          <t>2026-05-11 22:45</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>2026년 수미감자</t>
+          <t>특가 대추방울토마토</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5359,19 +5359,19 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-05-10 22:31</t>
+          <t>2026-05-11 22:45</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -5381,7 +5381,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>2026년 강원도감자</t>
+          <t>햇 수미감자</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -5406,29 +5406,29 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-05-10 22:31</t>
+          <t>2026-05-11 22:45</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>2025년 홍 감자</t>
+          <t>대저 흑대추방울토마토</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -5453,29 +5453,29 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-05-10 22:31</t>
+          <t>2026-05-11 22:46</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>부여 대추방울토마토</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5500,29 +5500,29 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-10 22:31</t>
+          <t>2026-05-11 22:48</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>유럽종 완숙토마토</t>
+          <t>성주참외</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5547,19 +5547,19 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001969</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-10 22:31</t>
+          <t>2026-05-11 22:48</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>대추 방울토마토</t>
+          <t>대저 토마토 / 짭짤이</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5594,14 +5594,14 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002113</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-10 22:31</t>
+          <t>2026-05-11 22:49</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5611,12 +5611,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>흑대추 방울 토마토</t>
+          <t>2026년 햇 감자</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5641,14 +5641,14 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-10 22:32</t>
+          <t>2026-05-11 22:49</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5658,12 +5658,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>고당도 성주 참외 ※선물세트 포함</t>
+          <t>두백감자 ★7월 재오픈</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5688,14 +5688,14 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-10 22:32</t>
+          <t>2026-05-11 22:49</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5710,7 +5710,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>스테비아 감자 ★7월 재오픈</t>
+          <t>2026년 수미감자</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5735,14 +5735,14 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-10 22:32</t>
+          <t>2026-05-11 22:49</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -5752,12 +5752,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>스테비야 방울토마토</t>
+          <t>2026년 강원도감자</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5782,14 +5782,14 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-10 22:32</t>
+          <t>2026-05-11 22:49</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -5799,35 +5799,364 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
+          <t>감자</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>2025년 홍 감자</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-05-11 22:50</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>감자</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>돼지감자</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-05-11 22:50</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
           <t>토마토</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr">
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>대추 방울토마토</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-05-11 22:50</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>토마토</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>흑대추 방울 토마토</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-05-11 22:50</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>참외</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>고당도 성주 참외 ※선물세트 포함</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-05-11 22:51</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>감자</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>스테비아 감자 ★7월 재오픈</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-05-11 22:51</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>토마토</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>스테비야 방울토마토</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-05-11 22:51</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>토마토</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
         <is>
           <t>스테비아 완숙 토마토</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H115" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I115" t="inlineStr">
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
         <is>
           <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000582</t>
         </is>

</xml_diff>

<commit_message>
Auto Update Prices: Tue May 12 22:58:06 UTC 2026
</commit_message>
<xml_diff>
--- a/가격이력.xlsx
+++ b/가격이력.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I122"/>
+  <dimension ref="A1:I131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-11 22:10</t>
+          <t>2026-05-12 22:15</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -525,7 +525,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-11 22:10</t>
+          <t>2026-05-12 22:15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -572,7 +572,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-11 22:11</t>
+          <t>2026-05-12 22:15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-11 22:11</t>
+          <t>2026-05-12 22:16</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-11 22:11</t>
+          <t>2026-05-12 22:16</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -713,7 +713,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-11 22:11</t>
+          <t>2026-05-12 22:16</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -760,7 +760,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-11 22:11</t>
+          <t>2026-05-12 22:16</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-11 22:11</t>
+          <t>2026-05-12 22:16</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-11 22:11</t>
+          <t>2026-05-12 22:16</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-11 22:12</t>
+          <t>2026-05-12 22:16</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -948,7 +948,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-11 22:12</t>
+          <t>2026-05-12 22:17</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -995,7 +995,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-11 22:12</t>
+          <t>2026-05-12 22:17</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-11 22:12</t>
+          <t>2026-05-12 22:17</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1089,7 +1089,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-11 22:13</t>
+          <t>2026-05-12 22:17</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1136,7 +1136,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-11 22:13</t>
+          <t>2026-05-12 22:18</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-11 22:13</t>
+          <t>2026-05-12 22:18</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1230,7 +1230,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-11 22:14</t>
+          <t>2026-05-12 22:19</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-11 22:14</t>
+          <t>2026-05-12 22:19</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1324,7 +1324,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-11 22:15</t>
+          <t>2026-05-12 22:20</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 혼합과</t>
+          <t>## (박스포함) 참외 가정용 / 10kg / 소과</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1364,14 +1364,14 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011646</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011733</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-11 22:15</t>
+          <t>2026-05-12 22:20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 대과</t>
+          <t>## (박스포함) 참외 가정용 / 10kg / 로얄과</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1411,14 +1411,14 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011645</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011732</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-11 22:16</t>
+          <t>2026-05-12 22:20</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 로얄과</t>
+          <t>## (박스포함) 참외 가정용 / 10kg / 대과</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1458,14 +1458,14 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011644</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011731</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-11 22:16</t>
+          <t>2026-05-12 22:20</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 소과</t>
+          <t>## (박스포함) 참외 가정용 / 10kg / 혼합과</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1505,14 +1505,14 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011643</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011730</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-11 22:16</t>
+          <t>2026-05-12 22:20</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 혼합과</t>
+          <t>## (박스포함) 참외 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1552,14 +1552,14 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011642</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011729</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-11 22:16</t>
+          <t>2026-05-12 22:20</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 대과</t>
+          <t>## (박스포함) 참외 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1599,14 +1599,14 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011641</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011728</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-11 22:16</t>
+          <t>2026-05-12 22:20</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 로얄과</t>
+          <t>## (박스포함) 참외 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1646,14 +1646,14 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011640</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011727</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-11 22:16</t>
+          <t>2026-05-12 22:20</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 소과</t>
+          <t>## (박스포함) 참외 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1693,14 +1693,14 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011639</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011726</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-11 22:16</t>
+          <t>2026-05-12 22:21</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 혼합과</t>
+          <t>## (박스포함) 참외 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1740,14 +1740,14 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011638</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011725</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-11 22:16</t>
+          <t>2026-05-12 22:21</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 대과</t>
+          <t>## (박스포함) 참외 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1787,14 +1787,14 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011637</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011724</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-11 22:16</t>
+          <t>2026-05-12 22:21</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 로얄과</t>
+          <t>## (박스포함) 참외 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1834,14 +1834,14 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011636</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011723</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-11 22:16</t>
+          <t>2026-05-12 22:21</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 소과</t>
+          <t>## (박스포함) 참외 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1881,14 +1881,14 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011635</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011722</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-11 22:17</t>
+          <t>2026-05-12 22:21</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1898,12 +1898,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
+          <t>특가 ★ 대추방울토마토 5kg / 대과 / 1-2번과</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1928,14 +1928,14 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011721</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-11 22:17</t>
+          <t>2026-05-12 22:21</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1945,12 +1945,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
+          <t>특가 ★ 대추방울토마토 2kg / 대과 / 1-2번과</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1975,14 +1975,14 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011720</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-11 22:17</t>
+          <t>2026-05-12 22:21</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1992,12 +1992,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
+          <t>특가 ★ 대추방울토마토 1kg / 대과 / 1-2번과</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2022,14 +2022,14 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011719</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-11 22:17</t>
+          <t>2026-05-12 22:21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
+          <t>행사 (박스포함) 참외 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2069,14 +2069,14 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011646</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-11 22:17</t>
+          <t>2026-05-12 22:21</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2086,12 +2086,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>흑대추방울토마토 5kg</t>
+          <t>행사 (박스포함) 참외 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2116,14 +2116,14 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011224</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011645</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-11 22:17</t>
+          <t>2026-05-12 22:21</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2133,12 +2133,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>흑대추방울토마토 2kg</t>
+          <t>행사 (박스포함) 참외 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2163,14 +2163,14 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011223</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011644</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-11 22:17</t>
+          <t>2026-05-12 22:22</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2180,12 +2180,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>흑대추방울토마토 1kg</t>
+          <t>행사 (박스포함) 참외 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2210,14 +2210,14 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011222</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011643</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-11 22:17</t>
+          <t>2026-05-12 22:22</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2232,7 +2232,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
+          <t>행사 (박스포함) 참외 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2257,14 +2257,14 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011642</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-11 22:17</t>
+          <t>2026-05-12 22:22</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
+          <t>행사 (박스포함) 참외 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2304,14 +2304,14 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011641</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-11 22:17</t>
+          <t>2026-05-12 22:22</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
+          <t>행사 (박스포함) 참외 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2351,14 +2351,14 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011640</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-11 22:17</t>
+          <t>2026-05-12 22:22</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
+          <t>행사 (박스포함) 참외 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2398,14 +2398,14 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011639</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-11 22:18</t>
+          <t>2026-05-12 22:22</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
+          <t>행사 (박스포함) 참외 가정용 / 10kg / 혼합과</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2445,14 +2445,14 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011638</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-11 22:18</t>
+          <t>2026-05-12 22:22</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
+          <t>행사 (박스포함) 참외 가정용 / 10kg / 대과</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2492,14 +2492,14 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011637</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-11 22:18</t>
+          <t>2026-05-12 22:22</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
+          <t>행사 (박스포함) 참외 가정용 / 10kg / 로얄과</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2539,14 +2539,14 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011636</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-11 22:18</t>
+          <t>2026-05-12 22:22</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
+          <t>행사 (박스포함) 참외 가정용 / 10kg / 소과</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2586,14 +2586,14 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011635</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-11 22:18</t>
+          <t>2026-05-12 22:22</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2633,14 +2633,14 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-11 22:18</t>
+          <t>2026-05-12 22:23</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2680,14 +2680,14 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-11 22:18</t>
+          <t>2026-05-12 22:23</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2727,14 +2727,14 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-11 22:18</t>
+          <t>2026-05-12 22:23</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2774,14 +2774,14 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011123</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-11 22:19</t>
+          <t>2026-05-12 22:23</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토★4kg / 혼합과</t>
+          <t>흑대추방울토마토 5kg</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2821,14 +2821,14 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010320</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011224</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-11 22:19</t>
+          <t>2026-05-12 22:23</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토★3kg / 혼합과</t>
+          <t>흑대추방울토마토 2kg</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2868,14 +2868,14 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010319</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011223</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-11 22:19</t>
+          <t>2026-05-12 22:23</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토 4kg / 혼합과</t>
+          <t>흑대추방울토마토 1kg</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2915,14 +2915,14 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010318</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011222</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-11 22:19</t>
+          <t>2026-05-12 22:23</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2932,12 +2932,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토 3kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2962,14 +2962,14 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010317</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-11 22:19</t>
+          <t>2026-05-12 22:23</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2979,12 +2979,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>(박스포함)★완숙토마토 5kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3009,29 +3009,29 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010107</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-11 22:20</t>
+          <t>2026-05-12 22:23</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>정품 우곡수박</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3056,29 +3056,29 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002058</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-11 22:21</t>
+          <t>2026-05-12 22:23</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3103,29 +3103,29 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002048</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-11 22:21</t>
+          <t>2026-05-12 22:23</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>하우스 천도복숭아</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3150,29 +3150,29 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002047</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-11 22:21</t>
+          <t>2026-05-12 22:24</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>[예약판매] 하우스 대극천복숭아</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3197,29 +3197,29 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001975</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-11 22:21</t>
+          <t>2026-05-12 22:24</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>★특가★ 하우스 대석자두</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3244,29 +3244,29 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002042</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-11 22:21</t>
+          <t>2026-05-12 22:24</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>하우스 대석자두</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3291,29 +3291,29 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001958</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-05-11 22:21</t>
+          <t>2026-05-12 22:24</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>하우스 털복숭아</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3338,29 +3338,29 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001942</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-11 22:22</t>
+          <t>2026-05-12 22:24</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>★특가★ 가정용 하우스수박</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3385,29 +3385,29 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-11 22:22</t>
+          <t>2026-05-12 22:24</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>2026 국내산 햇감자</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3432,14 +3432,14 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-11 22:22</t>
+          <t>2026-05-12 22:25</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3449,12 +3449,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2026 국내산 햇양파</t>
+          <t>정품 우곡수박</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3479,14 +3479,14 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002058</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-05-11 22:22</t>
+          <t>2026-05-12 22:25</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3496,12 +3496,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외 (박스포함)</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3526,14 +3526,14 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002048</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-11 22:22</t>
+          <t>2026-05-12 22:25</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3543,12 +3543,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외</t>
+          <t>하우스 천도복숭아</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3573,14 +3573,14 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002047</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-11 22:23</t>
+          <t>2026-05-12 22:25</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3590,12 +3590,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>★특가★ 짭짤이토마토</t>
+          <t>[예약판매] 하우스 대극천복숭아</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3620,14 +3620,14 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001857</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001975</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-11 22:23</t>
+          <t>2026-05-12 22:26</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3637,12 +3637,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>★특가★ 대추방울토마토</t>
+          <t>★특가★ 하우스 대석자두</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3667,14 +3667,14 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002042</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-05-11 22:23</t>
+          <t>2026-05-12 22:26</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3684,12 +3684,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>★특가★ 유럽종 완숙토마토</t>
+          <t>하우스 대석자두</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3714,14 +3714,14 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001958</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-11 22:24</t>
+          <t>2026-05-12 22:26</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3731,12 +3731,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>스테비아 방울토마토</t>
+          <t>하우스 털복숭아</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3761,14 +3761,14 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001942</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-05-11 22:24</t>
+          <t>2026-05-12 22:26</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3778,12 +3778,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>흑대추방울토마토</t>
+          <t>★특가★ 가정용 하우스수박</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3808,29 +3808,29 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001718</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-11 22:25</t>
+          <t>2026-05-12 22:27</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>★별담특가 가정용 참외★</t>
+          <t>2026 국내산 햇감자</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3855,19 +3855,19 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-05-11 22:25</t>
+          <t>2026-05-12 22:27</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3877,7 +3877,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>2026 햇양파</t>
+          <t>2026 국내산 햇양파</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3902,29 +3902,29 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-11 22:26</t>
+          <t>2026-05-12 22:27</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>★특가★ 성주 꿀참외 (박스포함)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3949,29 +3949,29 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008676</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-05-11 22:26</t>
+          <t>2026-05-12 22:27</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>★특가★ 성주 꿀참외</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3996,29 +3996,29 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-11 22:26</t>
+          <t>2026-05-12 22:28</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>★특가★ 짭짤이토마토</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4043,29 +4043,29 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001857</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-05-11 22:27</t>
+          <t>2026-05-12 22:28</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>★특가★ 대추방울토마토</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4090,19 +4090,19 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-11 22:29</t>
+          <t>2026-05-12 22:28</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>대저 토마토</t>
+          <t>★특가★ 유럽종 완숙토마토</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4137,19 +4137,19 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008441</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05-11 22:31</t>
+          <t>2026-05-12 22:28</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4159,7 +4159,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>스테비아 방울토마토</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -4184,29 +4184,29 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-11 22:31</t>
+          <t>2026-05-12 22:29</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>흑대추방울토마토</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4231,29 +4231,29 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001718</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-05-11 22:31</t>
+          <t>2026-05-12 22:30</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>★별담특가 가정용 참외★</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -4278,29 +4278,29 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-11 22:32</t>
+          <t>2026-05-12 22:30</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>대저토마토</t>
+          <t>2026 햇양파</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -4325,29 +4325,29 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-05-11 22:34</t>
+          <t>2026-05-12 22:30</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>★당도보장★ 농협선별 스테비아 수박</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -4372,19 +4372,19 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008676</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-11 22:35</t>
+          <t>2026-05-12 22:30</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>[N-81] 신비복숭아</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4419,29 +4419,29 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-05-11 22:35</t>
+          <t>2026-05-12 22:31</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>🔥초특가🔥 [N-81] 가정용 성주참외</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4466,29 +4466,29 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001101</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-11 22:35</t>
+          <t>2026-05-12 22:31</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>[N-81] 가성비 성주참외</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4513,29 +4513,29 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001013</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-05-11 22:35</t>
+          <t>2026-05-12 22:33</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
+          <t>대저 토마토</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4560,29 +4560,29 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008441</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-11 22:35</t>
+          <t>2026-05-12 22:35</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>가정용 하우스수박 (기박)</t>
+          <t>햇 감자</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4607,29 +4607,29 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002108</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-05-11 22:37</t>
+          <t>2026-05-12 22:36</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4654,29 +4654,29 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-11 22:38</t>
+          <t>2026-05-12 22:36</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4701,29 +4701,29 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-05-11 22:38</t>
+          <t>2026-05-12 22:36</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>농협인증 당도선별 스테비아 수박</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -4748,29 +4748,29 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-11 22:38</t>
+          <t>2026-05-12 22:36</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>국내산 무주 수박무말랭이</t>
+          <t>대저토마토</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4795,19 +4795,19 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-05-11 22:39</t>
+          <t>2026-05-12 22:39</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>정품 수박</t>
+          <t>★당도보장★ 농협선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4842,29 +4842,29 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-11 22:39</t>
+          <t>2026-05-12 22:39</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>대추 방울 토마토 소과</t>
+          <t>[N-81] 신비복숭아</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4889,29 +4889,29 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-05-11 22:39</t>
+          <t>2026-05-12 22:39</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>가정용 흑수박 5kg 이상</t>
+          <t>🔥초특가🔥 [N-81] 가정용 성주참외</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4936,19 +4936,19 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001101</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-11 22:40</t>
+          <t>2026-05-12 22:40</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
+          <t>[N-81] 가성비 성주참외</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4983,29 +4983,29 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001013</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-05-11 22:44</t>
+          <t>2026-05-12 22:40</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>하우스 털 복숭아</t>
+          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -5030,29 +5030,29 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-11 22:44</t>
+          <t>2026-05-12 22:40</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>❤️성주참외</t>
+          <t>가정용 하우스수박 (기박)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -5077,19 +5077,19 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-05-11 22:44</t>
+          <t>2026-05-12 22:42</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -5124,29 +5124,29 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-11 22:44</t>
+          <t>2026-05-12 22:42</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5171,29 +5171,29 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-05-11 22:44</t>
+          <t>2026-05-12 22:43</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>농협인증 당도선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5218,29 +5218,29 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-05-11 22:45</t>
+          <t>2026-05-12 22:43</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>햇 홍감자</t>
+          <t>국내산 무주 수박무말랭이</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5265,29 +5265,29 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-05-11 22:45</t>
+          <t>2026-05-12 22:43</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>햇 설봉감자</t>
+          <t>정품 수박</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -5312,19 +5312,19 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-05-11 22:45</t>
+          <t>2026-05-12 22:43</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -5334,7 +5334,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>특가 대추방울토마토</t>
+          <t>대추 방울 토마토 소과</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5359,29 +5359,29 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-05-11 22:45</t>
+          <t>2026-05-12 22:43</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>햇 수미감자</t>
+          <t>가정용 흑수박 5kg 이상</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -5406,29 +5406,29 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-05-11 22:45</t>
+          <t>2026-05-12 22:44</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>대저 흑대추방울토마토</t>
+          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -5453,14 +5453,14 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-05-11 22:46</t>
+          <t>2026-05-12 22:48</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -5470,12 +5470,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>부여 대추방울토마토</t>
+          <t>[고품위] 하우스 털 복숭아</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5500,14 +5500,14 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-11 22:48</t>
+          <t>2026-05-12 22:48</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>성주참외</t>
+          <t>❤️성주참외</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5547,14 +5547,14 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001969</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-11 22:48</t>
+          <t>2026-05-12 22:49</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5564,12 +5564,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>대저 토마토 / 짭짤이</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5594,29 +5594,29 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002113</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-11 22:49</t>
+          <t>2026-05-12 22:49</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>2026년 햇 감자</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5641,29 +5641,29 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-11 22:49</t>
+          <t>2026-05-12 22:49</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>두백감자 ★7월 재오픈</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5688,19 +5688,19 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-11 22:49</t>
+          <t>2026-05-12 22:49</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -5710,7 +5710,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>2026년 수미감자</t>
+          <t>햇 홍감자</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5735,19 +5735,19 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-11 22:49</t>
+          <t>2026-05-12 22:49</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -5757,7 +5757,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>2026년 강원도감자</t>
+          <t>햇 설봉감자</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5782,29 +5782,29 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-11 22:49</t>
+          <t>2026-05-12 22:49</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2025년 홍 감자</t>
+          <t>특가 대추방울토마토</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5829,19 +5829,19 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-11 22:50</t>
+          <t>2026-05-12 22:50</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>햇 수미감자</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -5876,19 +5876,19 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-11 22:50</t>
+          <t>2026-05-12 22:50</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -5898,7 +5898,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>대추 방울토마토</t>
+          <t>대저 흑대추방울토마토</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5923,19 +5923,19 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-11 22:50</t>
+          <t>2026-05-12 22:50</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -5945,7 +5945,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>흑대추 방울 토마토</t>
+          <t>부여 대추방울토마토</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5970,29 +5970,29 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-11 22:50</t>
+          <t>2026-05-12 22:52</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>고당도 성주 참외 ※선물세트 포함</t>
+          <t>대저 토마토 / 짭짤이</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -6017,14 +6017,14 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002113</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-11 22:51</t>
+          <t>2026-05-12 22:53</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -6039,7 +6039,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>스테비아 감자 ★7월 재오픈</t>
+          <t>2026년 햇 감자</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -6064,14 +6064,14 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-11 22:51</t>
+          <t>2026-05-12 22:53</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -6081,12 +6081,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>스테비야 방울토마토</t>
+          <t>두백감자 ★7월 재오픈</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -6111,14 +6111,14 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-11 22:51</t>
+          <t>2026-05-12 22:53</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -6128,35 +6128,458 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
+          <t>감자</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>2026년 수미감자</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-05-12 22:54</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>감자</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>2026년 강원도감자</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-05-12 22:54</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>감자</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>2025년 홍 감자</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-05-12 22:54</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>감자</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>돼지감자</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-05-12 22:54</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
           <t>토마토</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr">
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>대추 방울토마토</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-05-12 22:54</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>토마토</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>흑대추 방울 토마토</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-05-12 22:54</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>참외</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>고당도 성주 참외 ※선물세트 포함</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-05-12 22:55</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>감자</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>스테비아 감자 ★7월 재오픈</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-05-12 22:55</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>토마토</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>스테비야 방울토마토</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-05-12 22:55</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>토마토</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
         <is>
           <t>스테비아 완숙 토마토</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H122" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I122" t="inlineStr">
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
         <is>
           <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000582</t>
         </is>

</xml_diff>

<commit_message>
Auto Update Prices: Wed May 13 22:59:48 UTC 2026
</commit_message>
<xml_diff>
--- a/가격이력.xlsx
+++ b/가격이력.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I131"/>
+  <dimension ref="A1:I124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-12 22:15</t>
+          <t>2026-05-13 22:17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -525,7 +525,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-12 22:15</t>
+          <t>2026-05-13 22:17</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -572,7 +572,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-12 22:15</t>
+          <t>2026-05-13 22:17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-12 22:16</t>
+          <t>2026-05-13 22:17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-12 22:16</t>
+          <t>2026-05-13 22:17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -713,7 +713,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-12 22:16</t>
+          <t>2026-05-13 22:18</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -760,7 +760,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-12 22:16</t>
+          <t>2026-05-13 22:18</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-12 22:16</t>
+          <t>2026-05-13 22:18</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-12 22:16</t>
+          <t>2026-05-13 22:18</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-12 22:16</t>
+          <t>2026-05-13 22:18</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -948,7 +948,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-12 22:17</t>
+          <t>2026-05-13 22:18</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -995,7 +995,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-12 22:17</t>
+          <t>2026-05-13 22:18</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-12 22:17</t>
+          <t>2026-05-13 22:19</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1089,7 +1089,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-12 22:17</t>
+          <t>2026-05-13 22:19</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1136,7 +1136,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-12 22:18</t>
+          <t>2026-05-13 22:19</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-12 22:18</t>
+          <t>2026-05-13 22:20</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1230,7 +1230,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-12 22:19</t>
+          <t>2026-05-13 22:20</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-12 22:19</t>
+          <t>2026-05-13 22:21</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1324,7 +1324,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-12 22:20</t>
+          <t>2026-05-13 22:22</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>## (박스포함) 참외 가정용 / 10kg / 소과</t>
+          <t>행사 (박스포함) 참외 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1364,14 +1364,14 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011733</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011646</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-12 22:20</t>
+          <t>2026-05-13 22:22</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>## (박스포함) 참외 가정용 / 10kg / 로얄과</t>
+          <t>행사 (박스포함) 참외 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1411,14 +1411,14 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011732</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011645</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-12 22:20</t>
+          <t>2026-05-13 22:22</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>## (박스포함) 참외 가정용 / 10kg / 대과</t>
+          <t>행사 (박스포함) 참외 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1458,14 +1458,14 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011731</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011644</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-12 22:20</t>
+          <t>2026-05-13 22:22</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>## (박스포함) 참외 가정용 / 10kg / 혼합과</t>
+          <t>행사 (박스포함) 참외 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1505,14 +1505,14 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011730</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011643</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-12 22:20</t>
+          <t>2026-05-13 22:22</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>## (박스포함) 참외 가정용 / 5kg / 소과</t>
+          <t>행사 (박스포함) 참외 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1552,14 +1552,14 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011729</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011642</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-12 22:20</t>
+          <t>2026-05-13 22:22</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>## (박스포함) 참외 가정용 / 5kg / 로얄과</t>
+          <t>행사 (박스포함) 참외 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1599,14 +1599,14 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011728</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011641</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-12 22:20</t>
+          <t>2026-05-13 22:22</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>## (박스포함) 참외 가정용 / 5kg / 대과</t>
+          <t>행사 (박스포함) 참외 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1646,14 +1646,14 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011727</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011640</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-12 22:20</t>
+          <t>2026-05-13 22:22</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>## (박스포함) 참외 가정용 / 5kg / 혼합과</t>
+          <t>행사 (박스포함) 참외 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1693,14 +1693,14 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011726</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011639</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-12 22:21</t>
+          <t>2026-05-13 22:22</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>## (박스포함) 참외 가정용 / 3kg / 소과</t>
+          <t>행사 (박스포함) 참외 가정용 / 10kg / 혼합과</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1740,14 +1740,14 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011725</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011638</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-12 22:21</t>
+          <t>2026-05-13 22:22</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>## (박스포함) 참외 가정용 / 3kg / 로얄과</t>
+          <t>행사 (박스포함) 참외 가정용 / 10kg / 대과</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1787,14 +1787,14 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011724</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011637</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-12 22:21</t>
+          <t>2026-05-13 22:23</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>## (박스포함) 참외 가정용 / 3kg / 대과</t>
+          <t>행사 (박스포함) 참외 가정용 / 10kg / 로얄과</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1834,14 +1834,14 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011723</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011636</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-12 22:21</t>
+          <t>2026-05-13 22:23</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>## (박스포함) 참외 가정용 / 3kg / 혼합과</t>
+          <t>행사 (박스포함) 참외 가정용 / 10kg / 소과</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1881,14 +1881,14 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011722</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011635</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-12 22:21</t>
+          <t>2026-05-13 22:23</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1898,12 +1898,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>특가 ★ 대추방울토마토 5kg / 대과 / 1-2번과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1928,14 +1928,14 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011721</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-12 22:21</t>
+          <t>2026-05-13 22:23</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1945,12 +1945,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>특가 ★ 대추방울토마토 2kg / 대과 / 1-2번과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1975,14 +1975,14 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011720</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-12 22:21</t>
+          <t>2026-05-13 22:23</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1992,12 +1992,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>특가 ★ 대추방울토마토 1kg / 대과 / 1-2번과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2022,14 +2022,14 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011719</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-12 22:21</t>
+          <t>2026-05-13 22:23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2069,14 +2069,14 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011646</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-12 22:21</t>
+          <t>2026-05-13 22:23</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2086,12 +2086,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 대과</t>
+          <t>흑대추방울토마토 5kg</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2116,14 +2116,14 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011645</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011224</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-12 22:21</t>
+          <t>2026-05-13 22:23</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2133,12 +2133,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 로얄과</t>
+          <t>흑대추방울토마토 2kg</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2163,14 +2163,14 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011644</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011223</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-12 22:22</t>
+          <t>2026-05-13 22:23</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2180,12 +2180,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 소과</t>
+          <t>흑대추방울토마토 1kg</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2210,14 +2210,14 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011643</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011222</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-12 22:22</t>
+          <t>2026-05-13 22:23</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2232,7 +2232,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2257,14 +2257,14 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011642</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-12 22:22</t>
+          <t>2026-05-13 22:24</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2304,14 +2304,14 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011641</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-12 22:22</t>
+          <t>2026-05-13 22:24</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2351,14 +2351,14 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011640</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-12 22:22</t>
+          <t>2026-05-13 22:24</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2398,14 +2398,14 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011639</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-12 22:22</t>
+          <t>2026-05-13 22:24</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2445,14 +2445,14 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011638</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-12 22:22</t>
+          <t>2026-05-13 22:24</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2492,14 +2492,14 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011637</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-12 22:22</t>
+          <t>2026-05-13 22:24</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2539,14 +2539,14 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011636</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-12 22:22</t>
+          <t>2026-05-13 22:24</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2586,14 +2586,14 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011635</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-12 22:22</t>
+          <t>2026-05-13 22:24</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2633,14 +2633,14 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-12 22:23</t>
+          <t>2026-05-13 22:24</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2680,14 +2680,14 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-12 22:23</t>
+          <t>2026-05-13 22:24</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2727,14 +2727,14 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-12 22:23</t>
+          <t>2026-05-13 22:24</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 혼합과</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2774,14 +2774,14 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011123</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-12 22:23</t>
+          <t>2026-05-13 22:25</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>흑대추방울토마토 5kg</t>
+          <t>(박스포함) 완숙토마토★4kg / 혼합과</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2821,14 +2821,14 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011224</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010320</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-12 22:23</t>
+          <t>2026-05-13 22:25</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>흑대추방울토마토 2kg</t>
+          <t>(박스포함) 완숙토마토★3kg / 혼합과</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2868,14 +2868,14 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011223</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010319</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-12 22:23</t>
+          <t>2026-05-13 22:25</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>흑대추방울토마토 1kg</t>
+          <t>(박스포함) 완숙토마토 4kg / 혼합과</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2915,14 +2915,14 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011222</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010318</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-12 22:23</t>
+          <t>2026-05-13 22:25</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2932,12 +2932,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
+          <t>(박스포함) 완숙토마토 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2962,29 +2962,29 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010317</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-12 22:23</t>
+          <t>2026-05-13 22:27</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
+          <t>정품 우곡수박</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3009,29 +3009,29 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002058</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-12 22:23</t>
+          <t>2026-05-13 22:27</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3056,29 +3056,29 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002048</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-12 22:23</t>
+          <t>2026-05-13 22:27</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
+          <t>하우스 천도복숭아</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3103,29 +3103,29 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002047</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-12 22:23</t>
+          <t>2026-05-13 22:27</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
+          <t>[예약판매] 하우스 대극천복숭아</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3150,29 +3150,29 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001975</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-12 22:24</t>
+          <t>2026-05-13 22:27</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
+          <t>★특가★ 하우스 대석자두</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3197,29 +3197,29 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002042</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-12 22:24</t>
+          <t>2026-05-13 22:28</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
+          <t>하우스 대석자두</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3244,29 +3244,29 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001958</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-12 22:24</t>
+          <t>2026-05-13 22:28</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
+          <t>하우스 털복숭아</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3291,29 +3291,29 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001942</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-05-12 22:24</t>
+          <t>2026-05-13 22:28</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
+          <t>★특가★ 가정용 하우스수박</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3338,29 +3338,29 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-12 22:24</t>
+          <t>2026-05-13 22:28</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
+          <t>2026 국내산 햇감자</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3385,29 +3385,29 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-12 22:24</t>
+          <t>2026-05-13 22:29</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
+          <t>2026 국내산 햇양파</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3432,14 +3432,14 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-12 22:25</t>
+          <t>2026-05-13 22:29</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3449,12 +3449,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>정품 우곡수박</t>
+          <t>★특가★ 성주 꿀참외 (박스포함)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3479,14 +3479,14 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002058</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-05-12 22:25</t>
+          <t>2026-05-13 22:29</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3496,12 +3496,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>★특가★ 성주 꿀참외</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3526,14 +3526,14 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002048</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-12 22:25</t>
+          <t>2026-05-13 22:29</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3543,12 +3543,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>하우스 천도복숭아</t>
+          <t>★특가★ 짭짤이토마토</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3573,14 +3573,14 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002047</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001857</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-12 22:25</t>
+          <t>2026-05-13 22:29</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3590,12 +3590,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>[예약판매] 하우스 대극천복숭아</t>
+          <t>★특가★ 대추방울토마토</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3620,14 +3620,14 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001975</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-12 22:26</t>
+          <t>2026-05-13 22:29</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3637,12 +3637,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>★특가★ 하우스 대석자두</t>
+          <t>★특가★ 유럽종 완숙토마토</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3667,14 +3667,14 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002042</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-05-12 22:26</t>
+          <t>2026-05-13 22:30</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3684,12 +3684,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>하우스 대석자두</t>
+          <t>스테비아 방울토마토</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3714,14 +3714,14 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001958</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-12 22:26</t>
+          <t>2026-05-13 22:30</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3731,12 +3731,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>하우스 털복숭아</t>
+          <t>흑대추방울토마토</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3761,29 +3761,29 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001942</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001718</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-05-12 22:26</t>
+          <t>2026-05-13 22:31</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>★특가★ 가정용 하우스수박</t>
+          <t>★별담특가 가정용 참외★</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3808,29 +3808,29 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-12 22:27</t>
+          <t>2026-05-13 22:32</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>2026 국내산 햇감자</t>
+          <t>2026 햇양파</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3855,29 +3855,29 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-05-12 22:27</t>
+          <t>2026-05-13 22:32</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>2026 국내산 햇양파</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3902,29 +3902,29 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008676</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-12 22:27</t>
+          <t>2026-05-13 22:32</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외 (박스포함)</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3949,29 +3949,29 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-05-12 22:27</t>
+          <t>2026-05-13 22:32</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3996,29 +3996,29 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-12 22:28</t>
+          <t>2026-05-13 22:33</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>★특가★ 짭짤이토마토</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4043,19 +4043,19 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001857</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-05-12 22:28</t>
+          <t>2026-05-13 22:35</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -4065,7 +4065,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>★특가★ 대추방울토마토</t>
+          <t>대저 토마토</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4090,29 +4090,29 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008441</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-12 22:28</t>
+          <t>2026-05-13 22:37</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>★특가★ 유럽종 완숙토마토</t>
+          <t>★특가★ 가성비 참외</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4137,29 +4137,29 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002133</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05-12 22:28</t>
+          <t>2026-05-13 22:37</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>스테비아 방울토마토</t>
+          <t>햇 감자</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -4184,29 +4184,29 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002108</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-12 22:29</t>
+          <t>2026-05-13 22:37</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>흑대추방울토마토</t>
+          <t>햇 양파</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4231,29 +4231,29 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001718</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000186</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-05-12 22:30</t>
+          <t>2026-05-13 22:37</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>★별담특가 가정용 참외★</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -4278,29 +4278,29 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-12 22:30</t>
+          <t>2026-05-13 22:38</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>2026 햇양파</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -4325,29 +4325,29 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-05-12 22:30</t>
+          <t>2026-05-13 22:38</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -4372,29 +4372,29 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008676</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-12 22:30</t>
+          <t>2026-05-13 22:38</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>대저토마토</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4419,29 +4419,29 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-05-12 22:31</t>
+          <t>2026-05-13 22:41</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>★당도보장★ 농협선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4466,29 +4466,29 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-12 22:31</t>
+          <t>2026-05-13 22:41</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>[N-81] 신비복숭아</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4513,29 +4513,29 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-05-12 22:33</t>
+          <t>2026-05-13 22:41</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>대저 토마토</t>
+          <t>[N-81] 가정용 성주참외</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4560,29 +4560,29 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008441</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001101</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-12 22:35</t>
+          <t>2026-05-13 22:42</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>햇 감자</t>
+          <t>[N-81] 가성비 성주참외</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4607,29 +4607,29 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002108</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001013</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-05-12 22:36</t>
+          <t>2026-05-13 22:42</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4654,29 +4654,29 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-12 22:36</t>
+          <t>2026-05-13 22:42</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>가정용 하우스수박 (기박)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4701,29 +4701,29 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-05-12 22:36</t>
+          <t>2026-05-13 22:44</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -4748,29 +4748,29 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-12 22:36</t>
+          <t>2026-05-13 22:45</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>대저토마토</t>
+          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4795,19 +4795,19 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-05-12 22:39</t>
+          <t>2026-05-13 22:45</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>★당도보장★ 농협선별 스테비아 수박</t>
+          <t>농협인증 당도선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4842,29 +4842,29 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-12 22:39</t>
+          <t>2026-05-13 22:45</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>[N-81] 신비복숭아</t>
+          <t>국내산 무주 수박무말랭이</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4889,29 +4889,29 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-05-12 22:39</t>
+          <t>2026-05-13 22:45</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>🔥초특가🔥 [N-81] 가정용 성주참외</t>
+          <t>정품 수박</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4936,29 +4936,29 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001101</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-12 22:40</t>
+          <t>2026-05-13 22:45</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>[N-81] 가성비 성주참외</t>
+          <t>대추 방울 토마토 소과</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4983,29 +4983,29 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001013</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-05-12 22:40</t>
+          <t>2026-05-13 22:46</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
+          <t>가정용 흑수박 5kg 이상</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -5030,29 +5030,29 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-12 22:40</t>
+          <t>2026-05-13 22:47</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>가정용 하우스수박 (기박)</t>
+          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -5077,29 +5077,29 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-05-12 22:42</t>
+          <t>2026-05-13 22:50</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
+          <t>성주참외</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -5124,29 +5124,29 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003357</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-12 22:42</t>
+          <t>2026-05-13 22:50</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
+          <t>❤️성주참외</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5171,19 +5171,19 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-05-12 22:43</t>
+          <t>2026-05-13 22:50</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>농협인증 당도선별 스테비아 수박</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5218,29 +5218,29 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-05-12 22:43</t>
+          <t>2026-05-13 22:50</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>국내산 무주 수박무말랭이</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5265,29 +5265,29 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-05-12 22:43</t>
+          <t>2026-05-13 22:50</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>정품 수박</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -5312,29 +5312,29 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-05-12 22:43</t>
+          <t>2026-05-13 22:51</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>대추 방울 토마토 소과</t>
+          <t>[고품위] 하우스 털 복숭아</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5359,29 +5359,29 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-05-12 22:43</t>
+          <t>2026-05-13 22:52</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>가정용 흑수박 5kg 이상</t>
+          <t>햇 홍감자</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -5406,29 +5406,29 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-05-12 22:44</t>
+          <t>2026-05-13 22:52</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
+          <t>햇 설봉감자</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -5453,14 +5453,14 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-05-12 22:48</t>
+          <t>2026-05-13 22:52</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -5470,12 +5470,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>[고품위] 하우스 털 복숭아</t>
+          <t>특가 대추방울토마토</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5500,14 +5500,14 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-12 22:48</t>
+          <t>2026-05-13 22:52</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5517,12 +5517,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>❤️성주참외</t>
+          <t>햇 수미감자</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5547,14 +5547,14 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-12 22:49</t>
+          <t>2026-05-13 22:52</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5564,12 +5564,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>대저 흑대추방울토마토</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5594,14 +5594,14 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-12 22:49</t>
+          <t>2026-05-13 22:53</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5611,12 +5611,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>부여 대추방울토마토</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5641,14 +5641,14 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-12 22:49</t>
+          <t>2026-05-13 22:54</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5658,12 +5658,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>대저 토마토 / 짭짤이</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5688,19 +5688,19 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002113</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-12 22:49</t>
+          <t>2026-05-13 22:55</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>더그린</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -5710,7 +5710,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>햇 홍감자</t>
+          <t>2026년 강원도감자</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5735,19 +5735,19 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-12 22:49</t>
+          <t>2026-05-13 22:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>더그린</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -5757,7 +5757,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>햇 설봉감자</t>
+          <t>2026년 수미감자</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5782,29 +5782,29 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-12 22:49</t>
+          <t>2026-05-13 22:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>더그린</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>특가 대추방울토마토</t>
+          <t>2026년 햇 감자</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5829,19 +5829,19 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-12 22:50</t>
+          <t>2026-05-13 22:55</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>더그린</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>햇 수미감자</t>
+          <t>2025년 홍 감자</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -5876,29 +5876,29 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-12 22:50</t>
+          <t>2026-05-13 22:56</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>더그린</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>대저 흑대추방울토마토</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5923,29 +5923,29 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-12 22:50</t>
+          <t>2026-05-13 22:56</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>더그린</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>부여 대추방울토마토</t>
+          <t>두백감자 ★7월 재오픈</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5970,19 +5970,19 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-12 22:52</t>
+          <t>2026-05-13 22:56</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>더그린</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5992,7 +5992,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>대저 토마토 / 짭짤이</t>
+          <t>대추 방울토마토</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -6017,14 +6017,14 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002113</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-12 22:53</t>
+          <t>2026-05-13 22:56</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -6034,12 +6034,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>2026년 햇 감자</t>
+          <t>흑대추 방울 토마토</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -6064,14 +6064,14 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-12 22:53</t>
+          <t>2026-05-13 22:56</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -6081,12 +6081,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>두백감자 ★7월 재오픈</t>
+          <t>고당도 성주 참외 ※선물세트 포함</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -6111,14 +6111,14 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-12 22:53</t>
+          <t>2026-05-13 22:57</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>2026년 수미감자</t>
+          <t>스테비아 감자 ★7월 재오픈</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -6158,14 +6158,14 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-12 22:54</t>
+          <t>2026-05-13 22:57</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -6175,12 +6175,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>2026년 강원도감자</t>
+          <t>스테비야 방울토마토</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -6205,14 +6205,14 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-12 22:54</t>
+          <t>2026-05-13 22:57</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -6222,12 +6222,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>2025년 홍 감자</t>
+          <t>스테비아 완숙 토마토</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -6251,335 +6251,6 @@
         </is>
       </c>
       <c r="I124" t="inlineStr">
-        <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>2026-05-12 22:54</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>더그린</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>감자</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>돼지감자</t>
-        </is>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H125" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>2026-05-12 22:54</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>더그린</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>토마토</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>대추 방울토마토</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H126" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>2026-05-12 22:54</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>더그린</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>토마토</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>흑대추 방울 토마토</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H127" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>2026-05-12 22:54</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>더그린</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>참외</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>고당도 성주 참외 ※선물세트 포함</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H128" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>2026-05-12 22:55</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>더그린</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>감자</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>스테비아 감자 ★7월 재오픈</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H129" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>2026-05-12 22:55</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>더그린</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>토마토</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>스테비야 방울토마토</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G130" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H130" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>2026-05-12 22:55</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>더그린</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>토마토</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>스테비아 완숙 토마토</t>
-        </is>
-      </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F131" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H131" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I131" t="inlineStr">
         <is>
           <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000582</t>
         </is>

</xml_diff>

<commit_message>
Auto Update Prices: Thu May 14 22:57:31 UTC 2026
</commit_message>
<xml_diff>
--- a/가격이력.xlsx
+++ b/가격이력.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I124"/>
+  <dimension ref="A1:I127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-13 22:17</t>
+          <t>2026-05-14 22:15</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -525,7 +525,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-13 22:17</t>
+          <t>2026-05-14 22:15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -572,7 +572,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-13 22:17</t>
+          <t>2026-05-14 22:15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-13 22:17</t>
+          <t>2026-05-14 22:15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-13 22:17</t>
+          <t>2026-05-14 22:15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -713,7 +713,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-13 22:18</t>
+          <t>2026-05-14 22:16</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -760,7 +760,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-13 22:18</t>
+          <t>2026-05-14 22:16</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-13 22:18</t>
+          <t>2026-05-14 22:16</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-13 22:18</t>
+          <t>2026-05-14 22:16</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-13 22:18</t>
+          <t>2026-05-14 22:16</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -948,7 +948,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-13 22:18</t>
+          <t>2026-05-14 22:16</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -995,7 +995,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-13 22:18</t>
+          <t>2026-05-14 22:16</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-13 22:19</t>
+          <t>2026-05-14 22:16</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1089,7 +1089,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-13 22:19</t>
+          <t>2026-05-14 22:17</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1136,7 +1136,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-13 22:19</t>
+          <t>2026-05-14 22:17</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-13 22:20</t>
+          <t>2026-05-14 22:18</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1230,7 +1230,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-13 22:20</t>
+          <t>2026-05-14 22:18</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-13 22:21</t>
+          <t>2026-05-14 22:19</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1324,7 +1324,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-13 22:22</t>
+          <t>2026-05-14 22:19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1371,7 +1371,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-13 22:22</t>
+          <t>2026-05-14 22:20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1418,7 +1418,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-13 22:22</t>
+          <t>2026-05-14 22:20</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-13 22:22</t>
+          <t>2026-05-14 22:20</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1512,7 +1512,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-13 22:22</t>
+          <t>2026-05-14 22:20</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1559,7 +1559,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-13 22:22</t>
+          <t>2026-05-14 22:20</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1606,7 +1606,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-13 22:22</t>
+          <t>2026-05-14 22:20</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1653,7 +1653,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-13 22:22</t>
+          <t>2026-05-14 22:20</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1700,7 +1700,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-13 22:22</t>
+          <t>2026-05-14 22:20</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1747,7 +1747,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-13 22:22</t>
+          <t>2026-05-14 22:20</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1794,7 +1794,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-13 22:23</t>
+          <t>2026-05-14 22:20</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1841,7 +1841,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-13 22:23</t>
+          <t>2026-05-14 22:20</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1888,7 +1888,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-13 22:23</t>
+          <t>2026-05-14 22:21</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1935,7 +1935,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-13 22:23</t>
+          <t>2026-05-14 22:21</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1982,7 +1982,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-13 22:23</t>
+          <t>2026-05-14 22:21</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2029,7 +2029,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-13 22:23</t>
+          <t>2026-05-14 22:21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2076,7 +2076,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-13 22:23</t>
+          <t>2026-05-14 22:21</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2123,7 +2123,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-13 22:23</t>
+          <t>2026-05-14 22:21</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2170,7 +2170,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-13 22:23</t>
+          <t>2026-05-14 22:21</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2217,7 +2217,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-13 22:23</t>
+          <t>2026-05-14 22:21</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2264,7 +2264,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-13 22:24</t>
+          <t>2026-05-14 22:21</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2311,7 +2311,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-13 22:24</t>
+          <t>2026-05-14 22:21</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2358,7 +2358,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-13 22:24</t>
+          <t>2026-05-14 22:22</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2405,7 +2405,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-13 22:24</t>
+          <t>2026-05-14 22:22</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2452,7 +2452,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-13 22:24</t>
+          <t>2026-05-14 22:22</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2499,7 +2499,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-13 22:24</t>
+          <t>2026-05-14 22:22</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-13 22:24</t>
+          <t>2026-05-14 22:22</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2593,7 +2593,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-13 22:24</t>
+          <t>2026-05-14 22:22</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2640,7 +2640,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-13 22:24</t>
+          <t>2026-05-14 22:22</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-13 22:24</t>
+          <t>2026-05-14 22:22</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2734,7 +2734,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-13 22:24</t>
+          <t>2026-05-14 22:22</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2781,7 +2781,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-13 22:25</t>
+          <t>2026-05-14 22:23</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2828,7 +2828,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-13 22:25</t>
+          <t>2026-05-14 22:23</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2875,7 +2875,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-13 22:25</t>
+          <t>2026-05-14 22:23</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2922,7 +2922,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-13 22:25</t>
+          <t>2026-05-14 22:23</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2969,7 +2969,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-13 22:27</t>
+          <t>2026-05-14 22:25</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3016,7 +3016,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-13 22:27</t>
+          <t>2026-05-14 22:25</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3063,7 +3063,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-13 22:27</t>
+          <t>2026-05-14 22:25</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3110,7 +3110,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-13 22:27</t>
+          <t>2026-05-14 22:25</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>[예약판매] 하우스 대극천복숭아</t>
+          <t>하우스 대극천복숭아</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3157,7 +3157,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-13 22:27</t>
+          <t>2026-05-14 22:25</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3204,7 +3204,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-13 22:28</t>
+          <t>2026-05-14 22:26</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3251,7 +3251,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-13 22:28</t>
+          <t>2026-05-14 22:26</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3298,7 +3298,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-05-13 22:28</t>
+          <t>2026-05-14 22:26</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3308,12 +3308,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>★특가★ 가정용 하우스수박</t>
+          <t>★특가★ 성주 꿀참외 (박스포함)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3338,14 +3338,14 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-13 22:28</t>
+          <t>2026-05-14 22:26</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3355,12 +3355,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2026 국내산 햇감자</t>
+          <t>★특가★ 성주 꿀참외</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3385,14 +3385,14 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-13 22:29</t>
+          <t>2026-05-14 22:26</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3402,12 +3402,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>2026 국내산 햇양파</t>
+          <t>★특가★ 가정용 하우스수박</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3432,14 +3432,14 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-13 22:29</t>
+          <t>2026-05-14 22:26</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3449,12 +3449,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외 (박스포함)</t>
+          <t>정품 하우스수박</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3479,14 +3479,14 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001536</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-05-13 22:29</t>
+          <t>2026-05-14 22:26</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3496,12 +3496,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외</t>
+          <t>고당도 흑수박</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3526,14 +3526,14 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000630</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-13 22:29</t>
+          <t>2026-05-14 22:27</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3543,12 +3543,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>★특가★ 짭짤이토마토</t>
+          <t>2026 국내산 햇감자</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3573,14 +3573,14 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001857</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-13 22:29</t>
+          <t>2026-05-14 22:27</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3590,12 +3590,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>★특가★ 대추방울토마토</t>
+          <t>2026 국내산 햇양파</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3620,14 +3620,14 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-13 22:29</t>
+          <t>2026-05-14 22:27</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>★특가★ 유럽종 완숙토마토</t>
+          <t>★특가★ 대추방울토마토</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3667,14 +3667,14 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-05-13 22:30</t>
+          <t>2026-05-14 22:28</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3689,7 +3689,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>스테비아 방울토마토</t>
+          <t>★특가★ 유럽종 완숙토마토</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3714,14 +3714,14 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-13 22:30</t>
+          <t>2026-05-14 22:28</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3736,7 +3736,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>흑대추방울토마토</t>
+          <t>스테비아 방울토마토</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3761,29 +3761,29 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001718</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-05-13 22:31</t>
+          <t>2026-05-14 22:28</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>★별담특가 가정용 참외★</t>
+          <t>흑대추방울토마토</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3808,14 +3808,14 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001718</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-13 22:32</t>
+          <t>2026-05-14 22:29</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3825,12 +3825,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>2026 햇양파</t>
+          <t>★별담특가 가정용 참외★</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3855,14 +3855,14 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-05-13 22:32</t>
+          <t>2026-05-14 22:29</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3872,12 +3872,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>2026 햇양파</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3902,14 +3902,14 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008676</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-13 22:32</t>
+          <t>2026-05-14 22:30</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3924,7 +3924,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3949,14 +3949,14 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008676</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-05-13 22:32</t>
+          <t>2026-05-14 22:30</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3966,12 +3966,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3996,14 +3996,14 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-13 22:33</t>
+          <t>2026-05-14 22:30</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4013,12 +4013,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4043,14 +4043,14 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-05-13 22:35</t>
+          <t>2026-05-14 22:31</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4060,12 +4060,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>대저 토마토</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4090,29 +4090,29 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008441</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-13 22:37</t>
+          <t>2026-05-14 22:33</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>★특가★ 가성비 참외</t>
+          <t>대저 토마토</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4137,14 +4137,14 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002133</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008441</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05-13 22:37</t>
+          <t>2026-05-14 22:34</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4154,12 +4154,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>햇 감자</t>
+          <t>★특가★ 가성비 참외</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -4184,14 +4184,14 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002108</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002133</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-13 22:37</t>
+          <t>2026-05-14 22:35</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4201,12 +4201,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>햇 양파</t>
+          <t>햇 감자</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4231,14 +4231,14 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000186</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002108</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-05-13 22:37</t>
+          <t>2026-05-14 22:35</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4248,12 +4248,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>햇 양파</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -4278,14 +4278,14 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000186</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-13 22:38</t>
+          <t>2026-05-14 22:35</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4295,12 +4295,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -4325,14 +4325,14 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-05-13 22:38</t>
+          <t>2026-05-14 22:35</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4342,12 +4342,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -4372,14 +4372,14 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-13 22:38</t>
+          <t>2026-05-14 22:36</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4389,12 +4389,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>대저토마토</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4419,29 +4419,29 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-05-13 22:41</t>
+          <t>2026-05-14 22:36</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>★당도보장★ 농협선별 스테비아 수박</t>
+          <t>대저토마토</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4466,14 +4466,14 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-13 22:41</t>
+          <t>2026-05-14 22:39</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4483,12 +4483,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>[N-81] 신비복숭아</t>
+          <t>🔥핫딜🔥 가정용 성주참외</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4513,14 +4513,14 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001165</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-05-13 22:41</t>
+          <t>2026-05-14 22:39</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4530,12 +4530,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>[N-81] 가정용 성주참외</t>
+          <t>★당도보장★ 농협선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4560,14 +4560,14 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001101</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-13 22:42</t>
+          <t>2026-05-14 22:39</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4577,12 +4577,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>[N-81] 가성비 성주참외</t>
+          <t>[N-81] 신비복숭아</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4607,14 +4607,14 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001013</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-05-13 22:42</t>
+          <t>2026-05-14 22:39</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4629,7 +4629,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
+          <t>[N-81] 가정용 성주참외</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4654,14 +4654,14 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001101</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-13 22:42</t>
+          <t>2026-05-14 22:40</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4671,12 +4671,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>가정용 하우스수박 (기박)</t>
+          <t>[N-81] 가성비 성주참외</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4701,29 +4701,29 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001013</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-05-13 22:44</t>
+          <t>2026-05-14 22:40</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
+          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -4748,19 +4748,19 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-13 22:45</t>
+          <t>2026-05-14 22:40</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4770,7 +4770,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
+          <t>가정용 하우스수박 (기박)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4795,14 +4795,14 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-05-13 22:45</t>
+          <t>2026-05-14 22:41</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4812,12 +4812,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>농협인증 당도선별 스테비아 수박</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4842,14 +4842,14 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006697</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-13 22:45</t>
+          <t>2026-05-14 22:42</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>국내산 무주 수박무말랭이</t>
+          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4889,14 +4889,14 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-05-13 22:45</t>
+          <t>2026-05-14 22:43</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>정품 수박</t>
+          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4936,14 +4936,14 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-13 22:45</t>
+          <t>2026-05-14 22:43</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4953,12 +4953,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>대추 방울 토마토 소과</t>
+          <t>농협인증 당도선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4983,14 +4983,14 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-05-13 22:46</t>
+          <t>2026-05-14 22:43</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -5005,7 +5005,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>가정용 흑수박 5kg 이상</t>
+          <t>국내산 무주 수박무말랭이</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -5030,14 +5030,14 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-13 22:47</t>
+          <t>2026-05-14 22:44</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -5047,12 +5047,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
+          <t>정품 수박</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -5077,29 +5077,29 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-05-13 22:50</t>
+          <t>2026-05-14 22:44</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>성주참외</t>
+          <t>대추 방울 토마토 소과</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -5124,29 +5124,29 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003357</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-13 22:50</t>
+          <t>2026-05-14 22:44</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>❤️성주참외</t>
+          <t>가정용 흑수박 5kg 이상</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5171,29 +5171,29 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-05-13 22:50</t>
+          <t>2026-05-14 22:45</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5218,14 +5218,14 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-05-13 22:50</t>
+          <t>2026-05-14 22:48</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -5235,12 +5235,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>❤️성주참외</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5265,14 +5265,14 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-05-13 22:50</t>
+          <t>2026-05-14 22:48</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -5282,12 +5282,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>성주참외</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -5312,14 +5312,14 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003357</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-05-13 22:51</t>
+          <t>2026-05-14 22:48</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -5329,12 +5329,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>[고품위] 하우스 털 복숭아</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5359,14 +5359,14 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-05-13 22:52</t>
+          <t>2026-05-14 22:48</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -5376,12 +5376,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>햇 홍감자</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -5406,14 +5406,14 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-05-13 22:52</t>
+          <t>2026-05-14 22:48</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -5423,12 +5423,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>햇 설봉감자</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -5453,14 +5453,14 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-05-13 22:52</t>
+          <t>2026-05-14 22:49</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -5470,12 +5470,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>특가 대추방울토마토</t>
+          <t>[고품위] 하우스 털 복숭아</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5500,14 +5500,14 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-13 22:52</t>
+          <t>2026-05-14 22:50</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>햇 수미감자</t>
+          <t>햇 홍감자</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5547,14 +5547,14 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-13 22:52</t>
+          <t>2026-05-14 22:50</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5564,12 +5564,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>대저 흑대추방울토마토</t>
+          <t>햇 설봉감자</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5594,14 +5594,14 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-13 22:53</t>
+          <t>2026-05-14 22:50</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5616,7 +5616,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>부여 대추방울토마토</t>
+          <t>특가 대추방울토마토</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5641,14 +5641,14 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-13 22:54</t>
+          <t>2026-05-14 22:50</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5658,12 +5658,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>대저 토마토 / 짭짤이</t>
+          <t>햇 수미감자</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5688,29 +5688,29 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002113</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-13 22:55</t>
+          <t>2026-05-14 22:50</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>2026년 강원도감자</t>
+          <t>대저 흑대추방울토마토</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5735,29 +5735,29 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-13 22:55</t>
+          <t>2026-05-14 22:50</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>2026년 수미감자</t>
+          <t>부여 대추방울토마토</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5782,29 +5782,29 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-13 22:55</t>
+          <t>2026-05-14 22:52</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2026년 햇 감자</t>
+          <t>대저 토마토 / 짭짤이</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5829,14 +5829,14 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002113</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-13 22:55</t>
+          <t>2026-05-14 22:53</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>2025년 홍 감자</t>
+          <t>2026년 강원도감자</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -5876,14 +5876,14 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-13 22:56</t>
+          <t>2026-05-14 22:53</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -5898,7 +5898,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>2026년 수미감자</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5923,14 +5923,14 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-13 22:56</t>
+          <t>2026-05-14 22:53</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -5945,7 +5945,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>두백감자 ★7월 재오픈</t>
+          <t>2026년 햇 감자</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5970,14 +5970,14 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-13 22:56</t>
+          <t>2026-05-14 22:53</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -5987,12 +5987,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>대추 방울토마토</t>
+          <t>2025년 홍 감자</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -6017,14 +6017,14 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-13 22:56</t>
+          <t>2026-05-14 22:53</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -6034,12 +6034,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>흑대추 방울 토마토</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -6064,14 +6064,14 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-13 22:56</t>
+          <t>2026-05-14 22:53</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -6081,12 +6081,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>고당도 성주 참외 ※선물세트 포함</t>
+          <t>두백감자 ★7월 재오픈</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -6111,14 +6111,14 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-13 22:57</t>
+          <t>2026-05-14 22:53</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -6128,12 +6128,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>스테비아 감자 ★7월 재오픈</t>
+          <t>대추 방울토마토</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -6158,14 +6158,14 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-13 22:57</t>
+          <t>2026-05-14 22:54</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -6180,7 +6180,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>스테비야 방울토마토</t>
+          <t>흑대추 방울 토마토</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -6205,14 +6205,14 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-13 22:57</t>
+          <t>2026-05-14 22:54</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -6222,35 +6222,176 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
+          <t>참외</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>고당도 성주 참외 ※선물세트 포함</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-05-14 22:54</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>감자</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>스테비아 감자 ★7월 재오픈</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-05-14 22:54</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
           <t>토마토</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr">
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>스테비야 방울토마토</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-05-14 22:54</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>토마토</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
         <is>
           <t>스테비아 완숙 토마토</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H124" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I124" t="inlineStr">
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
         <is>
           <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000582</t>
         </is>

</xml_diff>

<commit_message>
Auto Update Prices: Fri May 15 22:45:36 UTC 2026
</commit_message>
<xml_diff>
--- a/가격이력.xlsx
+++ b/가격이력.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I127"/>
+  <dimension ref="A1:I123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-14 22:15</t>
+          <t>2026-05-15 22:02</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -525,7 +525,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-14 22:15</t>
+          <t>2026-05-15 22:02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -572,7 +572,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-14 22:15</t>
+          <t>2026-05-15 22:03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-14 22:15</t>
+          <t>2026-05-15 22:03</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-14 22:15</t>
+          <t>2026-05-15 22:03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -713,7 +713,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-14 22:16</t>
+          <t>2026-05-15 22:03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -760,7 +760,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-14 22:16</t>
+          <t>2026-05-15 22:03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-14 22:16</t>
+          <t>2026-05-15 22:03</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-14 22:16</t>
+          <t>2026-05-15 22:04</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-14 22:16</t>
+          <t>2026-05-15 22:04</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -948,7 +948,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-14 22:16</t>
+          <t>2026-05-15 22:04</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -995,7 +995,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-14 22:16</t>
+          <t>2026-05-15 22:04</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-14 22:16</t>
+          <t>2026-05-15 22:04</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1089,7 +1089,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-14 22:17</t>
+          <t>2026-05-15 22:05</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1136,7 +1136,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-14 22:17</t>
+          <t>2026-05-15 22:05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-14 22:18</t>
+          <t>2026-05-15 22:05</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1230,7 +1230,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-14 22:18</t>
+          <t>2026-05-15 22:06</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-14 22:19</t>
+          <t>2026-05-15 22:06</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1324,7 +1324,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-14 22:19</t>
+          <t>2026-05-15 22:07</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1364,14 +1364,14 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011646</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-14 22:20</t>
+          <t>2026-05-15 22:07</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1411,14 +1411,14 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011645</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-14 22:20</t>
+          <t>2026-05-15 22:07</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1458,14 +1458,14 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011644</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-14 22:20</t>
+          <t>2026-05-15 22:07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 3kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1505,14 +1505,14 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011643</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-14 22:20</t>
+          <t>2026-05-15 22:08</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1552,14 +1552,14 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011642</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-14 22:20</t>
+          <t>2026-05-15 22:08</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1599,14 +1599,14 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011641</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-14 22:20</t>
+          <t>2026-05-15 22:08</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1646,14 +1646,14 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011640</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-14 22:20</t>
+          <t>2026-05-15 22:08</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 5kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1693,14 +1693,14 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011639</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-14 22:20</t>
+          <t>2026-05-15 22:08</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1740,14 +1740,14 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011638</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-14 22:20</t>
+          <t>2026-05-15 22:08</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1787,14 +1787,14 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011637</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-14 22:20</t>
+          <t>2026-05-15 22:08</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1834,14 +1834,14 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011636</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-14 22:20</t>
+          <t>2026-05-15 22:08</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>행사 (박스포함) 참외 가정용 / 10kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1881,14 +1881,14 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011635</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-14 22:21</t>
+          <t>2026-05-15 22:08</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1928,14 +1928,14 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-14 22:21</t>
+          <t>2026-05-15 22:08</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1975,14 +1975,14 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-14 22:21</t>
+          <t>2026-05-15 22:08</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2022,14 +2022,14 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-14 22:21</t>
+          <t>2026-05-15 22:09</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 혼합과</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2069,14 +2069,14 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011123</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-14 22:21</t>
+          <t>2026-05-15 22:09</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>흑대추방울토마토 5kg</t>
+          <t>(박스포함) 완숙토마토★4kg / 혼합과</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2116,14 +2116,14 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011224</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010320</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-14 22:21</t>
+          <t>2026-05-15 22:09</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>흑대추방울토마토 2kg</t>
+          <t>(박스포함) 완숙토마토★3kg / 혼합과</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2163,14 +2163,14 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011223</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010319</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-14 22:21</t>
+          <t>2026-05-15 22:09</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>흑대추방울토마토 1kg</t>
+          <t>(박스포함) 완숙토마토 4kg / 혼합과</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2210,14 +2210,14 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011222</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010318</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-14 22:21</t>
+          <t>2026-05-15 22:09</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2227,12 +2227,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
+          <t>(박스포함) 완숙토마토 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2257,14 +2257,14 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010317</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-14 22:21</t>
+          <t>2026-05-15 22:10</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2274,12 +2274,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
+          <t>(박스포함)★완숙토마토 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2304,14 +2304,14 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010107</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-14 22:21</t>
+          <t>2026-05-15 22:10</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2351,14 +2351,14 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011410</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-14 22:22</t>
+          <t>2026-05-15 22:10</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2398,14 +2398,14 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011409</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-14 22:22</t>
+          <t>2026-05-15 22:10</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2445,14 +2445,14 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011408</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-14 22:22</t>
+          <t>2026-05-15 22:10</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2492,14 +2492,14 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011407</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-14 22:22</t>
+          <t>2026-05-15 22:10</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2539,14 +2539,14 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011405</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-14 22:22</t>
+          <t>2026-05-15 22:10</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2586,14 +2586,14 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011404</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-14 22:22</t>
+          <t>2026-05-15 22:10</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2633,14 +2633,14 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011403</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-14 22:22</t>
+          <t>2026-05-15 22:11</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2680,14 +2680,14 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011402</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-14 22:22</t>
+          <t>2026-05-15 22:11</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 소과</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2727,14 +2727,14 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011401</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-14 22:22</t>
+          <t>2026-05-15 22:11</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 혼합과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 로얄과</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2774,14 +2774,14 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011123</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011400</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-14 22:23</t>
+          <t>2026-05-15 22:11</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2791,12 +2791,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토★4kg / 혼합과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 대과</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2821,14 +2821,14 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010320</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011399</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-14 22:23</t>
+          <t>2026-05-15 22:11</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2838,12 +2838,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토★3kg / 혼합과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 혼합과</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2868,29 +2868,29 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010319</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011398</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-14 22:23</t>
+          <t>2026-05-15 22:12</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토 4kg / 혼합과</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2915,29 +2915,29 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010318</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002048</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-14 22:23</t>
+          <t>2026-05-15 22:12</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토 3kg / 혼합과</t>
+          <t>하우스 천도복숭아</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2962,14 +2962,14 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010317</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002047</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-14 22:25</t>
+          <t>2026-05-15 22:12</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2979,12 +2979,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>정품 우곡수박</t>
+          <t>하우스 대극천복숭아</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3009,14 +3009,14 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002058</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001975</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-14 22:25</t>
+          <t>2026-05-15 22:13</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3026,12 +3026,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>★특가★ 하우스 대석자두</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3056,14 +3056,14 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002048</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002042</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-14 22:25</t>
+          <t>2026-05-15 22:13</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3073,12 +3073,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>하우스 천도복숭아</t>
+          <t>하우스 대석자두</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3103,14 +3103,14 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002047</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001958</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-14 22:25</t>
+          <t>2026-05-15 22:13</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>하우스 대극천복숭아</t>
+          <t>하우스 털복숭아</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3150,14 +3150,14 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001975</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001942</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-14 22:25</t>
+          <t>2026-05-15 22:13</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3167,12 +3167,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>★특가★ 하우스 대석자두</t>
+          <t>★특가★ 성주 꿀참외 (박스포함)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3197,14 +3197,14 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002042</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-14 22:26</t>
+          <t>2026-05-15 22:13</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3214,12 +3214,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>하우스 대석자두</t>
+          <t>★특가★ 성주 꿀참외</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3244,14 +3244,14 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001958</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-14 22:26</t>
+          <t>2026-05-15 22:13</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3261,12 +3261,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>하우스 털복숭아</t>
+          <t>정품 우곡수박</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3291,14 +3291,14 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001942</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002058</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-05-14 22:26</t>
+          <t>2026-05-15 22:14</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3308,12 +3308,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외 (박스포함)</t>
+          <t>★특가★ 가정용 하우스수박</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3338,14 +3338,14 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-14 22:26</t>
+          <t>2026-05-15 22:14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3355,12 +3355,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외</t>
+          <t>정품 하우스수박</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3385,14 +3385,14 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001536</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-14 22:26</t>
+          <t>2026-05-15 22:14</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3407,7 +3407,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>★특가★ 가정용 하우스수박</t>
+          <t>고당도 흑수박</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3432,14 +3432,14 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000630</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-14 22:26</t>
+          <t>2026-05-15 22:15</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3449,12 +3449,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>정품 하우스수박</t>
+          <t>2026 국내산 햇감자</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3479,14 +3479,14 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001536</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-05-14 22:26</t>
+          <t>2026-05-15 22:15</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3496,12 +3496,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>고당도 흑수박</t>
+          <t>2026 국내산 햇양파</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3526,14 +3526,14 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000630</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-14 22:27</t>
+          <t>2026-05-15 22:15</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3543,12 +3543,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2026 국내산 햇감자</t>
+          <t>★특가★ 대추방울토마토</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3573,14 +3573,14 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-14 22:27</t>
+          <t>2026-05-15 22:16</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3590,12 +3590,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2026 국내산 햇양파</t>
+          <t>★특가★ 유럽종 완숙토마토</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3620,14 +3620,14 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-14 22:27</t>
+          <t>2026-05-15 22:16</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>★특가★ 대추방울토마토</t>
+          <t>스테비아 방울토마토</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3667,14 +3667,14 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-05-14 22:28</t>
+          <t>2026-05-15 22:16</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3689,7 +3689,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>★특가★ 유럽종 완숙토마토</t>
+          <t>흑대추방울토마토</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3714,29 +3714,29 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001718</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-14 22:28</t>
+          <t>2026-05-15 22:17</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>스테비아 방울토마토</t>
+          <t>★별담특가 가정용 참외★</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3761,29 +3761,29 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-05-14 22:28</t>
+          <t>2026-05-15 22:17</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>흑대추방울토마토</t>
+          <t>2026 햇양파</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3808,14 +3808,14 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001718</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-14 22:29</t>
+          <t>2026-05-15 22:17</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3825,12 +3825,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>★별담특가 가정용 참외★</t>
+          <t>고당도 하우스 수박(12브릭스 이상)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3855,14 +3855,14 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008785</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-05-14 22:29</t>
+          <t>2026-05-15 22:17</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3872,12 +3872,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>2026 햇양파</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3902,14 +3902,14 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008787</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-14 22:30</t>
+          <t>2026-05-15 22:19</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3924,7 +3924,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3949,14 +3949,14 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008676</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-05-14 22:30</t>
+          <t>2026-05-15 22:19</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3966,12 +3966,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3996,14 +3996,14 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-14 22:30</t>
+          <t>2026-05-15 22:20</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4013,12 +4013,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4043,29 +4043,29 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-05-14 22:31</t>
+          <t>2026-05-15 22:22</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>★특가★ 가성비 참외</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4090,29 +4090,29 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002133</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-14 22:33</t>
+          <t>2026-05-15 22:23</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>대저 토마토</t>
+          <t>햇 감자</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4137,14 +4137,14 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008441</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002108</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05-14 22:34</t>
+          <t>2026-05-15 22:23</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4154,12 +4154,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>★특가★ 가성비 참외</t>
+          <t>햇 양파</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -4184,14 +4184,14 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002133</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000186</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-14 22:35</t>
+          <t>2026-05-15 22:23</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4201,12 +4201,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>햇 감자</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4231,14 +4231,14 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002108</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-05-14 22:35</t>
+          <t>2026-05-15 22:23</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4248,12 +4248,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>햇 양파</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -4278,14 +4278,14 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000186</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-14 22:35</t>
+          <t>2026-05-15 22:23</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4295,12 +4295,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -4325,14 +4325,14 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-05-14 22:35</t>
+          <t>2026-05-15 22:24</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4342,12 +4342,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>대저토마토</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -4372,29 +4372,29 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-14 22:36</t>
+          <t>2026-05-15 22:27</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>🔥핫딜🔥 가정용 성주참외</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4419,29 +4419,29 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001165</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-05-14 22:36</t>
+          <t>2026-05-15 22:27</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>대저토마토</t>
+          <t>★당도보장★ 농협선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4466,14 +4466,14 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-14 22:39</t>
+          <t>2026-05-15 22:27</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4483,12 +4483,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>🔥핫딜🔥 가정용 성주참외</t>
+          <t>[N-81] 신비복숭아</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4513,14 +4513,14 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001165</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-05-14 22:39</t>
+          <t>2026-05-15 22:28</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4530,12 +4530,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>★당도보장★ 농협선별 스테비아 수박</t>
+          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4560,14 +4560,14 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-14 22:39</t>
+          <t>2026-05-15 22:28</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4577,12 +4577,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>[N-81] 신비복숭아</t>
+          <t>가정용 하우스수박 (기박)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4607,29 +4607,29 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-05-14 22:39</t>
+          <t>2026-05-15 22:29</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>[N-81] 가정용 성주참외</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4654,29 +4654,29 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001101</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006697</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-14 22:40</t>
+          <t>2026-05-15 22:30</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>[N-81] 가성비 성주참외</t>
+          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4701,29 +4701,29 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001013</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-05-14 22:40</t>
+          <t>2026-05-15 22:31</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
+          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -4748,19 +4748,19 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-14 22:40</t>
+          <t>2026-05-15 22:31</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4770,7 +4770,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>가정용 하우스수박 (기박)</t>
+          <t>농협인증 당도선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4795,14 +4795,14 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-05-14 22:41</t>
+          <t>2026-05-15 22:31</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4812,12 +4812,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>국내산 무주 수박무말랭이</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4842,14 +4842,14 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006697</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-14 22:42</t>
+          <t>2026-05-15 22:31</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
+          <t>정품 수박</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4889,14 +4889,14 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-05-14 22:43</t>
+          <t>2026-05-15 22:32</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4906,12 +4906,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
+          <t>대추 방울 토마토 소과</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4936,14 +4936,14 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-14 22:43</t>
+          <t>2026-05-15 22:32</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>농협인증 당도선별 스테비아 수박</t>
+          <t>가정용 흑수박 5kg 이상</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4983,14 +4983,14 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-05-14 22:43</t>
+          <t>2026-05-15 22:33</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -5000,12 +5000,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>국내산 무주 수박무말랭이</t>
+          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -5030,19 +5030,19 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-14 22:44</t>
+          <t>2026-05-15 22:36</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>정품 수박</t>
+          <t>하우스 수박 / 8kg 내외</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -5077,29 +5077,29 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003366</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-05-14 22:44</t>
+          <t>2026-05-15 22:36</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>대추 방울 토마토 소과</t>
+          <t>❤️성주참외</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -5124,29 +5124,29 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-14 22:44</t>
+          <t>2026-05-15 22:36</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>가정용 흑수박 5kg 이상</t>
+          <t>성주참외</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5171,29 +5171,29 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003357</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-05-14 22:45</t>
+          <t>2026-05-15 22:36</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5218,14 +5218,14 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-05-14 22:48</t>
+          <t>2026-05-15 22:36</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -5235,12 +5235,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>❤️성주참외</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5265,14 +5265,14 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-05-14 22:48</t>
+          <t>2026-05-15 22:36</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -5282,12 +5282,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>성주참외</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -5312,14 +5312,14 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003357</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-05-14 22:48</t>
+          <t>2026-05-15 22:37</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -5329,12 +5329,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>[고품위] 하우스 털 복숭아</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5359,14 +5359,14 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-05-14 22:48</t>
+          <t>2026-05-15 22:38</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -5376,12 +5376,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>햇 홍감자</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -5406,14 +5406,14 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-05-14 22:48</t>
+          <t>2026-05-15 22:38</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -5423,12 +5423,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>햇 설봉감자</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -5453,14 +5453,14 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-05-14 22:49</t>
+          <t>2026-05-15 22:38</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -5470,12 +5470,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>[고품위] 하우스 털 복숭아</t>
+          <t>특가 대추방울토마토</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5500,14 +5500,14 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-14 22:50</t>
+          <t>2026-05-15 22:38</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>햇 홍감자</t>
+          <t>햇 수미감자</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5547,14 +5547,14 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-14 22:50</t>
+          <t>2026-05-15 22:38</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5564,12 +5564,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>햇 설봉감자</t>
+          <t>대저 흑대추방울토마토</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5594,14 +5594,14 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-14 22:50</t>
+          <t>2026-05-15 22:39</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5616,7 +5616,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>특가 대추방울토마토</t>
+          <t>부여 대추방울토마토</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5641,19 +5641,19 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-14 22:50</t>
+          <t>2026-05-15 22:41</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>더그린</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>햇 수미감자</t>
+          <t>2026년 강원도감자</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5688,29 +5688,29 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-14 22:50</t>
+          <t>2026-05-15 22:41</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>더그린</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>대저 흑대추방울토마토</t>
+          <t>2026년 수미감자</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5735,29 +5735,29 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-14 22:50</t>
+          <t>2026-05-15 22:41</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>더그린</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>부여 대추방울토마토</t>
+          <t>2026년 햇 감자</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5782,29 +5782,29 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-14 22:52</t>
+          <t>2026-05-15 22:41</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>더그린</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>대저 토마토 / 짭짤이</t>
+          <t>2025년 홍 감자</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5829,14 +5829,14 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002113</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-14 22:53</t>
+          <t>2026-05-15 22:41</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>2026년 강원도감자</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -5876,14 +5876,14 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-14 22:53</t>
+          <t>2026-05-15 22:41</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -5898,7 +5898,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>2026년 수미감자</t>
+          <t>두백감자 ★7월 재오픈</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5923,14 +5923,14 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-14 22:53</t>
+          <t>2026-05-15 22:42</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -5940,12 +5940,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>2026년 햇 감자</t>
+          <t>대추 방울토마토</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5970,14 +5970,14 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-14 22:53</t>
+          <t>2026-05-15 22:42</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -5987,12 +5987,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>2025년 홍 감자</t>
+          <t>흑대추 방울 토마토</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -6017,14 +6017,14 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-14 22:53</t>
+          <t>2026-05-15 22:42</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -6034,12 +6034,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>고당도 성주 참외 ※선물세트 포함</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -6064,14 +6064,14 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-14 22:53</t>
+          <t>2026-05-15 22:42</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>두백감자 ★7월 재오픈</t>
+          <t>스테비아 감자 ★7월 재오픈</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -6111,14 +6111,14 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-14 22:53</t>
+          <t>2026-05-15 22:42</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>대추 방울토마토</t>
+          <t>스테비야 방울토마토</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -6158,14 +6158,14 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-14 22:54</t>
+          <t>2026-05-15 22:42</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -6180,7 +6180,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>흑대추 방울 토마토</t>
+          <t>스테비아 완숙 토마토</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -6204,194 +6204,6 @@
         </is>
       </c>
       <c r="I123" t="inlineStr">
-        <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>2026-05-14 22:54</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>더그린</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>참외</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>고당도 성주 참외 ※선물세트 포함</t>
-        </is>
-      </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H124" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I124" t="inlineStr">
-        <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>2026-05-14 22:54</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>더그린</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>감자</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>스테비아 감자 ★7월 재오픈</t>
-        </is>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H125" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>2026-05-14 22:54</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>더그린</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>토마토</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>스테비야 방울토마토</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H126" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>2026-05-14 22:54</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>더그린</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>토마토</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>스테비아 완숙 토마토</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H127" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I127" t="inlineStr">
         <is>
           <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000582</t>
         </is>

</xml_diff>

<commit_message>
Auto Update Prices: Sat May 16 22:38:04 UTC 2026
</commit_message>
<xml_diff>
--- a/가격이력.xlsx
+++ b/가격이력.xlsx
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-15 22:02</t>
+          <t>2026-05-16 21:55</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -525,7 +525,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-15 22:02</t>
+          <t>2026-05-16 21:55</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -572,7 +572,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-15 22:03</t>
+          <t>2026-05-16 21:55</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-15 22:03</t>
+          <t>2026-05-16 21:55</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-15 22:03</t>
+          <t>2026-05-16 21:55</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -713,7 +713,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-15 22:03</t>
+          <t>2026-05-16 21:55</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -760,7 +760,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-15 22:03</t>
+          <t>2026-05-16 21:56</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-15 22:03</t>
+          <t>2026-05-16 21:56</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-15 22:04</t>
+          <t>2026-05-16 21:56</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-15 22:04</t>
+          <t>2026-05-16 21:56</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -948,7 +948,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-15 22:04</t>
+          <t>2026-05-16 21:56</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -995,7 +995,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-15 22:04</t>
+          <t>2026-05-16 21:56</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-15 22:04</t>
+          <t>2026-05-16 21:56</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1089,7 +1089,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-15 22:05</t>
+          <t>2026-05-16 21:57</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1136,7 +1136,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-15 22:05</t>
+          <t>2026-05-16 21:57</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-15 22:05</t>
+          <t>2026-05-16 21:58</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1230,7 +1230,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-15 22:06</t>
+          <t>2026-05-16 21:58</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-15 22:06</t>
+          <t>2026-05-16 21:58</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1324,7 +1324,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-15 22:07</t>
+          <t>2026-05-16 22:00</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1371,7 +1371,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-15 22:07</t>
+          <t>2026-05-16 22:00</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1418,7 +1418,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-15 22:07</t>
+          <t>2026-05-16 22:00</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-15 22:07</t>
+          <t>2026-05-16 22:00</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1512,7 +1512,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-15 22:08</t>
+          <t>2026-05-16 22:00</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1559,7 +1559,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-15 22:08</t>
+          <t>2026-05-16 22:00</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1606,7 +1606,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-15 22:08</t>
+          <t>2026-05-16 22:00</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1653,7 +1653,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-15 22:08</t>
+          <t>2026-05-16 22:00</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1700,7 +1700,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-15 22:08</t>
+          <t>2026-05-16 22:00</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1747,7 +1747,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-15 22:08</t>
+          <t>2026-05-16 22:00</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1794,7 +1794,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-15 22:08</t>
+          <t>2026-05-16 22:00</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1841,7 +1841,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-15 22:08</t>
+          <t>2026-05-16 22:01</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1888,7 +1888,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-15 22:08</t>
+          <t>2026-05-16 22:01</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1935,7 +1935,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-15 22:08</t>
+          <t>2026-05-16 22:01</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1982,7 +1982,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-15 22:08</t>
+          <t>2026-05-16 22:01</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2029,7 +2029,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-15 22:09</t>
+          <t>2026-05-16 22:01</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2076,7 +2076,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-15 22:09</t>
+          <t>2026-05-16 22:02</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2123,7 +2123,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-15 22:09</t>
+          <t>2026-05-16 22:02</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2170,7 +2170,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-15 22:09</t>
+          <t>2026-05-16 22:02</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2217,7 +2217,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-15 22:09</t>
+          <t>2026-05-16 22:02</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2264,7 +2264,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-15 22:10</t>
+          <t>2026-05-16 22:02</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2311,7 +2311,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-15 22:10</t>
+          <t>2026-05-16 22:02</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2358,7 +2358,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-15 22:10</t>
+          <t>2026-05-16 22:02</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2405,7 +2405,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-15 22:10</t>
+          <t>2026-05-16 22:02</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2452,7 +2452,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-15 22:10</t>
+          <t>2026-05-16 22:02</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2499,7 +2499,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-15 22:10</t>
+          <t>2026-05-16 22:03</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-15 22:10</t>
+          <t>2026-05-16 22:03</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2593,7 +2593,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-15 22:10</t>
+          <t>2026-05-16 22:03</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2640,7 +2640,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-15 22:11</t>
+          <t>2026-05-16 22:03</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-15 22:11</t>
+          <t>2026-05-16 22:03</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2734,7 +2734,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-15 22:11</t>
+          <t>2026-05-16 22:03</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2781,7 +2781,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-15 22:11</t>
+          <t>2026-05-16 22:03</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2828,7 +2828,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-15 22:11</t>
+          <t>2026-05-16 22:03</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2875,7 +2875,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-15 22:12</t>
+          <t>2026-05-16 22:05</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2922,7 +2922,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-15 22:12</t>
+          <t>2026-05-16 22:05</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2969,7 +2969,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-15 22:12</t>
+          <t>2026-05-16 22:05</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3016,7 +3016,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-15 22:13</t>
+          <t>2026-05-16 22:05</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3063,7 +3063,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-15 22:13</t>
+          <t>2026-05-16 22:05</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3110,7 +3110,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-15 22:13</t>
+          <t>2026-05-16 22:05</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3157,7 +3157,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-15 22:13</t>
+          <t>2026-05-16 22:05</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3204,7 +3204,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-15 22:13</t>
+          <t>2026-05-16 22:05</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3251,7 +3251,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-15 22:13</t>
+          <t>2026-05-16 22:06</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3298,7 +3298,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-05-15 22:14</t>
+          <t>2026-05-16 22:06</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3345,7 +3345,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-15 22:14</t>
+          <t>2026-05-16 22:06</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3392,7 +3392,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-15 22:14</t>
+          <t>2026-05-16 22:06</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3439,7 +3439,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-15 22:15</t>
+          <t>2026-05-16 22:08</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3486,7 +3486,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-05-15 22:15</t>
+          <t>2026-05-16 22:08</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3533,7 +3533,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-15 22:15</t>
+          <t>2026-05-16 22:08</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3580,7 +3580,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-15 22:16</t>
+          <t>2026-05-16 22:08</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3627,7 +3627,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-15 22:16</t>
+          <t>2026-05-16 22:08</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3674,7 +3674,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-05-15 22:16</t>
+          <t>2026-05-16 22:08</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3721,7 +3721,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-15 22:17</t>
+          <t>2026-05-16 22:09</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3768,7 +3768,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-05-15 22:17</t>
+          <t>2026-05-16 22:10</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3815,7 +3815,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-15 22:17</t>
+          <t>2026-05-16 22:10</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3862,7 +3862,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-05-15 22:17</t>
+          <t>2026-05-16 22:10</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3909,7 +3909,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-15 22:19</t>
+          <t>2026-05-16 22:11</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3956,7 +3956,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-05-15 22:19</t>
+          <t>2026-05-16 22:11</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4003,7 +4003,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-15 22:20</t>
+          <t>2026-05-16 22:12</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4050,7 +4050,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-05-15 22:22</t>
+          <t>2026-05-16 22:14</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-15 22:23</t>
+          <t>2026-05-16 22:15</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4144,7 +4144,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05-15 22:23</t>
+          <t>2026-05-16 22:15</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4191,7 +4191,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-15 22:23</t>
+          <t>2026-05-16 22:15</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4238,7 +4238,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-05-15 22:23</t>
+          <t>2026-05-16 22:16</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4285,7 +4285,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-15 22:23</t>
+          <t>2026-05-16 22:16</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4332,7 +4332,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-05-15 22:24</t>
+          <t>2026-05-16 22:16</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4379,7 +4379,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-15 22:27</t>
+          <t>2026-05-16 22:19</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4426,7 +4426,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-05-15 22:27</t>
+          <t>2026-05-16 22:19</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4473,7 +4473,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-15 22:27</t>
+          <t>2026-05-16 22:19</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4520,7 +4520,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-05-15 22:28</t>
+          <t>2026-05-16 22:20</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4567,7 +4567,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-15 22:28</t>
+          <t>2026-05-16 22:20</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4614,7 +4614,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-05-15 22:29</t>
+          <t>2026-05-16 22:22</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4661,7 +4661,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-15 22:30</t>
+          <t>2026-05-16 22:23</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4708,7 +4708,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-05-15 22:31</t>
+          <t>2026-05-16 22:23</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4755,7 +4755,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-15 22:31</t>
+          <t>2026-05-16 22:24</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4802,7 +4802,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-05-15 22:31</t>
+          <t>2026-05-16 22:24</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4849,7 +4849,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-15 22:31</t>
+          <t>2026-05-16 22:24</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4896,7 +4896,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-05-15 22:32</t>
+          <t>2026-05-16 22:24</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4943,7 +4943,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-15 22:32</t>
+          <t>2026-05-16 22:24</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4990,7 +4990,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-05-15 22:33</t>
+          <t>2026-05-16 22:25</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -5037,7 +5037,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-15 22:36</t>
+          <t>2026-05-16 22:28</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -5084,7 +5084,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-05-15 22:36</t>
+          <t>2026-05-16 22:28</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5131,7 +5131,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-15 22:36</t>
+          <t>2026-05-16 22:28</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -5178,7 +5178,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-05-15 22:36</t>
+          <t>2026-05-16 22:29</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -5225,7 +5225,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-05-15 22:36</t>
+          <t>2026-05-16 22:29</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -5272,7 +5272,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-05-15 22:36</t>
+          <t>2026-05-16 22:29</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -5319,7 +5319,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-05-15 22:37</t>
+          <t>2026-05-16 22:29</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -5366,7 +5366,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-05-15 22:38</t>
+          <t>2026-05-16 22:30</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -5413,7 +5413,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-05-15 22:38</t>
+          <t>2026-05-16 22:30</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -5460,7 +5460,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-05-15 22:38</t>
+          <t>2026-05-16 22:30</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-15 22:38</t>
+          <t>2026-05-16 22:30</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5554,7 +5554,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-15 22:38</t>
+          <t>2026-05-16 22:31</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5601,7 +5601,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-15 22:39</t>
+          <t>2026-05-16 22:31</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5648,7 +5648,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-15 22:41</t>
+          <t>2026-05-16 22:33</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5695,7 +5695,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-15 22:41</t>
+          <t>2026-05-16 22:34</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5742,7 +5742,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-15 22:41</t>
+          <t>2026-05-16 22:34</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -5789,7 +5789,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-15 22:41</t>
+          <t>2026-05-16 22:34</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -5836,7 +5836,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-15 22:41</t>
+          <t>2026-05-16 22:34</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -5883,7 +5883,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-15 22:41</t>
+          <t>2026-05-16 22:34</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -5930,7 +5930,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-15 22:42</t>
+          <t>2026-05-16 22:34</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -5977,7 +5977,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-15 22:42</t>
+          <t>2026-05-16 22:34</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -6024,7 +6024,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-15 22:42</t>
+          <t>2026-05-16 22:34</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -6071,7 +6071,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-15 22:42</t>
+          <t>2026-05-16 22:35</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -6118,7 +6118,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-15 22:42</t>
+          <t>2026-05-16 22:35</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -6165,7 +6165,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-15 22:42</t>
+          <t>2026-05-16 22:35</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">

</xml_diff>

<commit_message>
Auto Update Prices: Sun May 17 22:42:05 UTC 2026
</commit_message>
<xml_diff>
--- a/가격이력.xlsx
+++ b/가격이력.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I123"/>
+  <dimension ref="A1:I122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-16 21:55</t>
+          <t>2026-05-17 21:59</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -525,7 +525,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-16 21:55</t>
+          <t>2026-05-17 21:59</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -572,7 +572,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-16 21:55</t>
+          <t>2026-05-17 21:59</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-16 21:55</t>
+          <t>2026-05-17 22:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-16 21:55</t>
+          <t>2026-05-17 22:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -713,7 +713,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-16 21:55</t>
+          <t>2026-05-17 22:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -760,7 +760,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-16 21:56</t>
+          <t>2026-05-17 22:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-16 21:56</t>
+          <t>2026-05-17 22:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-16 21:56</t>
+          <t>2026-05-17 22:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-16 21:56</t>
+          <t>2026-05-17 22:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -948,7 +948,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-16 21:56</t>
+          <t>2026-05-17 22:01</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -995,7 +995,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-16 21:56</t>
+          <t>2026-05-17 22:01</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-16 21:56</t>
+          <t>2026-05-17 22:01</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1089,7 +1089,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-16 21:57</t>
+          <t>2026-05-17 22:01</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1136,7 +1136,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-16 21:57</t>
+          <t>2026-05-17 22:02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-16 21:58</t>
+          <t>2026-05-17 22:02</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1230,7 +1230,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-16 21:58</t>
+          <t>2026-05-17 22:02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1277,22 +1277,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-16 21:58</t>
+          <t>2026-05-17 22:04</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>팡이농장</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>특★가 양파</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1317,14 +1317,14 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009488</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-16 22:00</t>
+          <t>2026-05-17 22:04</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1364,14 +1364,14 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-16 22:00</t>
+          <t>2026-05-17 22:04</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1411,14 +1411,14 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-16 22:00</t>
+          <t>2026-05-17 22:04</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1458,14 +1458,14 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-16 22:00</t>
+          <t>2026-05-17 22:04</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1505,14 +1505,14 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-16 22:00</t>
+          <t>2026-05-17 22:04</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1552,14 +1552,14 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-16 22:00</t>
+          <t>2026-05-17 22:04</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1599,14 +1599,14 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-16 22:00</t>
+          <t>2026-05-17 22:04</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1646,14 +1646,14 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-16 22:00</t>
+          <t>2026-05-17 22:04</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1693,14 +1693,14 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-16 22:00</t>
+          <t>2026-05-17 22:05</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1740,14 +1740,14 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-16 22:00</t>
+          <t>2026-05-17 22:05</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1787,14 +1787,14 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-16 22:00</t>
+          <t>2026-05-17 22:05</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1834,14 +1834,14 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-16 22:01</t>
+          <t>2026-05-17 22:05</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1881,14 +1881,14 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-16 22:01</t>
+          <t>2026-05-17 22:05</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1928,14 +1928,14 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-16 22:01</t>
+          <t>2026-05-17 22:05</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1975,14 +1975,14 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-16 22:01</t>
+          <t>2026-05-17 22:05</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 혼합과</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2022,14 +2022,14 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011123</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-16 22:01</t>
+          <t>2026-05-17 22:06</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2039,12 +2039,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 혼합과</t>
+          <t>(박스포함) 완숙토마토★4kg / 혼합과</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2069,14 +2069,14 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011123</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010320</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-16 22:02</t>
+          <t>2026-05-17 22:06</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토★4kg / 혼합과</t>
+          <t>(박스포함) 완숙토마토★3kg / 혼합과</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2116,14 +2116,14 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010320</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010319</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-16 22:02</t>
+          <t>2026-05-17 22:06</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토★3kg / 혼합과</t>
+          <t>(박스포함) 완숙토마토 4kg / 혼합과</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2163,14 +2163,14 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010319</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010318</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-16 22:02</t>
+          <t>2026-05-17 22:06</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토 4kg / 혼합과</t>
+          <t>(박스포함) 완숙토마토 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2210,14 +2210,14 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010318</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010317</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-16 22:02</t>
+          <t>2026-05-17 22:06</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2232,7 +2232,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토 3kg / 혼합과</t>
+          <t>(박스포함)★완숙토마토 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2257,14 +2257,14 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010317</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010107</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-16 22:02</t>
+          <t>2026-05-17 22:06</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2274,12 +2274,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>(박스포함)★완숙토마토 5kg / 혼합과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2304,14 +2304,14 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010107</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011410</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-16 22:02</t>
+          <t>2026-05-17 22:07</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 소과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2351,14 +2351,14 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011410</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011409</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-16 22:02</t>
+          <t>2026-05-17 22:07</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 로얄과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2398,14 +2398,14 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011409</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011408</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-16 22:02</t>
+          <t>2026-05-17 22:07</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 대과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2445,14 +2445,14 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011408</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011407</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-16 22:02</t>
+          <t>2026-05-17 22:07</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 혼합과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2492,14 +2492,14 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011407</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011405</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-16 22:03</t>
+          <t>2026-05-17 22:07</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 소과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2539,14 +2539,14 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011405</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011404</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-16 22:03</t>
+          <t>2026-05-17 22:07</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 로얄과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2586,14 +2586,14 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011404</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011403</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-16 22:03</t>
+          <t>2026-05-17 22:07</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 대과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2633,14 +2633,14 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011403</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011402</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-16 22:03</t>
+          <t>2026-05-17 22:07</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 혼합과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 소과</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2680,14 +2680,14 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011402</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011401</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-16 22:03</t>
+          <t>2026-05-17 22:07</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 소과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 로얄과</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2727,14 +2727,14 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011401</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011400</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-16 22:03</t>
+          <t>2026-05-17 22:07</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 로얄과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 대과</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2774,14 +2774,14 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011400</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011399</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-16 22:03</t>
+          <t>2026-05-17 22:07</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 대과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 혼합과</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2821,29 +2821,29 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011399</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011398</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-16 22:03</t>
+          <t>2026-05-17 22:09</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 혼합과</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2868,14 +2868,14 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011398</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002048</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-16 22:05</t>
+          <t>2026-05-17 22:09</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>하우스 천도복숭아</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2915,14 +2915,14 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002048</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002047</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-16 22:05</t>
+          <t>2026-05-17 22:09</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>하우스 천도복숭아</t>
+          <t>하우스 대극천복숭아</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2962,14 +2962,14 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002047</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001975</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-16 22:05</t>
+          <t>2026-05-17 22:09</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2979,12 +2979,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>하우스 대극천복숭아</t>
+          <t>★특가★ 하우스 대석자두</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3009,14 +3009,14 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001975</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002042</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-16 22:05</t>
+          <t>2026-05-17 22:09</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>★특가★ 하우스 대석자두</t>
+          <t>하우스 대석자두</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3056,14 +3056,14 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002042</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001958</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-16 22:05</t>
+          <t>2026-05-17 22:09</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3073,12 +3073,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>하우스 대석자두</t>
+          <t>하우스 털복숭아</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3103,14 +3103,14 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001958</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001942</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-16 22:05</t>
+          <t>2026-05-17 22:09</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3120,12 +3120,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>하우스 털복숭아</t>
+          <t>★특가★ 성주 꿀참외 (박스포함)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3150,14 +3150,14 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001942</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-16 22:05</t>
+          <t>2026-05-17 22:10</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3172,7 +3172,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외 (박스포함)</t>
+          <t>★특가★ 성주 꿀참외</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3197,14 +3197,14 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-16 22:05</t>
+          <t>2026-05-17 22:10</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3214,12 +3214,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외</t>
+          <t>정품 우곡수박</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3244,14 +3244,14 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002058</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-16 22:06</t>
+          <t>2026-05-17 22:10</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3266,7 +3266,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>정품 우곡수박</t>
+          <t>★특가★ 가정용 하우스수박</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3291,14 +3291,14 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002058</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-05-16 22:06</t>
+          <t>2026-05-17 22:10</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>★특가★ 가정용 하우스수박</t>
+          <t>정품 하우스수박</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3338,14 +3338,14 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001536</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-16 22:06</t>
+          <t>2026-05-17 22:10</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>정품 하우스수박</t>
+          <t>고당도 흑수박</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3385,14 +3385,14 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001536</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000630</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-16 22:06</t>
+          <t>2026-05-17 22:12</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3402,12 +3402,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>고당도 흑수박</t>
+          <t>2026 국내산 햇감자</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3432,14 +3432,14 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000630</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-16 22:08</t>
+          <t>2026-05-17 22:12</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3449,12 +3449,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2026 국내산 햇감자</t>
+          <t>2026 국내산 햇양파</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3479,14 +3479,14 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-05-16 22:08</t>
+          <t>2026-05-17 22:12</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3496,12 +3496,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>2026 국내산 햇양파</t>
+          <t>★특가★ 대추방울토마토</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3526,14 +3526,14 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-16 22:08</t>
+          <t>2026-05-17 22:12</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3548,7 +3548,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>★특가★ 대추방울토마토</t>
+          <t>★특가★ 유럽종 완숙토마토</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3573,14 +3573,14 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-16 22:08</t>
+          <t>2026-05-17 22:12</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3595,7 +3595,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>★특가★ 유럽종 완숙토마토</t>
+          <t>스테비아 방울토마토</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3620,14 +3620,14 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-16 22:08</t>
+          <t>2026-05-17 22:12</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>스테비아 방울토마토</t>
+          <t>흑대추방울토마토</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3667,29 +3667,29 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001718</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-05-16 22:08</t>
+          <t>2026-05-17 22:14</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>흑대추방울토마토</t>
+          <t>★별담특가 가정용 참외★</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3714,14 +3714,14 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001718</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-16 22:09</t>
+          <t>2026-05-17 22:14</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3731,12 +3731,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>★별담특가 가정용 참외★</t>
+          <t>2026 햇양파</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3761,14 +3761,14 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-05-16 22:10</t>
+          <t>2026-05-17 22:14</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3778,12 +3778,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>2026 햇양파</t>
+          <t>고당도 하우스 수박(12브릭스 이상)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3808,14 +3808,14 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008785</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-16 22:10</t>
+          <t>2026-05-17 22:14</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3825,12 +3825,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>고당도 하우스 수박(12브릭스 이상)</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3855,14 +3855,14 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008785</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008787</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-05-16 22:10</t>
+          <t>2026-05-17 22:15</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3872,12 +3872,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3902,14 +3902,14 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008787</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-16 22:11</t>
+          <t>2026-05-17 22:15</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3919,12 +3919,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3949,14 +3949,14 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-05-16 22:11</t>
+          <t>2026-05-17 22:16</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3966,12 +3966,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3996,29 +3996,29 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-16 22:12</t>
+          <t>2026-05-17 22:18</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>★특가★ 가성비 참외</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4043,14 +4043,14 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002133</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-05-16 22:14</t>
+          <t>2026-05-17 22:19</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4060,12 +4060,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>★특가★ 가성비 참외</t>
+          <t>햇 감자</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4090,14 +4090,14 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002133</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002108</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-16 22:15</t>
+          <t>2026-05-17 22:19</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4107,12 +4107,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>햇 감자</t>
+          <t>햇 양파</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4137,14 +4137,14 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002108</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000186</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05-16 22:15</t>
+          <t>2026-05-17 22:19</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4154,12 +4154,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>햇 양파</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -4184,14 +4184,14 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000186</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-16 22:15</t>
+          <t>2026-05-17 22:20</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4201,12 +4201,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4231,14 +4231,14 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-05-16 22:16</t>
+          <t>2026-05-17 22:20</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4248,12 +4248,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -4278,14 +4278,14 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-16 22:16</t>
+          <t>2026-05-17 22:20</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4295,12 +4295,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>대저토마토</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -4325,29 +4325,29 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-05-16 22:16</t>
+          <t>2026-05-17 22:23</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>대저토마토</t>
+          <t>🔥핫딜🔥 가정용 성주참외</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -4372,14 +4372,14 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001165</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-16 22:19</t>
+          <t>2026-05-17 22:23</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4389,12 +4389,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>🔥핫딜🔥 가정용 성주참외</t>
+          <t>★당도보장★ 농협선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4419,14 +4419,14 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001165</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-05-16 22:19</t>
+          <t>2026-05-17 22:23</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4436,12 +4436,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>★당도보장★ 농협선별 스테비아 수박</t>
+          <t>[N-81] 신비복숭아</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4466,14 +4466,14 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-16 22:19</t>
+          <t>2026-05-17 22:24</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4483,12 +4483,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>[N-81] 신비복숭아</t>
+          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4513,14 +4513,14 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-05-16 22:20</t>
+          <t>2026-05-17 22:24</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4530,12 +4530,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
+          <t>가정용 하우스수박 (기박)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4560,29 +4560,29 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-16 22:20</t>
+          <t>2026-05-17 22:26</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>가정용 하우스수박 (기박)</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4607,14 +4607,14 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006697</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-05-16 22:22</t>
+          <t>2026-05-17 22:27</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4624,12 +4624,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4654,14 +4654,14 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006697</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-16 22:23</t>
+          <t>2026-05-17 22:27</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4676,7 +4676,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
+          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4701,14 +4701,14 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-05-16 22:23</t>
+          <t>2026-05-17 22:28</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
+          <t>농협인증 당도선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -4748,14 +4748,14 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-16 22:24</t>
+          <t>2026-05-17 22:28</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4770,7 +4770,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>농협인증 당도선별 스테비아 수박</t>
+          <t>국내산 무주 수박무말랭이</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4795,14 +4795,14 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-05-16 22:24</t>
+          <t>2026-05-17 22:28</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>국내산 무주 수박무말랭이</t>
+          <t>정품 수박</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4842,14 +4842,14 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-16 22:24</t>
+          <t>2026-05-17 22:28</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4859,12 +4859,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>정품 수박</t>
+          <t>대추 방울 토마토 소과</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4889,14 +4889,14 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-05-16 22:24</t>
+          <t>2026-05-17 22:28</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4906,12 +4906,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>대추 방울 토마토 소과</t>
+          <t>가정용 흑수박 5kg 이상</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4936,14 +4936,14 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-16 22:24</t>
+          <t>2026-05-17 22:29</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4953,12 +4953,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>가정용 흑수박 5kg 이상</t>
+          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4983,29 +4983,29 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-05-16 22:25</t>
+          <t>2026-05-17 22:32</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
+          <t>하우스 수박 / 8kg 내외</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -5030,14 +5030,14 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003366</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-16 22:28</t>
+          <t>2026-05-17 22:32</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -5047,12 +5047,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>하우스 수박 / 8kg 내외</t>
+          <t>❤️성주참외</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -5077,14 +5077,14 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003366</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-05-16 22:28</t>
+          <t>2026-05-17 22:32</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>❤️성주참외</t>
+          <t>성주참외</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -5124,14 +5124,14 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003357</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-16 22:28</t>
+          <t>2026-05-17 22:32</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -5141,12 +5141,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>성주참외</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5171,14 +5171,14 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003357</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-05-16 22:29</t>
+          <t>2026-05-17 22:33</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -5188,12 +5188,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5218,14 +5218,14 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-05-16 22:29</t>
+          <t>2026-05-17 22:33</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -5235,12 +5235,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5265,14 +5265,14 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-05-16 22:29</t>
+          <t>2026-05-17 22:33</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -5287,7 +5287,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>[고품위] 하우스 털 복숭아</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -5312,14 +5312,14 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-05-16 22:29</t>
+          <t>2026-05-17 22:34</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -5329,12 +5329,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>[고품위] 하우스 털 복숭아</t>
+          <t>햇 홍감자</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5359,14 +5359,14 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-05-16 22:30</t>
+          <t>2026-05-17 22:34</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -5381,7 +5381,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>햇 홍감자</t>
+          <t>햇 설봉감자</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -5406,14 +5406,14 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-05-16 22:30</t>
+          <t>2026-05-17 22:34</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -5423,12 +5423,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>햇 설봉감자</t>
+          <t>특가 대추방울토마토</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -5453,14 +5453,14 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-05-16 22:30</t>
+          <t>2026-05-17 22:34</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -5470,12 +5470,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>특가 대추방울토마토</t>
+          <t>햇 수미감자</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5500,14 +5500,14 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-16 22:30</t>
+          <t>2026-05-17 22:35</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5517,12 +5517,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>햇 수미감자</t>
+          <t>대저 흑대추방울토마토</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5547,14 +5547,14 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-16 22:31</t>
+          <t>2026-05-17 22:35</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>대저 흑대추방울토마토</t>
+          <t>부여 대추방울토마토</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5594,29 +5594,29 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-16 22:31</t>
+          <t>2026-05-17 22:37</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>더그린</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>부여 대추방울토마토</t>
+          <t>2026년 강원도감자</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5641,14 +5641,14 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-16 22:33</t>
+          <t>2026-05-17 22:37</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>2026년 강원도감자</t>
+          <t>2026년 수미감자</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5688,14 +5688,14 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-16 22:34</t>
+          <t>2026-05-17 22:38</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5710,7 +5710,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>2026년 수미감자</t>
+          <t>2026년 햇 감자</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5735,14 +5735,14 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-16 22:34</t>
+          <t>2026-05-17 22:38</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -5757,7 +5757,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>2026년 햇 감자</t>
+          <t>2025년 홍 감자</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5782,14 +5782,14 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-16 22:34</t>
+          <t>2026-05-17 22:38</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2025년 홍 감자</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5829,14 +5829,14 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-16 22:34</t>
+          <t>2026-05-17 22:38</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>두백감자 ★7월 재오픈</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -5876,14 +5876,14 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-16 22:34</t>
+          <t>2026-05-17 22:38</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -5893,12 +5893,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>두백감자 ★7월 재오픈</t>
+          <t>대추 방울토마토</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5923,14 +5923,14 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-16 22:34</t>
+          <t>2026-05-17 22:38</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -5945,7 +5945,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>대추 방울토마토</t>
+          <t>흑대추 방울 토마토</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5970,14 +5970,14 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-16 22:34</t>
+          <t>2026-05-17 22:38</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -5987,12 +5987,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>흑대추 방울 토마토</t>
+          <t>고당도 성주 참외 ※선물세트 포함</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -6017,14 +6017,14 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-16 22:34</t>
+          <t>2026-05-17 22:39</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -6034,12 +6034,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>고당도 성주 참외 ※선물세트 포함</t>
+          <t>스테비아 감자 ★7월 재오픈</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -6064,14 +6064,14 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-16 22:35</t>
+          <t>2026-05-17 22:39</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -6081,12 +6081,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>스테비아 감자 ★7월 재오픈</t>
+          <t>스테비야 방울토마토</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -6111,14 +6111,14 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-16 22:35</t>
+          <t>2026-05-17 22:39</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>스테비야 방울토마토</t>
+          <t>스테비아 완숙 토마토</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -6157,53 +6157,6 @@
         </is>
       </c>
       <c r="I122" t="inlineStr">
-        <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>2026-05-16 22:35</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>더그린</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>토마토</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>스테비아 완숙 토마토</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H123" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I123" t="inlineStr">
         <is>
           <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000582</t>
         </is>

</xml_diff>

<commit_message>
Auto Update Prices: Mon May 18 22:49:44 UTC 2026
</commit_message>
<xml_diff>
--- a/가격이력.xlsx
+++ b/가격이력.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I122"/>
+  <dimension ref="A1:I127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-17 21:59</t>
+          <t>2026-05-18 22:06</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -488,12 +488,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>하우스 흑미수박</t>
+          <t>그린황도 복숭아</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -518,14 +518,14 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010144</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010213</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-17 21:59</t>
+          <t>2026-05-18 22:07</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -535,12 +535,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>스테비아방울토마토</t>
+          <t>하우스 흑미수박</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -565,14 +565,14 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010143</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010144</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-17 21:59</t>
+          <t>2026-05-18 22:07</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -582,12 +582,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>우곡수박</t>
+          <t>스테비아방울토마토</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -612,14 +612,14 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010136</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010143</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-17 22:00</t>
+          <t>2026-05-18 22:07</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -629,12 +629,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>천도복숭아</t>
+          <t>우곡수박</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -659,14 +659,14 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010109</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010136</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-17 22:00</t>
+          <t>2026-05-18 22:07</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>신비복숭아</t>
+          <t>천도복숭아</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -706,14 +706,14 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010108</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010109</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-17 22:00</t>
+          <t>2026-05-18 22:07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>SVIP ★ 하우스 대극천복숭아 ★</t>
+          <t>신비복숭아</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -753,14 +753,14 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010048</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010108</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-17 22:00</t>
+          <t>2026-05-18 22:08</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -770,12 +770,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SVIP ★ 하우스 대석자두 ★</t>
+          <t>SVIP ★ 하우스 대극천복숭아 ★</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -800,14 +800,14 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010045</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010048</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-17 22:00</t>
+          <t>2026-05-18 22:08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>SVIP ★ 하우스 복숭아 ★</t>
+          <t>SVIP ★ 하우스 대석자두 ★</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -847,14 +847,14 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010044</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010045</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-17 22:00</t>
+          <t>2026-05-18 22:08</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>[VIP] 하우스복숭아</t>
+          <t>SVIP ★ 하우스 복숭아 ★</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -894,14 +894,14 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010007</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010044</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-17 22:00</t>
+          <t>2026-05-18 22:08</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -911,12 +911,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>[VIP] 하우스자두</t>
+          <t>[VIP] 하우스복숭아</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -941,14 +941,14 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010006</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010007</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-17 22:01</t>
+          <t>2026-05-18 22:08</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -958,12 +958,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>수박 (가정용/정품)</t>
+          <t>[VIP] 하우스자두</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -988,14 +988,14 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009976</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010006</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-17 22:01</t>
+          <t>2026-05-18 22:08</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1005,12 +1005,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>수박 (가정용/정품)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1035,14 +1035,14 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009960</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009976</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-17 22:01</t>
+          <t>2026-05-18 22:08</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>하우스 신선복숭아</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1082,14 +1082,14 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009959</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009960</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-17 22:01</t>
+          <t>2026-05-18 22:09</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1099,12 +1099,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>햇양파</t>
+          <t>하우스 신선복숭아</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1129,14 +1129,14 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009925</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009959</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-17 22:02</t>
+          <t>2026-05-18 22:09</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1146,12 +1146,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>햇양파</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1176,14 +1176,14 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009854</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009925</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-17 22:02</t>
+          <t>2026-05-18 22:10</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>완숙 찰 토마토</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1223,14 +1223,14 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009762</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009854</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-17 22:02</t>
+          <t>2026-05-18 22:10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>짭짤이 토마토</t>
+          <t>완숙 찰 토마토</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1270,29 +1270,29 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009744</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009762</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-17 22:04</t>
+          <t>2026-05-18 22:10</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>팡이농장</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
+          <t>짭짤이 토마토</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1317,14 +1317,14 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009744</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-17 22:04</t>
+          <t>2026-05-18 22:11</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1364,14 +1364,14 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-17 22:04</t>
+          <t>2026-05-18 22:12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1411,14 +1411,14 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-17 22:04</t>
+          <t>2026-05-18 22:12</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1458,14 +1458,14 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-17 22:04</t>
+          <t>2026-05-18 22:12</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1505,14 +1505,14 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-17 22:04</t>
+          <t>2026-05-18 22:12</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1552,14 +1552,14 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-17 22:04</t>
+          <t>2026-05-18 22:12</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1599,14 +1599,14 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-17 22:04</t>
+          <t>2026-05-18 22:12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1646,14 +1646,14 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-17 22:04</t>
+          <t>2026-05-18 22:12</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1693,14 +1693,14 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-17 22:05</t>
+          <t>2026-05-18 22:12</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1740,14 +1740,14 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-17 22:05</t>
+          <t>2026-05-18 22:12</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1787,14 +1787,14 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-17 22:05</t>
+          <t>2026-05-18 22:12</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1834,14 +1834,14 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-17 22:05</t>
+          <t>2026-05-18 22:12</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1881,14 +1881,14 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-17 22:05</t>
+          <t>2026-05-18 22:13</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1928,14 +1928,14 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-17 22:05</t>
+          <t>2026-05-18 22:13</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1975,14 +1975,14 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-17 22:05</t>
+          <t>2026-05-18 22:13</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2022,14 +2022,14 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011123</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-17 22:06</t>
+          <t>2026-05-18 22:13</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2039,12 +2039,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토★4kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 혼합과</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2069,14 +2069,14 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010320</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011123</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-17 22:06</t>
+          <t>2026-05-18 22:13</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토★3kg / 혼합과</t>
+          <t>(박스포함) 완숙토마토★4kg / 혼합과</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2116,14 +2116,14 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010319</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010320</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-17 22:06</t>
+          <t>2026-05-18 22:14</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토 4kg / 혼합과</t>
+          <t>(박스포함) 완숙토마토★3kg / 혼합과</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2163,14 +2163,14 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010318</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010319</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-17 22:06</t>
+          <t>2026-05-18 22:14</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토 3kg / 혼합과</t>
+          <t>(박스포함) 완숙토마토 4kg / 혼합과</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2210,14 +2210,14 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010317</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010318</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-17 22:06</t>
+          <t>2026-05-18 22:14</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2232,7 +2232,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>(박스포함)★완숙토마토 5kg / 혼합과</t>
+          <t>(박스포함) 완숙토마토 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2257,14 +2257,14 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010107</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010317</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-17 22:06</t>
+          <t>2026-05-18 22:14</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2274,12 +2274,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 소과</t>
+          <t>(박스포함)★완숙토마토 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2304,14 +2304,14 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011410</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010107</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-17 22:07</t>
+          <t>2026-05-18 22:14</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 로얄과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2351,14 +2351,14 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011409</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011410</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-17 22:07</t>
+          <t>2026-05-18 22:14</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 대과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2398,14 +2398,14 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011408</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011409</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-17 22:07</t>
+          <t>2026-05-18 22:14</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 혼합과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2445,14 +2445,14 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011407</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011408</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-17 22:07</t>
+          <t>2026-05-18 22:14</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 소과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2492,14 +2492,14 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011405</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011407</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-17 22:07</t>
+          <t>2026-05-18 22:14</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 로얄과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2539,14 +2539,14 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011404</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011405</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-17 22:07</t>
+          <t>2026-05-18 22:15</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 대과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2586,14 +2586,14 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011403</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011404</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-17 22:07</t>
+          <t>2026-05-18 22:15</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 혼합과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2633,14 +2633,14 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011402</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011403</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-17 22:07</t>
+          <t>2026-05-18 22:15</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 소과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2680,14 +2680,14 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011401</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011402</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-17 22:07</t>
+          <t>2026-05-18 22:15</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 로얄과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 소과</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2727,14 +2727,14 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011400</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011401</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-17 22:07</t>
+          <t>2026-05-18 22:15</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 대과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 로얄과</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2774,14 +2774,14 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011399</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011400</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-17 22:07</t>
+          <t>2026-05-18 22:15</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 혼합과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 대과</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2821,29 +2821,29 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011398</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011399</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-17 22:09</t>
+          <t>2026-05-18 22:15</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 혼합과</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2868,14 +2868,14 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002048</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011398</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-17 22:09</t>
+          <t>2026-05-18 22:16</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2885,12 +2885,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>하우스 천도복숭아</t>
+          <t>햇 홍감자</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2915,14 +2915,14 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002047</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000596</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-17 22:09</t>
+          <t>2026-05-18 22:17</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>하우스 대극천복숭아</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2962,14 +2962,14 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001975</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002048</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-17 22:09</t>
+          <t>2026-05-18 22:17</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2979,12 +2979,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>★특가★ 하우스 대석자두</t>
+          <t>하우스 천도복숭아</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3009,14 +3009,14 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002042</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002047</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-17 22:09</t>
+          <t>2026-05-18 22:17</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3026,12 +3026,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>하우스 대석자두</t>
+          <t>하우스 대극천복숭아</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3056,14 +3056,14 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001958</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001975</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-17 22:09</t>
+          <t>2026-05-18 22:17</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3073,12 +3073,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>하우스 털복숭아</t>
+          <t>★특가★ 하우스 대석자두</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3103,14 +3103,14 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001942</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002042</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-17 22:09</t>
+          <t>2026-05-18 22:17</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3120,12 +3120,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외 (박스포함)</t>
+          <t>하우스 대석자두</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3150,14 +3150,14 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001958</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-17 22:10</t>
+          <t>2026-05-18 22:17</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3167,12 +3167,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외</t>
+          <t>하우스 털복숭아</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3197,14 +3197,14 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001942</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-17 22:10</t>
+          <t>2026-05-18 22:17</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3214,12 +3214,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>정품 우곡수박</t>
+          <t>★특가★ 성주 꿀참외 (박스포함)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3244,14 +3244,14 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002058</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-17 22:10</t>
+          <t>2026-05-18 22:17</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3261,12 +3261,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>★특가★ 가정용 하우스수박</t>
+          <t>★특가★ 성주 꿀참외</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3291,14 +3291,14 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-05-17 22:10</t>
+          <t>2026-05-18 22:18</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>정품 하우스수박</t>
+          <t>정품 우곡수박</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3338,14 +3338,14 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001536</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002058</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-17 22:10</t>
+          <t>2026-05-18 22:18</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>고당도 흑수박</t>
+          <t>★특가★ 가정용 하우스수박</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3385,14 +3385,14 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000630</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-17 22:12</t>
+          <t>2026-05-18 22:18</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3402,12 +3402,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>2026 국내산 햇감자</t>
+          <t>정품 하우스수박</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3432,14 +3432,14 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001536</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-17 22:12</t>
+          <t>2026-05-18 22:18</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3449,12 +3449,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2026 국내산 햇양파</t>
+          <t>고당도 흑수박</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3479,14 +3479,14 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000630</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-05-17 22:12</t>
+          <t>2026-05-18 22:20</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3496,12 +3496,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>★특가★ 대추방울토마토</t>
+          <t>2026 국내산 햇감자</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3526,14 +3526,14 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-17 22:12</t>
+          <t>2026-05-18 22:20</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3543,12 +3543,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>★특가★ 유럽종 완숙토마토</t>
+          <t>2026 국내산 햇양파</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3573,14 +3573,14 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-17 22:12</t>
+          <t>2026-05-18 22:20</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3595,7 +3595,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>스테비아 방울토마토</t>
+          <t>★특가★ 대추방울토마토</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3620,14 +3620,14 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-17 22:12</t>
+          <t>2026-05-18 22:20</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>흑대추방울토마토</t>
+          <t>★특가★ 유럽종 완숙토마토</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3667,29 +3667,29 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001718</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-05-17 22:14</t>
+          <t>2026-05-18 22:20</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>★별담특가 가정용 참외★</t>
+          <t>스테비아 방울토마토</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3714,29 +3714,29 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-17 22:14</t>
+          <t>2026-05-18 22:20</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>2026 햇양파</t>
+          <t>흑대추방울토마토</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3761,14 +3761,14 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001718</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-05-17 22:14</t>
+          <t>2026-05-18 22:21</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3778,12 +3778,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>고당도 하우스 수박(12브릭스 이상)</t>
+          <t>★별담특가 가정용 참외★</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3808,14 +3808,14 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008785</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-17 22:14</t>
+          <t>2026-05-18 22:21</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3825,12 +3825,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>2026 햇양파</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3855,14 +3855,14 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008787</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-05-17 22:15</t>
+          <t>2026-05-18 22:22</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3872,12 +3872,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>고당도 하우스 수박(12브릭스 이상)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3902,14 +3902,14 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008785</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-17 22:15</t>
+          <t>2026-05-18 22:22</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3919,12 +3919,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3949,14 +3949,14 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008787</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-05-17 22:16</t>
+          <t>2026-05-18 22:23</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3966,12 +3966,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3996,29 +3996,29 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-17 22:18</t>
+          <t>2026-05-18 22:23</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>★특가★ 가성비 참외</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4043,29 +4043,29 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002133</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-05-17 22:19</t>
+          <t>2026-05-18 22:24</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>햇 감자</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4090,14 +4090,14 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002108</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-17 22:19</t>
+          <t>2026-05-18 22:26</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4107,12 +4107,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>햇 양파</t>
+          <t>★특가★ 가성비 참외</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4137,14 +4137,14 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000186</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002133</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05-17 22:19</t>
+          <t>2026-05-18 22:27</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4154,12 +4154,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>햇 감자</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -4184,14 +4184,14 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002108</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-17 22:20</t>
+          <t>2026-05-18 22:27</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4201,12 +4201,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>햇 양파</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4231,14 +4231,14 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000186</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-05-17 22:20</t>
+          <t>2026-05-18 22:27</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4248,12 +4248,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -4278,14 +4278,14 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-17 22:20</t>
+          <t>2026-05-18 22:27</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4295,12 +4295,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>대저토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -4325,29 +4325,29 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-05-17 22:23</t>
+          <t>2026-05-18 22:28</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>🔥핫딜🔥 가정용 성주참외</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -4372,29 +4372,29 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001165</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-17 22:23</t>
+          <t>2026-05-18 22:28</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>★당도보장★ 농협선별 스테비아 수박</t>
+          <t>대저토마토</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4419,14 +4419,14 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-05-17 22:23</t>
+          <t>2026-05-18 22:31</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4436,12 +4436,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>[N-81] 신비복숭아</t>
+          <t>🔥핫딜🔥 가정용 성주참외</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4466,14 +4466,14 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001165</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-17 22:24</t>
+          <t>2026-05-18 22:31</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4483,12 +4483,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
+          <t>★당도보장★ 농협선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4513,14 +4513,14 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-05-17 22:24</t>
+          <t>2026-05-18 22:31</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4530,12 +4530,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>가정용 하우스수박 (기박)</t>
+          <t>[N-81] 신비복숭아</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4560,29 +4560,29 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-17 22:26</t>
+          <t>2026-05-18 22:32</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4607,19 +4607,19 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006697</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-05-17 22:27</t>
+          <t>2026-05-18 22:32</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -4629,7 +4629,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
+          <t>가정용 하우스수박 (기박)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4654,14 +4654,14 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-17 22:27</t>
+          <t>2026-05-18 22:34</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4671,12 +4671,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4701,14 +4701,14 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006697</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-05-17 22:28</t>
+          <t>2026-05-18 22:35</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>농협인증 당도선별 스테비아 수박</t>
+          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -4748,14 +4748,14 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-17 22:28</t>
+          <t>2026-05-18 22:35</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4770,7 +4770,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>국내산 무주 수박무말랭이</t>
+          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4795,14 +4795,14 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-05-17 22:28</t>
+          <t>2026-05-18 22:36</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>정품 수박</t>
+          <t>농협인증 당도선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4842,14 +4842,14 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-17 22:28</t>
+          <t>2026-05-18 22:36</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4859,12 +4859,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>대추 방울 토마토 소과</t>
+          <t>국내산 무주 수박무말랭이</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4889,14 +4889,14 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-05-17 22:28</t>
+          <t>2026-05-18 22:36</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>가정용 흑수박 5kg 이상</t>
+          <t>정품 수박</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4936,14 +4936,14 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-17 22:29</t>
+          <t>2026-05-18 22:36</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4953,12 +4953,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
+          <t>대추 방울 토마토 소과</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4983,19 +4983,19 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-05-17 22:32</t>
+          <t>2026-05-18 22:36</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -5005,7 +5005,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>하우스 수박 / 8kg 내외</t>
+          <t>가정용 흑수박 5kg 이상</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -5030,19 +5030,19 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003366</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-17 22:32</t>
+          <t>2026-05-18 22:37</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>❤️성주참외</t>
+          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -5077,14 +5077,14 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-05-17 22:32</t>
+          <t>2026-05-18 22:40</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>성주참외</t>
+          <t>❤️성주참외</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -5124,14 +5124,14 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003357</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-17 22:32</t>
+          <t>2026-05-18 22:40</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -5141,12 +5141,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>성주참외</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5171,14 +5171,14 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003357</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-05-17 22:33</t>
+          <t>2026-05-18 22:40</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -5188,12 +5188,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5218,14 +5218,14 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-05-17 22:33</t>
+          <t>2026-05-18 22:40</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -5272,7 +5272,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-05-17 22:33</t>
+          <t>2026-05-18 22:40</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -5287,7 +5287,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>[고품위] 하우스 털 복숭아</t>
+          <t>하우스 천도복숭아</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -5312,14 +5312,14 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003423</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-05-17 22:34</t>
+          <t>2026-05-18 22:41</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -5329,12 +5329,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>햇 홍감자</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5359,14 +5359,14 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003424</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-05-17 22:34</t>
+          <t>2026-05-18 22:41</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -5376,12 +5376,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>햇 설봉감자</t>
+          <t>하우스 신선복숭아</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -5406,14 +5406,14 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003425</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-05-17 22:34</t>
+          <t>2026-05-18 22:41</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -5423,12 +5423,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>특가 대추방울토마토</t>
+          <t>[고품위] 하우스 털 복숭아</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -5453,14 +5453,14 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-05-17 22:34</t>
+          <t>2026-05-18 22:41</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -5470,12 +5470,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>햇 수미감자</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5500,14 +5500,14 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-17 22:35</t>
+          <t>2026-05-18 22:42</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5517,12 +5517,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>대저 흑대추방울토마토</t>
+          <t>남해 햇 홍감자</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5547,14 +5547,14 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-17 22:35</t>
+          <t>2026-05-18 22:42</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5564,12 +5564,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>부여 대추방울토마토</t>
+          <t>햇 설봉감자</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5594,29 +5594,29 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-17 22:37</t>
+          <t>2026-05-18 22:42</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>2026년 강원도감자</t>
+          <t>특가 대추방울토마토</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5641,19 +5641,19 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-17 22:37</t>
+          <t>2026-05-18 22:43</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>2026년 수미감자</t>
+          <t>햇 수미감자</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5688,29 +5688,29 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-17 22:38</t>
+          <t>2026-05-18 22:43</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>2026년 햇 감자</t>
+          <t>대저 흑대추방울토마토</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5735,29 +5735,29 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-17 22:38</t>
+          <t>2026-05-18 22:43</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>2025년 홍 감자</t>
+          <t>부여 대추방울토마토</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5782,14 +5782,14 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-17 22:38</t>
+          <t>2026-05-18 22:45</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>2026년 강원도감자</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5829,14 +5829,14 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-17 22:38</t>
+          <t>2026-05-18 22:45</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>두백감자 ★7월 재오픈</t>
+          <t>2026년 수미감자</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -5876,14 +5876,14 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-17 22:38</t>
+          <t>2026-05-18 22:45</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -5893,12 +5893,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>대추 방울토마토</t>
+          <t>2026년 햇 감자</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5923,14 +5923,14 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-17 22:38</t>
+          <t>2026-05-18 22:45</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -5940,12 +5940,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>흑대추 방울 토마토</t>
+          <t>26년 햇 홍감자</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5970,14 +5970,14 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001262</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-17 22:38</t>
+          <t>2026-05-18 22:46</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -5987,12 +5987,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>고당도 성주 참외 ※선물세트 포함</t>
+          <t>2025년 홍 감자</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -6017,14 +6017,14 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-17 22:39</t>
+          <t>2026-05-18 22:46</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -6039,7 +6039,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>스테비아 감자 ★7월 재오픈</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -6064,14 +6064,14 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-17 22:39</t>
+          <t>2026-05-18 22:46</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -6081,12 +6081,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>스테비야 방울토마토</t>
+          <t>두백감자 ★7월 재오픈</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -6111,14 +6111,14 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-17 22:39</t>
+          <t>2026-05-18 22:46</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -6133,30 +6133,265 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
+          <t>대추 방울토마토</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-05-18 22:46</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>토마토</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>흑대추 방울 토마토</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-05-18 22:46</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>참외</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>고당도 성주 참외 ※선물세트 포함</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-05-18 22:47</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>감자</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>스테비아 감자 ★7월 재오픈</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-05-18 22:47</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>토마토</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>스테비야 방울토마토</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-05-18 22:47</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>토마토</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
           <t>스테비아 완숙 토마토</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H122" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I122" t="inlineStr">
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
         <is>
           <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000582</t>
         </is>

</xml_diff>

<commit_message>
Auto Update Prices: Tue May 19 23:03:14 UTC 2026
</commit_message>
<xml_diff>
--- a/가격이력.xlsx
+++ b/가격이력.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I127"/>
+  <dimension ref="A1:I126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 22:06</t>
+          <t>2026-05-19 22:20</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -525,7 +525,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-18 22:07</t>
+          <t>2026-05-19 22:20</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -572,7 +572,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-18 22:07</t>
+          <t>2026-05-19 22:20</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-18 22:07</t>
+          <t>2026-05-19 22:20</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-18 22:07</t>
+          <t>2026-05-19 22:21</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -713,7 +713,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-18 22:07</t>
+          <t>2026-05-19 22:21</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -760,7 +760,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-18 22:08</t>
+          <t>2026-05-19 22:21</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-18 22:08</t>
+          <t>2026-05-19 22:21</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-18 22:08</t>
+          <t>2026-05-19 22:21</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-18 22:08</t>
+          <t>2026-05-19 22:21</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -948,7 +948,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-18 22:08</t>
+          <t>2026-05-19 22:21</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -995,7 +995,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-18 22:08</t>
+          <t>2026-05-19 22:22</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-18 22:08</t>
+          <t>2026-05-19 22:22</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1089,7 +1089,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-18 22:09</t>
+          <t>2026-05-19 22:22</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1136,7 +1136,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-18 22:09</t>
+          <t>2026-05-19 22:22</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-18 22:10</t>
+          <t>2026-05-19 22:23</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1230,7 +1230,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-18 22:10</t>
+          <t>2026-05-19 22:23</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1277,22 +1277,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-18 22:10</t>
+          <t>2026-05-19 22:25</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>팡이농장</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>짭짤이 토마토</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1317,14 +1317,14 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009744</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-18 22:11</t>
+          <t>2026-05-19 22:25</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1364,14 +1364,14 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-18 22:12</t>
+          <t>2026-05-19 22:25</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1411,14 +1411,14 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-18 22:12</t>
+          <t>2026-05-19 22:25</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1458,14 +1458,14 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-18 22:12</t>
+          <t>2026-05-19 22:25</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1505,14 +1505,14 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-18 22:12</t>
+          <t>2026-05-19 22:25</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1552,14 +1552,14 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-18 22:12</t>
+          <t>2026-05-19 22:25</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1599,14 +1599,14 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-18 22:12</t>
+          <t>2026-05-19 22:25</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1646,14 +1646,14 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-18 22:12</t>
+          <t>2026-05-19 22:25</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1693,14 +1693,14 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-18 22:12</t>
+          <t>2026-05-19 22:25</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1740,14 +1740,14 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-18 22:12</t>
+          <t>2026-05-19 22:25</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1787,14 +1787,14 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-18 22:12</t>
+          <t>2026-05-19 22:26</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1834,14 +1834,14 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-18 22:12</t>
+          <t>2026-05-19 22:26</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1881,14 +1881,14 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-18 22:13</t>
+          <t>2026-05-19 22:26</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1928,14 +1928,14 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-18 22:13</t>
+          <t>2026-05-19 22:26</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1975,14 +1975,14 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-18 22:13</t>
+          <t>2026-05-19 22:26</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 혼합과</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2022,14 +2022,14 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011123</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-18 22:13</t>
+          <t>2026-05-19 22:27</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2039,12 +2039,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 혼합과</t>
+          <t>(박스포함) 완숙토마토★4kg / 혼합과</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2069,14 +2069,14 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011123</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010320</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-18 22:13</t>
+          <t>2026-05-19 22:27</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토★4kg / 혼합과</t>
+          <t>(박스포함) 완숙토마토★3kg / 혼합과</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2116,14 +2116,14 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010320</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010319</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-18 22:14</t>
+          <t>2026-05-19 22:27</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토★3kg / 혼합과</t>
+          <t>(박스포함) 완숙토마토 4kg / 혼합과</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2163,14 +2163,14 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010319</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010318</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-18 22:14</t>
+          <t>2026-05-19 22:27</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토 4kg / 혼합과</t>
+          <t>(박스포함) 완숙토마토 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2210,14 +2210,14 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010318</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010317</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-18 22:14</t>
+          <t>2026-05-19 22:27</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2232,7 +2232,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토 3kg / 혼합과</t>
+          <t>(박스포함)★완숙토마토 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2257,14 +2257,14 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010317</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010107</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-18 22:14</t>
+          <t>2026-05-19 22:27</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2274,12 +2274,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>(박스포함)★완숙토마토 5kg / 혼합과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2304,14 +2304,14 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010107</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011410</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-18 22:14</t>
+          <t>2026-05-19 22:27</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 소과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2351,14 +2351,14 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011410</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011409</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-18 22:14</t>
+          <t>2026-05-19 22:27</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 로얄과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2398,14 +2398,14 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011409</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011408</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-18 22:14</t>
+          <t>2026-05-19 22:28</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 대과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2445,14 +2445,14 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011408</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011407</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-18 22:14</t>
+          <t>2026-05-19 22:28</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 혼합과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2492,14 +2492,14 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011407</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011405</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-18 22:14</t>
+          <t>2026-05-19 22:28</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 소과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2539,14 +2539,14 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011405</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011404</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-18 22:15</t>
+          <t>2026-05-19 22:28</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 로얄과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2586,14 +2586,14 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011404</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011403</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-18 22:15</t>
+          <t>2026-05-19 22:28</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 대과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2633,14 +2633,14 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011403</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011402</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-18 22:15</t>
+          <t>2026-05-19 22:28</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 혼합과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 소과</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2680,14 +2680,14 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011402</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011401</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-18 22:15</t>
+          <t>2026-05-19 22:28</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 소과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 로얄과</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2727,14 +2727,14 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011401</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011400</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-18 22:15</t>
+          <t>2026-05-19 22:28</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 로얄과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 대과</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2774,14 +2774,14 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011400</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011399</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-18 22:15</t>
+          <t>2026-05-19 22:28</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 대과</t>
+          <t>(박스포함) 참외 ★ 가정용 / 2kg / 혼합과</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2821,14 +2821,14 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011399</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011398</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-18 22:15</t>
+          <t>2026-05-19 22:28</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2838,12 +2838,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 혼합과</t>
+          <t>💪💪산지 최전선 '최고집' 하우스 자두💪💪</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2868,14 +2868,14 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011398</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011313</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-18 22:16</t>
+          <t>2026-05-19 22:30</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2922,7 +2922,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-18 22:17</t>
+          <t>2026-05-19 22:30</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2969,7 +2969,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-18 22:17</t>
+          <t>2026-05-19 22:30</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3016,7 +3016,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-18 22:17</t>
+          <t>2026-05-19 22:30</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3063,7 +3063,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-18 22:17</t>
+          <t>2026-05-19 22:30</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3110,7 +3110,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-18 22:17</t>
+          <t>2026-05-19 22:31</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3157,7 +3157,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-18 22:17</t>
+          <t>2026-05-19 22:31</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3204,7 +3204,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-18 22:17</t>
+          <t>2026-05-19 22:31</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3251,7 +3251,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-18 22:17</t>
+          <t>2026-05-19 22:31</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3298,7 +3298,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-05-18 22:18</t>
+          <t>2026-05-19 22:31</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3345,7 +3345,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-18 22:18</t>
+          <t>2026-05-19 22:32</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3392,7 +3392,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-18 22:18</t>
+          <t>2026-05-19 22:32</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3439,7 +3439,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-18 22:18</t>
+          <t>2026-05-19 22:32</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3486,7 +3486,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-05-18 22:20</t>
+          <t>2026-05-19 22:33</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3533,7 +3533,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-18 22:20</t>
+          <t>2026-05-19 22:33</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3580,7 +3580,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-18 22:20</t>
+          <t>2026-05-19 22:33</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3627,7 +3627,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-18 22:20</t>
+          <t>2026-05-19 22:33</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3674,7 +3674,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-05-18 22:20</t>
+          <t>2026-05-19 22:33</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3721,22 +3721,22 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-18 22:20</t>
+          <t>2026-05-19 22:34</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>흑대추방울토마토</t>
+          <t>★별담특가 가정용 참외★</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3761,14 +3761,14 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001718</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-05-18 22:21</t>
+          <t>2026-05-19 22:35</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3778,12 +3778,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>★별담특가 가정용 참외★</t>
+          <t>2026 햇양파</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3808,14 +3808,14 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-18 22:21</t>
+          <t>2026-05-19 22:35</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3825,12 +3825,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>2026 햇양파</t>
+          <t>고당도 하우스 수박(12브릭스 이상)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3855,14 +3855,14 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008785</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-05-18 22:22</t>
+          <t>2026-05-19 22:35</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3872,12 +3872,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>고당도 하우스 수박(12브릭스 이상)</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3902,14 +3902,14 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008785</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008787</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-18 22:22</t>
+          <t>2026-05-19 22:36</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3919,12 +3919,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3949,14 +3949,14 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008787</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-05-18 22:23</t>
+          <t>2026-05-19 22:36</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3966,12 +3966,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3996,14 +3996,14 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-18 22:23</t>
+          <t>2026-05-19 22:37</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4013,12 +4013,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4043,29 +4043,29 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-05-18 22:24</t>
+          <t>2026-05-19 22:39</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>★특가★ 가성비 참외</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4090,14 +4090,14 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002133</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-18 22:26</t>
+          <t>2026-05-19 22:40</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4107,12 +4107,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>★특가★ 가성비 참외</t>
+          <t>햇 감자</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4137,14 +4137,14 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002133</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002108</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05-18 22:27</t>
+          <t>2026-05-19 22:40</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4154,12 +4154,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>햇 감자</t>
+          <t>햇 양파</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -4184,14 +4184,14 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002108</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000186</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-18 22:27</t>
+          <t>2026-05-19 22:40</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4201,12 +4201,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>햇 양파</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4231,14 +4231,14 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000186</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-05-18 22:27</t>
+          <t>2026-05-19 22:41</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4248,12 +4248,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -4278,14 +4278,14 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-18 22:27</t>
+          <t>2026-05-19 22:41</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4295,12 +4295,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -4325,14 +4325,14 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-05-18 22:28</t>
+          <t>2026-05-19 22:41</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4342,12 +4342,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>대저토마토</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -4372,29 +4372,29 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-18 22:28</t>
+          <t>2026-05-19 22:44</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>대저토마토</t>
+          <t>🔥핫딜🔥 가정용 성주참외</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4419,14 +4419,14 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001165</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-05-18 22:31</t>
+          <t>2026-05-19 22:44</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4436,12 +4436,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>🔥핫딜🔥 가정용 성주참외</t>
+          <t>★당도보장★ 농협선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4466,14 +4466,14 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001165</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-18 22:31</t>
+          <t>2026-05-19 22:44</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4483,12 +4483,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>★당도보장★ 농협선별 스테비아 수박</t>
+          <t>[N-81] 신비복숭아</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4513,14 +4513,14 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-05-18 22:31</t>
+          <t>2026-05-19 22:45</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4530,12 +4530,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>[N-81] 신비복숭아</t>
+          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4560,14 +4560,14 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-18 22:32</t>
+          <t>2026-05-19 22:45</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4577,12 +4577,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
+          <t>가정용 하우스수박 (기박)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4607,29 +4607,29 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-05-18 22:32</t>
+          <t>2026-05-19 22:47</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>가정용 하우스수박 (기박)</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4654,14 +4654,14 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006697</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-18 22:34</t>
+          <t>2026-05-19 22:48</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4671,12 +4671,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4701,14 +4701,14 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006697</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-05-18 22:35</t>
+          <t>2026-05-19 22:48</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
+          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -4748,14 +4748,14 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-18 22:35</t>
+          <t>2026-05-19 22:49</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4770,7 +4770,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
+          <t>농협인증 당도선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4795,14 +4795,14 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-05-18 22:36</t>
+          <t>2026-05-19 22:49</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>농협인증 당도선별 스테비아 수박</t>
+          <t>국내산 무주 수박무말랭이</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4842,14 +4842,14 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-18 22:36</t>
+          <t>2026-05-19 22:49</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>국내산 무주 수박무말랭이</t>
+          <t>정품 수박</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4889,14 +4889,14 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-05-18 22:36</t>
+          <t>2026-05-19 22:49</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4906,12 +4906,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>정품 수박</t>
+          <t>대추 방울 토마토 소과</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4936,14 +4936,14 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-18 22:36</t>
+          <t>2026-05-19 22:49</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4953,12 +4953,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>대추 방울 토마토 소과</t>
+          <t>가정용 흑수박 5kg 이상</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4983,14 +4983,14 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-05-18 22:36</t>
+          <t>2026-05-19 22:50</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -5000,12 +5000,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>가정용 흑수박 5kg 이상</t>
+          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -5030,19 +5030,19 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-18 22:37</t>
+          <t>2026-05-19 22:53</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
+          <t>❤️성주참외</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -5077,14 +5077,14 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-05-18 22:40</t>
+          <t>2026-05-19 22:53</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>❤️성주참외</t>
+          <t>성주참외</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -5124,14 +5124,14 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003357</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-18 22:40</t>
+          <t>2026-05-19 22:53</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -5141,12 +5141,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>성주참외</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5171,14 +5171,14 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003357</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-05-18 22:40</t>
+          <t>2026-05-19 22:54</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -5188,12 +5188,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5218,14 +5218,14 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-05-18 22:40</t>
+          <t>2026-05-19 22:54</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>하우스 천도복숭아</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5265,14 +5265,14 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003423</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-05-18 22:40</t>
+          <t>2026-05-19 22:54</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -5287,7 +5287,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>하우스 천도복숭아</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -5312,14 +5312,14 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003423</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003424</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-05-18 22:41</t>
+          <t>2026-05-19 22:54</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -5334,7 +5334,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>하우스 신선복숭아</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5359,14 +5359,14 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003424</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003425</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-05-18 22:41</t>
+          <t>2026-05-19 22:54</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -5381,7 +5381,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>하우스 신선복숭아</t>
+          <t>[고품위] 하우스 털 복숭아</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -5406,14 +5406,14 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003425</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-05-18 22:41</t>
+          <t>2026-05-19 22:54</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -5423,12 +5423,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>[고품위] 하우스 털 복숭아</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -5453,14 +5453,14 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-05-18 22:41</t>
+          <t>2026-05-19 22:56</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -5470,12 +5470,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>남해 햇 홍감자</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5500,14 +5500,14 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-18 22:42</t>
+          <t>2026-05-19 22:56</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>남해 햇 홍감자</t>
+          <t>햇 설봉감자</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5547,14 +5547,14 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-18 22:42</t>
+          <t>2026-05-19 22:56</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5564,12 +5564,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>햇 설봉감자</t>
+          <t>특가 대추방울토마토</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5594,14 +5594,14 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-18 22:42</t>
+          <t>2026-05-19 22:56</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5611,12 +5611,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>특가 대추방울토마토</t>
+          <t>햇 수미감자</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5641,14 +5641,14 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-18 22:43</t>
+          <t>2026-05-19 22:56</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5658,12 +5658,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>햇 수미감자</t>
+          <t>대저 흑대추방울토마토</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5688,14 +5688,14 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-18 22:43</t>
+          <t>2026-05-19 22:56</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5710,7 +5710,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>대저 흑대추방울토마토</t>
+          <t>부여 대추방울토마토</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5735,29 +5735,29 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-18 22:43</t>
+          <t>2026-05-19 22:58</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>더그린</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>부여 대추방울토마토</t>
+          <t>2026년 강원도감자</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5782,14 +5782,14 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-18 22:45</t>
+          <t>2026-05-19 22:59</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2026년 강원도감자</t>
+          <t>2026년 수미감자</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5829,14 +5829,14 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-18 22:45</t>
+          <t>2026-05-19 22:59</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>2026년 수미감자</t>
+          <t>2026년 햇 감자</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -5876,14 +5876,14 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-18 22:45</t>
+          <t>2026-05-19 22:59</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -5898,7 +5898,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>2026년 햇 감자</t>
+          <t>2026년 햇 홍감자</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5923,14 +5923,14 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001262</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-18 22:45</t>
+          <t>2026-05-19 22:59</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -5945,7 +5945,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>26년 햇 홍감자</t>
+          <t>2025년 홍 감자</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5970,14 +5970,14 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001262</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-18 22:46</t>
+          <t>2026-05-19 22:59</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -5992,7 +5992,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>2025년 홍 감자</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -6017,14 +6017,14 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-18 22:46</t>
+          <t>2026-05-19 22:59</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -6039,7 +6039,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>두백감자 ★7월 재오픈</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -6064,14 +6064,14 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-18 22:46</t>
+          <t>2026-05-19 22:59</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -6081,12 +6081,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>두백감자 ★7월 재오픈</t>
+          <t>대추 방울토마토</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -6111,14 +6111,14 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-18 22:46</t>
+          <t>2026-05-19 22:59</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>대추 방울토마토</t>
+          <t>흑대추 방울 토마토</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -6158,14 +6158,14 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-18 22:46</t>
+          <t>2026-05-19 23:00</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -6175,12 +6175,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>흑대추 방울 토마토</t>
+          <t>고당도 성주 참외 ※선물세트 포함</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -6205,14 +6205,14 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-18 22:46</t>
+          <t>2026-05-19 23:00</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -6222,12 +6222,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>고당도 성주 참외 ※선물세트 포함</t>
+          <t>스테비아 감자 ★7월 재오픈</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -6252,14 +6252,14 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-18 22:47</t>
+          <t>2026-05-19 23:00</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -6269,12 +6269,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>스테비아 감자 ★7월 재오픈</t>
+          <t>스테비야 방울토마토</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -6299,14 +6299,14 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-18 22:47</t>
+          <t>2026-05-19 23:00</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -6321,7 +6321,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>스테비야 방울토마토</t>
+          <t>스테비아 완숙 토마토</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -6345,53 +6345,6 @@
         </is>
       </c>
       <c r="I126" t="inlineStr">
-        <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>2026-05-18 22:47</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>더그린</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>토마토</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>스테비아 완숙 토마토</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H127" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I127" t="inlineStr">
         <is>
           <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000582</t>
         </is>

</xml_diff>

<commit_message>
Auto Update Prices: Wed May 20 23:09:38 UTC 2026
</commit_message>
<xml_diff>
--- a/가격이력.xlsx
+++ b/가격이력.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I126"/>
+  <dimension ref="A1:I132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-19 22:20</t>
+          <t>2026-05-20 22:26</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -488,12 +488,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>그린황도 복숭아</t>
+          <t>햇 홍감자</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -518,14 +518,14 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010213</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010296</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-19 22:20</t>
+          <t>2026-05-20 22:26</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -535,12 +535,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>하우스 흑미수박</t>
+          <t>햇감자</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -565,14 +565,14 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010144</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010279</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-19 22:20</t>
+          <t>2026-05-20 22:26</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -582,12 +582,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>스테비아방울토마토</t>
+          <t>애플수박</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -612,14 +612,14 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010143</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010261</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-19 22:20</t>
+          <t>2026-05-20 22:26</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -629,12 +629,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>우곡수박</t>
+          <t>그린황도 복숭아</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -659,14 +659,14 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010136</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010213</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-19 22:21</t>
+          <t>2026-05-20 22:27</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -676,12 +676,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>천도복숭아</t>
+          <t>하우스 흑미수박</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -706,14 +706,14 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010109</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010144</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-19 22:21</t>
+          <t>2026-05-20 22:27</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -723,12 +723,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>신비복숭아</t>
+          <t>스테비아방울토마토</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -753,14 +753,14 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010108</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010143</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-19 22:21</t>
+          <t>2026-05-20 22:27</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -770,12 +770,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SVIP ★ 하우스 대극천복숭아 ★</t>
+          <t>우곡수박</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -800,14 +800,14 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010048</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010136</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-19 22:21</t>
+          <t>2026-05-20 22:27</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>SVIP ★ 하우스 대석자두 ★</t>
+          <t>천도복숭아</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -847,14 +847,14 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010045</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010109</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-19 22:21</t>
+          <t>2026-05-20 22:27</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>SVIP ★ 하우스 복숭아 ★</t>
+          <t>신비복숭아</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -894,14 +894,14 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010044</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010108</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-19 22:21</t>
+          <t>2026-05-20 22:28</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>[VIP] 하우스복숭아</t>
+          <t>SVIP ★ 하우스 대극천복숭아 ★</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -941,14 +941,14 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010007</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010048</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-19 22:21</t>
+          <t>2026-05-20 22:28</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>[VIP] 하우스자두</t>
+          <t>SVIP ★ 하우스 대석자두 ★</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -988,14 +988,14 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010006</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010045</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-19 22:22</t>
+          <t>2026-05-20 22:28</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1005,12 +1005,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>수박 (가정용/정품)</t>
+          <t>SVIP ★ 하우스 복숭아 ★</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1035,14 +1035,14 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009976</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010044</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-19 22:22</t>
+          <t>2026-05-20 22:28</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>[VIP] 하우스복숭아</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1082,14 +1082,14 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009960</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010007</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-19 22:22</t>
+          <t>2026-05-20 22:28</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1099,12 +1099,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>하우스 신선복숭아</t>
+          <t>[VIP] 하우스자두</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1129,14 +1129,14 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009959</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010006</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-19 22:22</t>
+          <t>2026-05-20 22:28</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1146,12 +1146,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>햇양파</t>
+          <t>수박 (가정용/정품)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1176,14 +1176,14 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009925</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009976</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-19 22:23</t>
+          <t>2026-05-20 22:28</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1193,12 +1193,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1223,14 +1223,14 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009854</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009960</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-19 22:23</t>
+          <t>2026-05-20 22:28</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1240,12 +1240,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>완숙 찰 토마토</t>
+          <t>하우스 신선복숭아</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1270,29 +1270,29 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009762</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009959</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-19 22:25</t>
+          <t>2026-05-20 22:29</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>팡이농장</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
+          <t>햇양파</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1317,29 +1317,29 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009925</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-19 22:25</t>
+          <t>2026-05-20 22:29</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>최고집(VIP)</t>
+          <t>팡이농장</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1364,14 +1364,14 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
+          <t>https://jaehwan0330.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10009854</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-19 22:25</t>
+          <t>2026-05-20 22:31</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1381,12 +1381,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
+          <t>행사 ★ (박스포함) 햇 양파 10kg / 특</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1411,14 +1411,14 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012069</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-19 22:25</t>
+          <t>2026-05-20 22:31</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1428,12 +1428,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
+          <t>행사 ★ (박스포함) 햇 양파 10kg / 대</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1458,14 +1458,14 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012068</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-19 22:25</t>
+          <t>2026-05-20 22:31</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1475,12 +1475,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
+          <t>행사 ★ (박스포함) 햇 양파 10kg / 중</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1505,14 +1505,14 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012067</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-19 22:25</t>
+          <t>2026-05-20 22:31</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1522,12 +1522,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
+          <t>행사 ★ (박스포함) 햇 양파 10kg / 소</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1552,14 +1552,14 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012066</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-19 22:25</t>
+          <t>2026-05-20 22:31</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1569,12 +1569,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
+          <t>행사 ★ (박스포함) 햇 양파 5kg / 특</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1599,14 +1599,14 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012065</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-19 22:25</t>
+          <t>2026-05-20 22:31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1616,12 +1616,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
+          <t>행사 ★ (박스포함) 햇 양파 5kg / 대</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1646,14 +1646,14 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012064</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-19 22:25</t>
+          <t>2026-05-20 22:31</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1663,12 +1663,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
+          <t>행사 ★ (박스포함) 햇 양파 5kg / 중</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1693,14 +1693,14 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012063</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-19 22:25</t>
+          <t>2026-05-20 22:31</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1710,12 +1710,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
+          <t>행사 ★ (박스포함) 햇 양파 5kg / 소</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1740,14 +1740,14 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012062</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-19 22:25</t>
+          <t>2026-05-20 22:31</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1757,12 +1757,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
+          <t>행사 ★ (박스포함) 햇 양파 3kg / 특</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1787,14 +1787,14 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012061</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-19 22:26</t>
+          <t>2026-05-20 22:31</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1804,12 +1804,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
+          <t>행사 ★ (박스포함) 햇 양파 3kg / 대</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1834,14 +1834,14 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012060</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-19 22:26</t>
+          <t>2026-05-20 22:31</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1851,12 +1851,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
+          <t>행사 ★ (박스포함) 햇 양파 3kg / 중</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1881,14 +1881,14 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012059</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-19 22:26</t>
+          <t>2026-05-20 22:32</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1898,12 +1898,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
+          <t>행사 ★ (박스포함) 햇 양파 3kg / 소</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1928,14 +1928,14 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012058</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-19 22:26</t>
+          <t>2026-05-20 22:32</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1945,12 +1945,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
+          <t>행사 (박스포함) 햇 양파 10kg / 특</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1975,14 +1975,14 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012057</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-19 22:26</t>
+          <t>2026-05-20 22:32</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1992,12 +1992,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 가정용 / 2kg / 혼합과</t>
+          <t>행사 (박스포함) 햇 양파 10kg / 대</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2022,14 +2022,14 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011123</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012056</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-19 22:27</t>
+          <t>2026-05-20 22:32</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2039,12 +2039,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토★4kg / 혼합과</t>
+          <t>행사 (박스포함) 햇 양파 10kg / 중</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2069,14 +2069,14 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010320</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012055</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-19 22:27</t>
+          <t>2026-05-20 22:32</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2086,12 +2086,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토★3kg / 혼합과</t>
+          <t>행사 (박스포함) 햇 양파 10kg / 소</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2116,14 +2116,14 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010319</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012054</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-19 22:27</t>
+          <t>2026-05-20 22:32</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2133,12 +2133,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토 4kg / 혼합과</t>
+          <t>행사 (박스포함) 햇 양파 5kg / 특</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2163,14 +2163,14 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010318</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012053</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-19 22:27</t>
+          <t>2026-05-20 22:32</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2180,12 +2180,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>(박스포함) 완숙토마토 3kg / 혼합과</t>
+          <t>행사 (박스포함) 햇 양파 5kg / 대</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2210,14 +2210,14 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010317</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012052</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-19 22:27</t>
+          <t>2026-05-20 22:32</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2227,12 +2227,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>(박스포함)★완숙토마토 5kg / 혼합과</t>
+          <t>행사 (박스포함) 햇 양파 5kg / 중</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2257,14 +2257,14 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010107</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012051</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-19 22:27</t>
+          <t>2026-05-20 22:32</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2274,12 +2274,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 소과</t>
+          <t>행사 (박스포함) 햇 양파 5kg / 소</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2304,14 +2304,14 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011410</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012050</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-19 22:27</t>
+          <t>2026-05-20 22:32</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2321,12 +2321,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 로얄과</t>
+          <t>행사 (박스포함) 햇 양파 3kg / 특</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2351,14 +2351,14 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011409</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012049</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-19 22:27</t>
+          <t>2026-05-20 22:32</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2368,12 +2368,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 대과</t>
+          <t>행사 (박스포함) 햇 양파 3kg / 대</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2398,14 +2398,14 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011408</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012048</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-19 22:28</t>
+          <t>2026-05-20 22:33</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2415,12 +2415,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 5kg / 혼합과</t>
+          <t>행사 (박스포함) 햇 양파 3kg / 중</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2445,14 +2445,14 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011407</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012047</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-19 22:28</t>
+          <t>2026-05-20 22:33</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2462,12 +2462,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 소과</t>
+          <t>행사 (박스포함) 햇 양파 3kg / 소</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2492,14 +2492,14 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011405</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10012046</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-19 22:28</t>
+          <t>2026-05-20 22:33</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 로얄과</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2539,14 +2539,14 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011404</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011323</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-19 22:28</t>
+          <t>2026-05-20 22:33</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 대과</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2586,14 +2586,14 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011403</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011322</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-19 22:28</t>
+          <t>2026-05-20 22:33</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 3kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 혼합과</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2633,14 +2633,14 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011402</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011321</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-19 22:28</t>
+          <t>2026-05-20 22:33</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 소과</t>
+          <t>(박스포함) 참외 가정용 / 10kg / 소과</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2680,14 +2680,14 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011401</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011320</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-19 22:28</t>
+          <t>2026-05-20 22:33</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 로얄과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 소과</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2727,14 +2727,14 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011400</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011134</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-19 22:28</t>
+          <t>2026-05-20 22:33</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 대과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 로얄과</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2774,14 +2774,14 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011399</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011133</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-19 22:28</t>
+          <t>2026-05-20 22:33</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>(박스포함) 참외 ★ 가정용 / 2kg / 혼합과</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 대과</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2821,14 +2821,14 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011398</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011132</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-19 22:28</t>
+          <t>2026-05-20 22:33</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2838,12 +2838,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>💪💪산지 최전선 '최고집' 하우스 자두💪💪</t>
+          <t>(박스포함) 참외 가정용 / 5kg / 혼합과</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2868,29 +2868,29 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011313</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011131</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-19 22:30</t>
+          <t>2026-05-20 22:34</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>햇 홍감자</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 소과</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2915,29 +2915,29 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000596</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011130</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-19 22:30</t>
+          <t>2026-05-20 22:34</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 로얄과</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2962,29 +2962,29 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002048</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011129</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-19 22:30</t>
+          <t>2026-05-20 22:34</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>하우스 천도복숭아</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 대과</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3009,29 +3009,29 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002047</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011128</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-19 22:30</t>
+          <t>2026-05-20 22:34</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>하우스 대극천복숭아</t>
+          <t>(박스포함) 참외 가정용 / 3kg / 혼합과</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3056,29 +3056,29 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001975</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011127</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-19 22:30</t>
+          <t>2026-05-20 22:34</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>★특가★ 하우스 대석자두</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 소과</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3103,29 +3103,29 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002042</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011126</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-19 22:31</t>
+          <t>2026-05-20 22:34</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>하우스 대석자두</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 로얄과</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3150,29 +3150,29 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001958</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011125</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-19 22:31</t>
+          <t>2026-05-20 22:34</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>하우스 털복숭아</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 대과</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3197,19 +3197,19 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001942</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011124</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-19 22:31</t>
+          <t>2026-05-20 22:34</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외 (박스포함)</t>
+          <t>(박스포함) 참외 가정용 / 2kg / 혼합과</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3244,29 +3244,29 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10011123</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-19 22:31</t>
+          <t>2026-05-20 22:35</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>늘푸른우리</t>
+          <t>최고집(VIP)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>★특가★ 성주 꿀참외</t>
+          <t>(박스포함) 완숙토마토★4kg / 혼합과</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3291,14 +3291,14 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
+          <t>https://zain0401.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10010320</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-05-19 22:31</t>
+          <t>2026-05-20 22:36</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3308,12 +3308,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>정품 우곡수박</t>
+          <t>햇 홍감자</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3338,14 +3338,14 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002058</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000596</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-19 22:32</t>
+          <t>2026-05-20 22:36</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3355,12 +3355,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>★특가★ 가정용 하우스수박</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3385,14 +3385,14 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002048</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-19 22:32</t>
+          <t>2026-05-20 22:36</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3402,12 +3402,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>정품 하우스수박</t>
+          <t>하우스 천도복숭아</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3432,14 +3432,14 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001536</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002047</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-19 22:32</t>
+          <t>2026-05-20 22:37</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3449,12 +3449,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>고당도 흑수박</t>
+          <t>하우스 대극천복숭아</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3479,14 +3479,14 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000630</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001975</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-05-19 22:33</t>
+          <t>2026-05-20 22:37</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3496,12 +3496,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>2026 국내산 햇감자</t>
+          <t>★특가★ 하우스 대석자두</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3526,14 +3526,14 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002042</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-19 22:33</t>
+          <t>2026-05-20 22:37</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3543,12 +3543,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2026 국내산 햇양파</t>
+          <t>하우스 대석자두</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3573,14 +3573,14 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001958</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-19 22:33</t>
+          <t>2026-05-20 22:37</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3590,12 +3590,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>★특가★ 대추방울토마토</t>
+          <t>하우스 털복숭아</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3620,14 +3620,14 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001942</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-19 22:33</t>
+          <t>2026-05-20 22:37</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3637,12 +3637,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>★특가★ 유럽종 완숙토마토</t>
+          <t>★특가★ 성주 꿀참외 (박스포함)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3667,14 +3667,14 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001616</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-05-19 22:33</t>
+          <t>2026-05-20 22:37</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3684,12 +3684,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>스테비아 방울토마토</t>
+          <t>★특가★ 성주 꿀참외</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3714,29 +3714,29 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000331</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-19 22:34</t>
+          <t>2026-05-20 22:38</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>★별담특가 가정용 참외★</t>
+          <t>정품 우곡수박</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3761,29 +3761,29 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002058</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-05-19 22:35</t>
+          <t>2026-05-20 22:38</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>2026 햇양파</t>
+          <t>★특가★ 가정용 하우스수박</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3808,19 +3808,19 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001981</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-19 22:35</t>
+          <t>2026-05-20 22:38</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3830,7 +3830,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>고당도 하우스 수박(12브릭스 이상)</t>
+          <t>정품 하우스수박</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3855,29 +3855,29 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008785</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001536</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-05-19 22:35</t>
+          <t>2026-05-20 22:38</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>고당도 흑수박</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3902,29 +3902,29 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008787</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000630</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-19 22:36</t>
+          <t>2026-05-20 22:39</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>2026 국내산 햇감자</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3949,29 +3949,29 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008652</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001916</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-05-19 22:36</t>
+          <t>2026-05-20 22:39</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>2026 국내산 햇양파</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3996,29 +3996,29 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008650</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001892</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-19 22:37</t>
+          <t>2026-05-20 22:40</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>팜허브</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>★특가★ 대추방울토마토</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4043,29 +4043,29 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001854</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-05-19 22:39</t>
+          <t>2026-05-20 22:40</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>★특가★ 가성비 참외</t>
+          <t>★특가★ 유럽종 완숙토마토</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4090,29 +4090,29 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002133</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001850</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-19 22:40</t>
+          <t>2026-05-20 22:40</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>늘푸른우리</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>햇 감자</t>
+          <t>스테비아 방울토마토</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4137,29 +4137,29 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002108</t>
+          <t>https://hwanggs3.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001800</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05-19 22:40</t>
+          <t>2026-05-20 22:41</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>양파</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>햇 양파</t>
+          <t>★별담특가 가정용 참외★</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -4184,29 +4184,29 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000186</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008571</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-19 22:40</t>
+          <t>2026-05-20 22:41</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>대추방울토마토</t>
+          <t>2026 햇양파</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4231,29 +4231,29 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008444</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-05-19 22:41</t>
+          <t>2026-05-20 22:41</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -4278,29 +4278,29 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008787</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-19 22:41</t>
+          <t>2026-05-20 22:43</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>덤덤몰</t>
+          <t>팜허브</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -4325,14 +4325,14 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
+          <t>https://priceit.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10008591</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-05-19 22:41</t>
+          <t>2026-05-20 22:46</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4342,12 +4342,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>대저토마토</t>
+          <t>★특가★ 가성비 참외</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -4372,29 +4372,29 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002133</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-19 22:44</t>
+          <t>2026-05-20 22:46</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>🔥핫딜🔥 가정용 성주참외</t>
+          <t>햇 감자</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4419,29 +4419,29 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001165</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002108</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-05-19 22:44</t>
+          <t>2026-05-20 22:46</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>양파</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>★당도보장★ 농협선별 스테비아 수박</t>
+          <t>햇 양파</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4466,29 +4466,29 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000186</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-19 22:44</t>
+          <t>2026-05-20 22:47</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>[N-81] 신비복숭아</t>
+          <t>대추방울토마토</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4513,19 +4513,19 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000351</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-05-19 22:45</t>
+          <t>2026-05-20 22:47</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -4535,7 +4535,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4560,29 +4560,29 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001913</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-05-19 22:45</t>
+          <t>2026-05-20 22:47</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>마니팜</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>가정용 하우스수박 (기박)</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4607,29 +4607,29 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001821</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-05-19 22:47</t>
+          <t>2026-05-20 22:47</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>덤덤몰</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>대저토마토</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4654,29 +4654,29 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006697</t>
+          <t>https://dumdummall.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001755</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-19 22:48</t>
+          <t>2026-05-20 22:50</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
+          <t>🔥핫딜🔥 가정용 성주참외</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4701,19 +4701,19 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001165</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-05-19 22:48</t>
+          <t>2026-05-20 22:51</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
+          <t>★당도보장★ 농협선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -4748,29 +4748,29 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001134</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-19 22:49</t>
+          <t>2026-05-20 22:51</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>농협인증 당도선별 스테비아 수박</t>
+          <t>[N-81] 신비복숭아</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4795,29 +4795,29 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001129</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-05-19 22:49</t>
+          <t>2026-05-20 22:51</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>수박</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>국내산 무주 수박무말랭이</t>
+          <t>★맛 없으면 무료반품 옵션★ [M-83] 성주참외</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4842,19 +4842,19 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001000</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-05-19 22:49</t>
+          <t>2026-05-20 22:51</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>산지이음</t>
+          <t>마니팜</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>정품 수박</t>
+          <t>가정용 하우스수박 (기박)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4889,14 +4889,14 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
+          <t>https://mp3462.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000961</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-05-19 22:49</t>
+          <t>2026-05-20 22:53</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4906,12 +4906,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>대추 방울 토마토 소과</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4936,14 +4936,14 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006697</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-05-19 22:49</t>
+          <t>2026-05-20 22:54</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>가정용 흑수박 5kg 이상</t>
+          <t>[못난이]맛은 정품 그대로! 깎아먹는 못난이 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4983,14 +4983,14 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006611</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-05-19 22:50</t>
+          <t>2026-05-20 22:55</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -5000,12 +5000,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
+          <t>깎아먹는 미니 애플수박 1.5kg (2-3입)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -5030,29 +5030,29 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006587</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-05-19 22:53</t>
+          <t>2026-05-20 22:55</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>❤️성주참외</t>
+          <t>농협인증 당도선별 스테비아 수박</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -5077,29 +5077,29 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006572</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-05-19 22:53</t>
+          <t>2026-05-20 22:55</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>성주참외</t>
+          <t>국내산 무주 수박무말랭이</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -5124,19 +5124,19 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003357</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006558</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-05-19 22:53</t>
+          <t>2026-05-20 22:55</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -5146,7 +5146,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>하우스 수박</t>
+          <t>정품 수박</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5171,29 +5171,29 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006540</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-05-19 22:54</t>
+          <t>2026-05-20 22:56</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>하우스 복숭아</t>
+          <t>대추 방울 토마토 소과</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5218,29 +5218,29 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006532</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-05-19 22:54</t>
+          <t>2026-05-20 22:56</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>하우스 천도복숭아</t>
+          <t>가정용 흑수박 5kg 이상</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5265,29 +5265,29 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003423</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006521</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-05-19 22:54</t>
+          <t>2026-05-20 22:57</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>팜플로우</t>
+          <t>산지이음</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>하우스 신비복숭아</t>
+          <t>껍질째 먹는 한입 꼬마 참외 (개당 110~140g)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -5312,14 +5312,14 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003424</t>
+          <t>https://orangec.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10006351</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-05-19 22:54</t>
+          <t>2026-05-20 23:00</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -5329,12 +5329,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>하우스 신선복숭아</t>
+          <t>❤️성주참외</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5359,14 +5359,14 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003425</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002544</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-05-19 22:54</t>
+          <t>2026-05-20 23:00</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -5376,12 +5376,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>복숭아</t>
+          <t>참외</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>[고품위] 하우스 털 복숭아</t>
+          <t>성주참외</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -5406,14 +5406,14 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003357</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-05-19 22:54</t>
+          <t>2026-05-20 23:00</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -5423,12 +5423,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>자두</t>
+          <t>수박</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>하우스 자두</t>
+          <t>하우스 수박</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -5453,14 +5453,14 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003033</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-05-19 22:56</t>
+          <t>2026-05-20 23:00</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -5470,12 +5470,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>남해 햇 홍감자</t>
+          <t>하우스 복숭아</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5500,14 +5500,14 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003221</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-05-19 22:56</t>
+          <t>2026-05-20 23:00</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5517,12 +5517,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>햇 설봉감자</t>
+          <t>하우스 천도복숭아</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5547,14 +5547,14 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003423</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-05-19 22:56</t>
+          <t>2026-05-20 23:00</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5564,12 +5564,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>특가 대추방울토마토</t>
+          <t>하우스 신비복숭아</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5594,14 +5594,14 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003424</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-05-19 22:56</t>
+          <t>2026-05-20 23:00</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5611,12 +5611,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>햇 수미감자</t>
+          <t>하우스 신선복숭아</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5641,14 +5641,14 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003425</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-05-19 22:56</t>
+          <t>2026-05-20 23:00</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5658,12 +5658,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>복숭아</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>대저 흑대추방울토마토</t>
+          <t>[고품위] 하우스 털 복숭아</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5688,14 +5688,14 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003313</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-05-19 22:56</t>
+          <t>2026-05-20 23:01</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5705,12 +5705,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>자두</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>부여 대추방울토마토</t>
+          <t>하우스 자두</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5735,19 +5735,19 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003222</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-05-19 22:58</t>
+          <t>2026-05-20 23:02</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -5757,7 +5757,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>2026년 강원도감자</t>
+          <t>남해 햇 홍감자</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5782,19 +5782,19 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003147</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-05-19 22:59</t>
+          <t>2026-05-20 23:02</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2026년 수미감자</t>
+          <t>햇 설봉감자</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5829,29 +5829,29 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003146</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-05-19 22:59</t>
+          <t>2026-05-20 23:02</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>2026년 햇 감자</t>
+          <t>특가 대추방울토마토</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -5876,19 +5876,19 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003187</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-05-19 22:59</t>
+          <t>2026-05-20 23:02</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -5898,7 +5898,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>2026년 햇 홍감자</t>
+          <t>햇 수미감자</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5923,29 +5923,29 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001262</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003145</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-05-19 22:59</t>
+          <t>2026-05-20 23:03</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>2025년 홍 감자</t>
+          <t>대저 흑대추방울토마토</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5970,29 +5970,29 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10003038</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-05-19 22:59</t>
+          <t>2026-05-20 23:03</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>더그린</t>
+          <t>팜플로우</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>감자</t>
+          <t>토마토</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>돼지감자</t>
+          <t>부여 대추방울토마토</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -6017,14 +6017,14 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
+          <t>https://farmflow.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10002702</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-05-19 22:59</t>
+          <t>2026-05-20 23:05</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -6039,7 +6039,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>두백감자 ★7월 재오픈</t>
+          <t>2026년 강원도감자</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -6064,14 +6064,14 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000998</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-05-19 22:59</t>
+          <t>2026-05-20 23:05</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -6081,12 +6081,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>대추 방울토마토</t>
+          <t>2026년 수미감자</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -6111,14 +6111,14 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000184</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-05-19 22:59</t>
+          <t>2026-05-20 23:05</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -6128,12 +6128,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>흑대추 방울 토마토</t>
+          <t>2026년 햇 감자</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -6158,14 +6158,14 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001024</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-05-19 23:00</t>
+          <t>2026-05-20 23:05</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -6175,12 +6175,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>참외</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>고당도 성주 참외 ※선물세트 포함</t>
+          <t>2026년 햇 홍감자</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -6205,14 +6205,14 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001262</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-05-19 23:00</t>
+          <t>2026-05-20 23:05</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>스테비아 감자 ★7월 재오픈</t>
+          <t>2025년 홍 감자</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -6252,14 +6252,14 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000305</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-05-19 23:00</t>
+          <t>2026-05-20 23:06</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -6269,12 +6269,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>토마토</t>
+          <t>감자</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>스테비야 방울토마토</t>
+          <t>돼지감자</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -6299,14 +6299,14 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001142</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-05-19 23:00</t>
+          <t>2026-05-20 23:06</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -6316,35 +6316,317 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
+          <t>감자</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>두백감자 ★7월 재오픈</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000006</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-05-20 23:06</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
           <t>토마토</t>
         </is>
       </c>
-      <c r="D126" t="inlineStr">
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>대추 방울토마토</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001135</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-05-20 23:06</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>토마토</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>흑대추 방울 토마토</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000262</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-05-20 23:06</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>참외</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>고당도 성주 참외 ※선물세트 포함</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10001088</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-05-20 23:07</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>감자</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>스테비아 감자 ★7월 재오픈</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000570</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-05-20 23:07</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>토마토</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>스테비야 방울토마토</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000574</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-05-20 23:07</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>더그린</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>토마토</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
         <is>
           <t>스테비아 완숙 토마토</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>단일품목</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>상세참조</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>있음</t>
-        </is>
-      </c>
-      <c r="H126" t="inlineStr">
-        <is>
-          <t>별도</t>
-        </is>
-      </c>
-      <c r="I126" t="inlineStr">
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>단일품목</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>상세참조</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>있음</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
         <is>
           <t>https://gl1248.adminplus.co.kr/partner/product/prt.detail.pop.php?pcode=10000582</t>
         </is>

</xml_diff>